<commit_message>
Fix XML recovery error: remove _xlfn. prefixes from dashboard formula
openpyxl-written _xlfn. prefixes on LET/FILTER/VSTACK/SORT caused Excel
to flag /xl/worksheets/sheet1.xml on open. Excel 365 evaluates these
functions natively without the prefix. Also fixed INDEX(combined,,1)
to INDEX(combined,0,1) for clean XML serialization.

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -1047,7 +1047,7 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>_xlfn.LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(_xlfn.FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(_xlfn.FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,_xlfn.VSTACK(ntFilt,reFilt),active,IFERROR(_xlfn.FILTER(combined,INDEX(combined,,1)&lt;&gt;""),{"No active jobs","","","","","",""}),_xlfn.SORT(active,1,1))</f>
+        <f>LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,VSTACK(ntFilt,reFilt),active,IFERROR(FILTER(combined,INDEX(combined,0,1)&lt;&gt;""),{"No active jobs","","","","","",""}),SORT(active,1,1))</f>
         <v/>
       </c>
       <c r="B10" s="39" t="n"/>
@@ -2190,42 +2190,42 @@
           <t>Days Until Deadline</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice #</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Date</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Sent Date</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Status</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice #</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AD12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Date</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
+      <c r="AE12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Amount ($)</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr">
+      <c r="AF12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Status</t>
         </is>
@@ -4370,42 +4370,42 @@
           <t>Days Until Deadline</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice #</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Date</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Sent Date</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Status</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice #</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Date</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Amount ($)</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Status</t>
         </is>

</xml_diff>

<commit_message>
Fix dashboard formula not evaluating: inject _xlfn. prefixes directly into XML
openpyxl strips _xlfn. prefixes when it serializes formulas, so Excel
cannot recognise LET/FILTER/VSTACK/SORT at open time. Fixed by patching
xl/worksheets/sheet1.xml directly inside the zip after openpyxl writes
the file, ensuring _xlfn.LET, _xlfn.FILTER, _xlfn.VSTACK, and _xlfn.SORT
are all present in the <f> element as Excel requires. Also expanded
sheet dimension ref to cover the dynamic spill area.

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -1047,15 +1047,15 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,VSTACK(ntFilt,reFilt),active,IFERROR(FILTER(combined,INDEX(combined,0,1)&lt;&gt;""),{"No active jobs","","","","","",""}),SORT(active,1,1))</f>
-        <v/>
-      </c>
-      <c r="B10" s="39" t="n"/>
-      <c r="C10" s="39" t="n"/>
-      <c r="D10" s="39" t="n"/>
-      <c r="E10" s="39" t="n"/>
-      <c r="F10" s="39" t="n"/>
-      <c r="G10" s="39" t="n"/>
+        <f>_xlfn.LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(_xlfn.FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(_xlfn.FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,_xlfn.VSTACK(ntFilt,reFilt),active,IFERROR(_xlfn.FILTER(combined,INDEX(combined,0,1)&lt;&gt;""),{"No active jobs","","","","","",""}),_xlfn.SORT(active,1,1))</f>
+        <v/>
+      </c>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="40" t="n"/>

</xml_diff>

<commit_message>
Replace dynamic array formula with classic INDEX/SMALL/IF approach
LET/FILTER/VSTACK/SORT cause XML recovery errors when written by openpyxl
regardless of prefix handling. Replaced with 100 rows of classic
INDEX/SMALL(IF(...))/COUNTIFS formulas (no _xlfn. dependencies).
Works on Excel 365 and 2019. No dynamic array functions used.

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -1047,906 +1047,3003 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>_xlfn.LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(_xlfn.FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(_xlfn.FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,_xlfn.VSTACK(ntFilt,reFilt),active,IFERROR(_xlfn.FILTER(combined,INDEX(combined,0,1)&lt;&gt;""),{"No active jobs","","","","","",""}),_xlfn.SORT(active,1,1))</f>
-        <v/>
-      </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="39">
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="40" t="n"/>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="41" t="n"/>
-      <c r="D11" s="41" t="n"/>
-      <c r="E11" s="40" t="n"/>
-      <c r="F11" s="40" t="n"/>
-      <c r="G11" s="41" t="n"/>
+      <c r="A11" s="40">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B11" s="40">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="41">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="41">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="40">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="40">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="41">
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="40" t="n"/>
-      <c r="B12" s="40" t="n"/>
-      <c r="C12" s="41" t="n"/>
-      <c r="D12" s="41" t="n"/>
-      <c r="E12" s="40" t="n"/>
-      <c r="F12" s="40" t="n"/>
-      <c r="G12" s="41" t="n"/>
+      <c r="A12" s="40">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B12" s="40">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="41">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="41">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="40">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="40">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="41">
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="40" t="n"/>
-      <c r="B13" s="40" t="n"/>
-      <c r="C13" s="41" t="n"/>
-      <c r="D13" s="41" t="n"/>
-      <c r="E13" s="40" t="n"/>
-      <c r="F13" s="40" t="n"/>
-      <c r="G13" s="41" t="n"/>
+      <c r="A13" s="40">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B13" s="40">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="41">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="41">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="40">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="40">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="41">
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="40" t="n"/>
-      <c r="B14" s="40" t="n"/>
-      <c r="C14" s="41" t="n"/>
-      <c r="D14" s="41" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="40" t="n"/>
-      <c r="G14" s="41" t="n"/>
+      <c r="A14" s="40">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B14" s="40">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="41">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="41">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="40">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="40">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="41">
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="40" t="n"/>
-      <c r="C15" s="41" t="n"/>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="40" t="n"/>
-      <c r="F15" s="40" t="n"/>
-      <c r="G15" s="41" t="n"/>
+      <c r="A15" s="40">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B15" s="40">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="41">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="41">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="40">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="40">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="41">
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="40" t="n"/>
-      <c r="B16" s="40" t="n"/>
-      <c r="C16" s="41" t="n"/>
-      <c r="D16" s="41" t="n"/>
-      <c r="E16" s="40" t="n"/>
-      <c r="F16" s="40" t="n"/>
-      <c r="G16" s="41" t="n"/>
+      <c r="A16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="40" t="n"/>
-      <c r="B17" s="40" t="n"/>
-      <c r="C17" s="41" t="n"/>
-      <c r="D17" s="41" t="n"/>
-      <c r="E17" s="40" t="n"/>
-      <c r="F17" s="40" t="n"/>
-      <c r="G17" s="41" t="n"/>
+      <c r="A17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="40" t="n"/>
-      <c r="B18" s="40" t="n"/>
-      <c r="C18" s="41" t="n"/>
-      <c r="D18" s="41" t="n"/>
-      <c r="E18" s="40" t="n"/>
-      <c r="F18" s="40" t="n"/>
-      <c r="G18" s="41" t="n"/>
+      <c r="A18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="40" t="n"/>
-      <c r="B19" s="40" t="n"/>
-      <c r="C19" s="41" t="n"/>
-      <c r="D19" s="41" t="n"/>
-      <c r="E19" s="40" t="n"/>
-      <c r="F19" s="40" t="n"/>
-      <c r="G19" s="41" t="n"/>
+      <c r="A19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
-      <c r="A20" s="40" t="n"/>
-      <c r="B20" s="40" t="n"/>
-      <c r="C20" s="41" t="n"/>
-      <c r="D20" s="41" t="n"/>
-      <c r="E20" s="40" t="n"/>
-      <c r="F20" s="40" t="n"/>
-      <c r="G20" s="41" t="n"/>
+      <c r="A20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="40" t="n"/>
-      <c r="C21" s="41" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
-      <c r="G21" s="41" t="n"/>
+      <c r="A21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
-      <c r="A22" s="40" t="n"/>
-      <c r="B22" s="40" t="n"/>
-      <c r="C22" s="41" t="n"/>
-      <c r="D22" s="41" t="n"/>
-      <c r="E22" s="40" t="n"/>
-      <c r="F22" s="40" t="n"/>
-      <c r="G22" s="41" t="n"/>
+      <c r="A22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
-      <c r="A23" s="40" t="n"/>
-      <c r="B23" s="40" t="n"/>
-      <c r="C23" s="41" t="n"/>
-      <c r="D23" s="41" t="n"/>
-      <c r="E23" s="40" t="n"/>
-      <c r="F23" s="40" t="n"/>
-      <c r="G23" s="41" t="n"/>
+      <c r="A23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
-      <c r="A24" s="40" t="n"/>
-      <c r="B24" s="40" t="n"/>
-      <c r="C24" s="41" t="n"/>
-      <c r="D24" s="41" t="n"/>
-      <c r="E24" s="40" t="n"/>
-      <c r="F24" s="40" t="n"/>
-      <c r="G24" s="41" t="n"/>
+      <c r="A24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
-      <c r="A25" s="40" t="n"/>
-      <c r="B25" s="40" t="n"/>
-      <c r="C25" s="41" t="n"/>
-      <c r="D25" s="41" t="n"/>
-      <c r="E25" s="40" t="n"/>
-      <c r="F25" s="40" t="n"/>
-      <c r="G25" s="41" t="n"/>
+      <c r="A25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
-      <c r="A26" s="40" t="n"/>
-      <c r="B26" s="40" t="n"/>
-      <c r="C26" s="41" t="n"/>
-      <c r="D26" s="41" t="n"/>
-      <c r="E26" s="40" t="n"/>
-      <c r="F26" s="40" t="n"/>
-      <c r="G26" s="41" t="n"/>
+      <c r="A26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
-      <c r="A27" s="40" t="n"/>
-      <c r="B27" s="40" t="n"/>
-      <c r="C27" s="41" t="n"/>
-      <c r="D27" s="41" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="40" t="n"/>
-      <c r="G27" s="41" t="n"/>
+      <c r="A27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
-      <c r="A28" s="40" t="n"/>
-      <c r="B28" s="40" t="n"/>
-      <c r="C28" s="41" t="n"/>
-      <c r="D28" s="41" t="n"/>
-      <c r="E28" s="40" t="n"/>
-      <c r="F28" s="40" t="n"/>
-      <c r="G28" s="41" t="n"/>
+      <c r="A28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
-      <c r="A29" s="40" t="n"/>
-      <c r="B29" s="40" t="n"/>
-      <c r="C29" s="41" t="n"/>
-      <c r="D29" s="41" t="n"/>
-      <c r="E29" s="40" t="n"/>
-      <c r="F29" s="40" t="n"/>
-      <c r="G29" s="41" t="n"/>
+      <c r="A29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
-      <c r="A30" s="40" t="n"/>
-      <c r="B30" s="40" t="n"/>
-      <c r="C30" s="41" t="n"/>
-      <c r="D30" s="41" t="n"/>
-      <c r="E30" s="40" t="n"/>
-      <c r="F30" s="40" t="n"/>
-      <c r="G30" s="41" t="n"/>
+      <c r="A30" s="40">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B30" s="40">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C30" s="41">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D30" s="41">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="41">
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
-      <c r="A31" s="40" t="n"/>
-      <c r="B31" s="40" t="n"/>
-      <c r="C31" s="41" t="n"/>
-      <c r="D31" s="41" t="n"/>
-      <c r="E31" s="40" t="n"/>
-      <c r="F31" s="40" t="n"/>
-      <c r="G31" s="41" t="n"/>
+      <c r="A31" s="40">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B31" s="40">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C31" s="41">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D31" s="41">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E31" s="40">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="40">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="41">
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
-      <c r="A32" s="40" t="n"/>
-      <c r="B32" s="40" t="n"/>
-      <c r="C32" s="41" t="n"/>
-      <c r="D32" s="41" t="n"/>
-      <c r="E32" s="40" t="n"/>
-      <c r="F32" s="40" t="n"/>
-      <c r="G32" s="41" t="n"/>
+      <c r="A32" s="40">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B32" s="40">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C32" s="41">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D32" s="41">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E32" s="40">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="40">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="41">
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
-      <c r="A33" s="40" t="n"/>
-      <c r="B33" s="40" t="n"/>
-      <c r="C33" s="41" t="n"/>
-      <c r="D33" s="41" t="n"/>
-      <c r="E33" s="40" t="n"/>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="41" t="n"/>
+      <c r="A33" s="40">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B33" s="40">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C33" s="41">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D33" s="41">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E33" s="40">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="40">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="41">
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
-      <c r="A34" s="40" t="n"/>
-      <c r="B34" s="40" t="n"/>
-      <c r="C34" s="41" t="n"/>
-      <c r="D34" s="41" t="n"/>
-      <c r="E34" s="40" t="n"/>
-      <c r="F34" s="40" t="n"/>
-      <c r="G34" s="41" t="n"/>
+      <c r="A34" s="40">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B34" s="40">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C34" s="41">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D34" s="41">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="40">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="40">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="41">
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
-      <c r="A35" s="40" t="n"/>
-      <c r="B35" s="40" t="n"/>
-      <c r="C35" s="41" t="n"/>
-      <c r="D35" s="41" t="n"/>
-      <c r="E35" s="40" t="n"/>
-      <c r="F35" s="40" t="n"/>
-      <c r="G35" s="41" t="n"/>
+      <c r="A35" s="40">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B35" s="40">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C35" s="41">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D35" s="41">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="40">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="40">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="41">
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
-      <c r="A36" s="40" t="n"/>
-      <c r="B36" s="40" t="n"/>
-      <c r="C36" s="41" t="n"/>
-      <c r="D36" s="41" t="n"/>
-      <c r="E36" s="40" t="n"/>
-      <c r="F36" s="40" t="n"/>
-      <c r="G36" s="41" t="n"/>
+      <c r="A36" s="40">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B36" s="40">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C36" s="41">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D36" s="41">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="40">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="40">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="41">
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
-      <c r="A37" s="40" t="n"/>
-      <c r="B37" s="40" t="n"/>
-      <c r="C37" s="41" t="n"/>
-      <c r="D37" s="41" t="n"/>
-      <c r="E37" s="40" t="n"/>
-      <c r="F37" s="40" t="n"/>
-      <c r="G37" s="41" t="n"/>
+      <c r="A37" s="40">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B37" s="40">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C37" s="41">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D37" s="41">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="40">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="40">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="41">
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
-      <c r="A38" s="40" t="n"/>
-      <c r="B38" s="40" t="n"/>
-      <c r="C38" s="41" t="n"/>
-      <c r="D38" s="41" t="n"/>
-      <c r="E38" s="40" t="n"/>
-      <c r="F38" s="40" t="n"/>
-      <c r="G38" s="41" t="n"/>
+      <c r="A38" s="40">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B38" s="40">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C38" s="41">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="41">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="40">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="40">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="41">
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
-      <c r="A39" s="40" t="n"/>
-      <c r="B39" s="40" t="n"/>
-      <c r="C39" s="41" t="n"/>
-      <c r="D39" s="41" t="n"/>
-      <c r="E39" s="40" t="n"/>
-      <c r="F39" s="40" t="n"/>
-      <c r="G39" s="41" t="n"/>
+      <c r="A39" s="40">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B39" s="40">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C39" s="41">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D39" s="41">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E39" s="40">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="40">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="41">
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
-      <c r="A40" s="40" t="n"/>
-      <c r="B40" s="40" t="n"/>
-      <c r="C40" s="41" t="n"/>
-      <c r="D40" s="41" t="n"/>
-      <c r="E40" s="40" t="n"/>
-      <c r="F40" s="40" t="n"/>
-      <c r="G40" s="41" t="n"/>
+      <c r="A40" s="40">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B40" s="40">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C40" s="41">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="41">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="40">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="40">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="41">
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
-      <c r="A41" s="40" t="n"/>
-      <c r="B41" s="40" t="n"/>
-      <c r="C41" s="41" t="n"/>
-      <c r="D41" s="41" t="n"/>
-      <c r="E41" s="40" t="n"/>
-      <c r="F41" s="40" t="n"/>
-      <c r="G41" s="41" t="n"/>
+      <c r="A41" s="40">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B41" s="40">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C41" s="41">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D41" s="41">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="40">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="40">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="41">
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
-      <c r="A42" s="40" t="n"/>
-      <c r="B42" s="40" t="n"/>
-      <c r="C42" s="41" t="n"/>
-      <c r="D42" s="41" t="n"/>
-      <c r="E42" s="40" t="n"/>
-      <c r="F42" s="40" t="n"/>
-      <c r="G42" s="41" t="n"/>
+      <c r="A42" s="40">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B42" s="40">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C42" s="41">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D42" s="41">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="40">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="40">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G42" s="41">
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
-      <c r="A43" s="40" t="n"/>
-      <c r="B43" s="40" t="n"/>
-      <c r="C43" s="41" t="n"/>
-      <c r="D43" s="41" t="n"/>
-      <c r="E43" s="40" t="n"/>
-      <c r="F43" s="40" t="n"/>
-      <c r="G43" s="41" t="n"/>
+      <c r="A43" s="40">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B43" s="40">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C43" s="41">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D43" s="41">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="40">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="40">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="41">
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
-      <c r="A44" s="40" t="n"/>
-      <c r="B44" s="40" t="n"/>
-      <c r="C44" s="41" t="n"/>
-      <c r="D44" s="41" t="n"/>
-      <c r="E44" s="40" t="n"/>
-      <c r="F44" s="40" t="n"/>
-      <c r="G44" s="41" t="n"/>
+      <c r="A44" s="40">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B44" s="40">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C44" s="41">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D44" s="41">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="40">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="40">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="41">
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
-      <c r="A45" s="40" t="n"/>
-      <c r="B45" s="40" t="n"/>
-      <c r="C45" s="41" t="n"/>
-      <c r="D45" s="41" t="n"/>
-      <c r="E45" s="40" t="n"/>
-      <c r="F45" s="40" t="n"/>
-      <c r="G45" s="41" t="n"/>
+      <c r="A45" s="40">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B45" s="40">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C45" s="41">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D45" s="41">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E45" s="40">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="40">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="41">
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
-      <c r="A46" s="40" t="n"/>
-      <c r="B46" s="40" t="n"/>
-      <c r="C46" s="41" t="n"/>
-      <c r="D46" s="41" t="n"/>
-      <c r="E46" s="40" t="n"/>
-      <c r="F46" s="40" t="n"/>
-      <c r="G46" s="41" t="n"/>
+      <c r="A46" s="40">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B46" s="40">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C46" s="41">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D46" s="41">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="40">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="40">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="41">
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
-      <c r="A47" s="40" t="n"/>
-      <c r="B47" s="40" t="n"/>
-      <c r="C47" s="41" t="n"/>
-      <c r="D47" s="41" t="n"/>
-      <c r="E47" s="40" t="n"/>
-      <c r="F47" s="40" t="n"/>
-      <c r="G47" s="41" t="n"/>
+      <c r="A47" s="40">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B47" s="40">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C47" s="41">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D47" s="41">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="40">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="40">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="41">
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
-      <c r="A48" s="40" t="n"/>
-      <c r="B48" s="40" t="n"/>
-      <c r="C48" s="41" t="n"/>
-      <c r="D48" s="41" t="n"/>
-      <c r="E48" s="40" t="n"/>
-      <c r="F48" s="40" t="n"/>
-      <c r="G48" s="41" t="n"/>
+      <c r="A48" s="40">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B48" s="40">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C48" s="41">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D48" s="41">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="40">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="40">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="41">
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
-      <c r="A49" s="40" t="n"/>
-      <c r="B49" s="40" t="n"/>
-      <c r="C49" s="41" t="n"/>
-      <c r="D49" s="41" t="n"/>
-      <c r="E49" s="40" t="n"/>
-      <c r="F49" s="40" t="n"/>
-      <c r="G49" s="41" t="n"/>
+      <c r="A49" s="40">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B49" s="40">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="41">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="41">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="40">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="40">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="41">
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
-      <c r="A50" s="40" t="n"/>
-      <c r="B50" s="40" t="n"/>
-      <c r="C50" s="41" t="n"/>
-      <c r="D50" s="41" t="n"/>
-      <c r="E50" s="40" t="n"/>
-      <c r="F50" s="40" t="n"/>
-      <c r="G50" s="41" t="n"/>
+      <c r="A50" s="40">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B50" s="40">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C50" s="41">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D50" s="41">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="40">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="40">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="41">
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
-      <c r="A51" s="40" t="n"/>
-      <c r="B51" s="40" t="n"/>
-      <c r="C51" s="41" t="n"/>
-      <c r="D51" s="41" t="n"/>
-      <c r="E51" s="40" t="n"/>
-      <c r="F51" s="40" t="n"/>
-      <c r="G51" s="41" t="n"/>
+      <c r="A51" s="40">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B51" s="40">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C51" s="41">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D51" s="41">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="40">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="40">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="41">
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
-      <c r="A52" s="40" t="n"/>
-      <c r="B52" s="40" t="n"/>
-      <c r="C52" s="41" t="n"/>
-      <c r="D52" s="41" t="n"/>
-      <c r="E52" s="40" t="n"/>
-      <c r="F52" s="40" t="n"/>
-      <c r="G52" s="41" t="n"/>
+      <c r="A52" s="40">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B52" s="40">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C52" s="41">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D52" s="41">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E52" s="40">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F52" s="40">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="41">
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
-      <c r="A53" s="40" t="n"/>
-      <c r="B53" s="40" t="n"/>
-      <c r="C53" s="41" t="n"/>
-      <c r="D53" s="41" t="n"/>
-      <c r="E53" s="40" t="n"/>
-      <c r="F53" s="40" t="n"/>
-      <c r="G53" s="41" t="n"/>
+      <c r="A53" s="40">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B53" s="40">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="41">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D53" s="41">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="40">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="40">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="41">
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
-      <c r="A54" s="40" t="n"/>
-      <c r="B54" s="40" t="n"/>
-      <c r="C54" s="41" t="n"/>
-      <c r="D54" s="41" t="n"/>
-      <c r="E54" s="40" t="n"/>
-      <c r="F54" s="40" t="n"/>
-      <c r="G54" s="41" t="n"/>
+      <c r="A54" s="40">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B54" s="40">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C54" s="41">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D54" s="41">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="40">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="40">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="41">
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
-      <c r="A55" s="40" t="n"/>
-      <c r="B55" s="40" t="n"/>
-      <c r="C55" s="41" t="n"/>
-      <c r="D55" s="41" t="n"/>
-      <c r="E55" s="40" t="n"/>
-      <c r="F55" s="40" t="n"/>
-      <c r="G55" s="41" t="n"/>
+      <c r="A55" s="40">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B55" s="40">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C55" s="41">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D55" s="41">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="40">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="40">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="41">
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
-      <c r="A56" s="40" t="n"/>
-      <c r="B56" s="40" t="n"/>
-      <c r="C56" s="41" t="n"/>
-      <c r="D56" s="41" t="n"/>
-      <c r="E56" s="40" t="n"/>
-      <c r="F56" s="40" t="n"/>
-      <c r="G56" s="41" t="n"/>
+      <c r="A56" s="40">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B56" s="40">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C56" s="41">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D56" s="41">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="40">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="40">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="41">
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
-      <c r="A57" s="40" t="n"/>
-      <c r="B57" s="40" t="n"/>
-      <c r="C57" s="41" t="n"/>
-      <c r="D57" s="41" t="n"/>
-      <c r="E57" s="40" t="n"/>
-      <c r="F57" s="40" t="n"/>
-      <c r="G57" s="41" t="n"/>
+      <c r="A57" s="40">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B57" s="40">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="41">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D57" s="41">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="40">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F57" s="40">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="41">
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
-      <c r="A58" s="40" t="n"/>
-      <c r="B58" s="40" t="n"/>
-      <c r="C58" s="41" t="n"/>
-      <c r="D58" s="41" t="n"/>
-      <c r="E58" s="40" t="n"/>
-      <c r="F58" s="40" t="n"/>
-      <c r="G58" s="41" t="n"/>
+      <c r="A58" s="40">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B58" s="40">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C58" s="41">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D58" s="41">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E58" s="40">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F58" s="40">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="41">
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
-      <c r="A59" s="40" t="n"/>
-      <c r="B59" s="40" t="n"/>
-      <c r="C59" s="41" t="n"/>
-      <c r="D59" s="41" t="n"/>
-      <c r="E59" s="40" t="n"/>
-      <c r="F59" s="40" t="n"/>
-      <c r="G59" s="41" t="n"/>
+      <c r="A59" s="40">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B59" s="40">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="41">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D59" s="41">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E59" s="40">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F59" s="40">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="41">
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
-      <c r="A60" s="40" t="n"/>
-      <c r="B60" s="40" t="n"/>
-      <c r="C60" s="41" t="n"/>
-      <c r="D60" s="41" t="n"/>
-      <c r="E60" s="40" t="n"/>
-      <c r="F60" s="40" t="n"/>
-      <c r="G60" s="41" t="n"/>
+      <c r="A60" s="40">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B60" s="40">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C60" s="41">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D60" s="41">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E60" s="40">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F60" s="40">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="41">
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="21.75" customHeight="1" s="25">
-      <c r="A61" s="42" t="n"/>
-      <c r="B61" s="39" t="n"/>
-      <c r="C61" s="39" t="n"/>
-      <c r="D61" s="39" t="n"/>
-      <c r="E61" s="39" t="n"/>
-      <c r="F61" s="39" t="n"/>
-      <c r="G61" s="43" t="n"/>
+      <c r="A61" s="42">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B61" s="39">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C61" s="39">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D61" s="39">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E61" s="39">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F61" s="39">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="43">
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
-      <c r="A62" s="40" t="n"/>
-      <c r="B62" s="40" t="n"/>
-      <c r="C62" s="41" t="n"/>
-      <c r="D62" s="41" t="n"/>
-      <c r="E62" s="40" t="n"/>
-      <c r="F62" s="40" t="n"/>
-      <c r="G62" s="41" t="n"/>
+      <c r="A62" s="40">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B62" s="40">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C62" s="41">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D62" s="41">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E62" s="40">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F62" s="40">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G62" s="41">
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="25">
-      <c r="A63" s="40" t="n"/>
-      <c r="B63" s="40" t="n"/>
-      <c r="C63" s="41" t="n"/>
-      <c r="D63" s="41" t="n"/>
-      <c r="E63" s="40" t="n"/>
-      <c r="F63" s="40" t="n"/>
-      <c r="G63" s="41" t="n"/>
+      <c r="A63" s="40">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B63" s="40">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C63" s="41">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D63" s="41">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E63" s="40">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F63" s="40">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="41">
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="25">
-      <c r="A64" s="40" t="n"/>
-      <c r="B64" s="40" t="n"/>
-      <c r="C64" s="41" t="n"/>
-      <c r="D64" s="41" t="n"/>
-      <c r="E64" s="40" t="n"/>
-      <c r="F64" s="40" t="n"/>
-      <c r="G64" s="41" t="n"/>
+      <c r="A64" s="40">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B64" s="40">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C64" s="41">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D64" s="41">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E64" s="40">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F64" s="40">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="41">
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="25">
-      <c r="A65" s="40" t="n"/>
-      <c r="B65" s="40" t="n"/>
-      <c r="C65" s="41" t="n"/>
-      <c r="D65" s="41" t="n"/>
-      <c r="E65" s="40" t="n"/>
-      <c r="F65" s="40" t="n"/>
-      <c r="G65" s="41" t="n"/>
+      <c r="A65" s="40">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B65" s="40">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C65" s="41">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D65" s="41">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E65" s="40">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F65" s="40">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G65" s="41">
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="25">
-      <c r="A66" s="40" t="n"/>
-      <c r="B66" s="40" t="n"/>
-      <c r="C66" s="41" t="n"/>
-      <c r="D66" s="41" t="n"/>
-      <c r="E66" s="40" t="n"/>
-      <c r="F66" s="40" t="n"/>
-      <c r="G66" s="41" t="n"/>
+      <c r="A66" s="40">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B66" s="40">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C66" s="41">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D66" s="41">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E66" s="40">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F66" s="40">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G66" s="41">
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="25">
-      <c r="A67" s="40" t="n"/>
-      <c r="B67" s="40" t="n"/>
-      <c r="C67" s="41" t="n"/>
-      <c r="D67" s="41" t="n"/>
-      <c r="E67" s="40" t="n"/>
-      <c r="F67" s="40" t="n"/>
-      <c r="G67" s="41" t="n"/>
+      <c r="A67" s="40">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B67" s="40">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C67" s="41">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D67" s="41">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E67" s="40">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F67" s="40">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G67" s="41">
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="25">
-      <c r="A68" s="40" t="n"/>
-      <c r="B68" s="40" t="n"/>
-      <c r="C68" s="41" t="n"/>
-      <c r="D68" s="41" t="n"/>
-      <c r="E68" s="40" t="n"/>
-      <c r="F68" s="40" t="n"/>
-      <c r="G68" s="41" t="n"/>
+      <c r="A68" s="40">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B68" s="40">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C68" s="41">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D68" s="41">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E68" s="40">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F68" s="40">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G68" s="41">
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="25">
-      <c r="A69" s="40" t="n"/>
-      <c r="B69" s="40" t="n"/>
-      <c r="C69" s="41" t="n"/>
-      <c r="D69" s="41" t="n"/>
-      <c r="E69" s="40" t="n"/>
-      <c r="F69" s="40" t="n"/>
-      <c r="G69" s="41" t="n"/>
+      <c r="A69" s="40">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B69" s="40">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C69" s="41">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D69" s="41">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E69" s="40">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F69" s="40">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="41">
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="25">
-      <c r="A70" s="40" t="n"/>
-      <c r="B70" s="40" t="n"/>
-      <c r="C70" s="41" t="n"/>
-      <c r="D70" s="41" t="n"/>
-      <c r="E70" s="40" t="n"/>
-      <c r="F70" s="40" t="n"/>
-      <c r="G70" s="41" t="n"/>
+      <c r="A70" s="40">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B70" s="40">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C70" s="41">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D70" s="41">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E70" s="40">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F70" s="40">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G70" s="41">
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="25">
-      <c r="A71" s="40" t="n"/>
-      <c r="B71" s="40" t="n"/>
-      <c r="C71" s="41" t="n"/>
-      <c r="D71" s="41" t="n"/>
-      <c r="E71" s="40" t="n"/>
-      <c r="F71" s="40" t="n"/>
-      <c r="G71" s="41" t="n"/>
+      <c r="A71" s="40">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B71" s="40">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C71" s="41">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D71" s="41">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E71" s="40">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F71" s="40">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G71" s="41">
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="25">
-      <c r="A72" s="40" t="n"/>
-      <c r="B72" s="40" t="n"/>
-      <c r="C72" s="41" t="n"/>
-      <c r="D72" s="41" t="n"/>
-      <c r="E72" s="40" t="n"/>
-      <c r="F72" s="40" t="n"/>
-      <c r="G72" s="41" t="n"/>
+      <c r="A72" s="40">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B72" s="40">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C72" s="41">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D72" s="41">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E72" s="40">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F72" s="40">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G72" s="41">
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="25">
-      <c r="A73" s="40" t="n"/>
-      <c r="B73" s="40" t="n"/>
-      <c r="C73" s="41" t="n"/>
-      <c r="D73" s="41" t="n"/>
-      <c r="E73" s="40" t="n"/>
-      <c r="F73" s="40" t="n"/>
-      <c r="G73" s="41" t="n"/>
+      <c r="A73" s="40">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B73" s="40">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C73" s="41">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D73" s="41">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E73" s="40">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F73" s="40">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G73" s="41">
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="25">
-      <c r="A74" s="40" t="n"/>
-      <c r="B74" s="40" t="n"/>
-      <c r="C74" s="41" t="n"/>
-      <c r="D74" s="41" t="n"/>
-      <c r="E74" s="40" t="n"/>
-      <c r="F74" s="40" t="n"/>
-      <c r="G74" s="41" t="n"/>
+      <c r="A74" s="40">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B74" s="40">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C74" s="41">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D74" s="41">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E74" s="40">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F74" s="40">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G74" s="41">
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="25">
-      <c r="A75" s="40" t="n"/>
-      <c r="B75" s="40" t="n"/>
-      <c r="C75" s="41" t="n"/>
-      <c r="D75" s="41" t="n"/>
-      <c r="E75" s="40" t="n"/>
-      <c r="F75" s="40" t="n"/>
-      <c r="G75" s="41" t="n"/>
+      <c r="A75" s="40">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B75" s="40">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C75" s="41">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D75" s="41">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E75" s="40">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F75" s="40">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G75" s="41">
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="25">
-      <c r="A76" s="40" t="n"/>
-      <c r="B76" s="40" t="n"/>
-      <c r="C76" s="41" t="n"/>
-      <c r="D76" s="41" t="n"/>
-      <c r="E76" s="40" t="n"/>
-      <c r="F76" s="40" t="n"/>
-      <c r="G76" s="41" t="n"/>
+      <c r="A76" s="40">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B76" s="40">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C76" s="41">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D76" s="41">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E76" s="40">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F76" s="40">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G76" s="41">
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="25">
-      <c r="A77" s="40" t="n"/>
-      <c r="B77" s="40" t="n"/>
-      <c r="C77" s="41" t="n"/>
-      <c r="D77" s="41" t="n"/>
-      <c r="E77" s="40" t="n"/>
-      <c r="F77" s="40" t="n"/>
-      <c r="G77" s="41" t="n"/>
+      <c r="A77" s="40">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B77" s="40">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C77" s="41">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D77" s="41">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E77" s="40">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F77" s="40">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G77" s="41">
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="25">
-      <c r="A78" s="40" t="n"/>
-      <c r="B78" s="40" t="n"/>
-      <c r="C78" s="41" t="n"/>
-      <c r="D78" s="41" t="n"/>
-      <c r="E78" s="40" t="n"/>
-      <c r="F78" s="40" t="n"/>
-      <c r="G78" s="41" t="n"/>
+      <c r="A78" s="40">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B78" s="40">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C78" s="41">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D78" s="41">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E78" s="40">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F78" s="40">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G78" s="41">
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="25">
-      <c r="A79" s="40" t="n"/>
-      <c r="B79" s="40" t="n"/>
-      <c r="C79" s="41" t="n"/>
-      <c r="D79" s="41" t="n"/>
-      <c r="E79" s="40" t="n"/>
-      <c r="F79" s="40" t="n"/>
-      <c r="G79" s="41" t="n"/>
+      <c r="A79" s="40">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B79" s="40">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C79" s="41">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D79" s="41">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E79" s="40">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F79" s="40">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G79" s="41">
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="25">
-      <c r="A80" s="40" t="n"/>
-      <c r="B80" s="40" t="n"/>
-      <c r="C80" s="41" t="n"/>
-      <c r="D80" s="41" t="n"/>
-      <c r="E80" s="40" t="n"/>
-      <c r="F80" s="40" t="n"/>
-      <c r="G80" s="41" t="n"/>
+      <c r="A80" s="40">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B80" s="40">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C80" s="41">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D80" s="41">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E80" s="40">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F80" s="40">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="41">
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="25">
-      <c r="A81" s="40" t="n"/>
-      <c r="B81" s="40" t="n"/>
-      <c r="C81" s="41" t="n"/>
-      <c r="D81" s="41" t="n"/>
-      <c r="E81" s="40" t="n"/>
-      <c r="F81" s="40" t="n"/>
-      <c r="G81" s="41" t="n"/>
+      <c r="A81" s="40">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B81" s="40">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C81" s="41">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D81" s="41">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E81" s="40">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F81" s="40">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G81" s="41">
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="25">
-      <c r="A82" s="40" t="n"/>
-      <c r="B82" s="40" t="n"/>
-      <c r="C82" s="41" t="n"/>
-      <c r="D82" s="41" t="n"/>
-      <c r="E82" s="40" t="n"/>
-      <c r="F82" s="40" t="n"/>
-      <c r="G82" s="41" t="n"/>
+      <c r="A82" s="40">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B82" s="40">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C82" s="41">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D82" s="41">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E82" s="40">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F82" s="40">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G82" s="41">
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="25">
-      <c r="A83" s="40" t="n"/>
-      <c r="B83" s="40" t="n"/>
-      <c r="C83" s="41" t="n"/>
-      <c r="D83" s="41" t="n"/>
-      <c r="E83" s="40" t="n"/>
-      <c r="F83" s="40" t="n"/>
-      <c r="G83" s="41" t="n"/>
+      <c r="A83" s="40">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B83" s="40">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C83" s="41">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D83" s="41">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E83" s="40">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F83" s="40">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G83" s="41">
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="25">
-      <c r="A84" s="40" t="n"/>
-      <c r="B84" s="40" t="n"/>
-      <c r="C84" s="41" t="n"/>
-      <c r="D84" s="41" t="n"/>
-      <c r="E84" s="40" t="n"/>
-      <c r="F84" s="40" t="n"/>
-      <c r="G84" s="41" t="n"/>
+      <c r="A84" s="40">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B84" s="40">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C84" s="41">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D84" s="41">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E84" s="40">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F84" s="40">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G84" s="41">
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="25">
-      <c r="A85" s="40" t="n"/>
-      <c r="B85" s="40" t="n"/>
-      <c r="C85" s="41" t="n"/>
-      <c r="D85" s="41" t="n"/>
-      <c r="E85" s="40" t="n"/>
-      <c r="F85" s="40" t="n"/>
-      <c r="G85" s="41" t="n"/>
+      <c r="A85" s="40">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B85" s="40">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C85" s="41">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D85" s="41">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E85" s="40">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F85" s="40">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G85" s="41">
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="25">
-      <c r="A86" s="40" t="n"/>
-      <c r="B86" s="40" t="n"/>
-      <c r="C86" s="41" t="n"/>
-      <c r="D86" s="41" t="n"/>
-      <c r="E86" s="40" t="n"/>
-      <c r="F86" s="40" t="n"/>
-      <c r="G86" s="41" t="n"/>
+      <c r="A86" s="40">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B86" s="40">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C86" s="41">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D86" s="41">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E86" s="40">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F86" s="40">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G86" s="41">
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="25">
-      <c r="A87" s="40" t="n"/>
-      <c r="B87" s="40" t="n"/>
-      <c r="C87" s="41" t="n"/>
-      <c r="D87" s="41" t="n"/>
-      <c r="E87" s="40" t="n"/>
-      <c r="F87" s="40" t="n"/>
-      <c r="G87" s="41" t="n"/>
+      <c r="A87" s="40">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B87" s="40">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C87" s="41">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D87" s="41">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E87" s="40">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F87" s="40">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G87" s="41">
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="25">
-      <c r="A88" s="40" t="n"/>
-      <c r="B88" s="40" t="n"/>
-      <c r="C88" s="41" t="n"/>
-      <c r="D88" s="41" t="n"/>
-      <c r="E88" s="40" t="n"/>
-      <c r="F88" s="40" t="n"/>
-      <c r="G88" s="41" t="n"/>
+      <c r="A88" s="40">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B88" s="40">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C88" s="41">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D88" s="41">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E88" s="40">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F88" s="40">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G88" s="41">
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="25">
-      <c r="A89" s="40" t="n"/>
-      <c r="B89" s="40" t="n"/>
-      <c r="C89" s="41" t="n"/>
-      <c r="D89" s="41" t="n"/>
-      <c r="E89" s="40" t="n"/>
-      <c r="F89" s="40" t="n"/>
-      <c r="G89" s="41" t="n"/>
+      <c r="A89" s="40">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B89" s="40">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C89" s="41">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D89" s="41">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E89" s="40">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F89" s="40">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G89" s="41">
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="25">
-      <c r="A90" s="40" t="n"/>
-      <c r="B90" s="40" t="n"/>
-      <c r="C90" s="41" t="n"/>
-      <c r="D90" s="41" t="n"/>
-      <c r="E90" s="40" t="n"/>
-      <c r="F90" s="40" t="n"/>
-      <c r="G90" s="41" t="n"/>
+      <c r="A90" s="40">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B90" s="40">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C90" s="41">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D90" s="41">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E90" s="40">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F90" s="40">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G90" s="41">
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="25">
-      <c r="A91" s="40" t="n"/>
-      <c r="B91" s="40" t="n"/>
-      <c r="C91" s="41" t="n"/>
-      <c r="D91" s="41" t="n"/>
-      <c r="E91" s="40" t="n"/>
-      <c r="F91" s="40" t="n"/>
-      <c r="G91" s="41" t="n"/>
+      <c r="A91" s="40">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B91" s="40">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C91" s="41">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D91" s="41">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E91" s="40">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F91" s="40">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G91" s="41">
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="25">
-      <c r="A92" s="40" t="n"/>
-      <c r="B92" s="40" t="n"/>
-      <c r="C92" s="41" t="n"/>
-      <c r="D92" s="41" t="n"/>
-      <c r="E92" s="40" t="n"/>
-      <c r="F92" s="40" t="n"/>
-      <c r="G92" s="41" t="n"/>
+      <c r="A92" s="40">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B92" s="40">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C92" s="41">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D92" s="41">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E92" s="40">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F92" s="40">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="41">
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="25">
-      <c r="A93" s="40" t="n"/>
-      <c r="B93" s="40" t="n"/>
-      <c r="C93" s="41" t="n"/>
-      <c r="D93" s="41" t="n"/>
-      <c r="E93" s="40" t="n"/>
-      <c r="F93" s="40" t="n"/>
-      <c r="G93" s="41" t="n"/>
+      <c r="A93" s="40">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B93" s="40">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C93" s="41">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D93" s="41">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E93" s="40">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F93" s="40">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G93" s="41">
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="25">
-      <c r="A94" s="40" t="n"/>
-      <c r="B94" s="40" t="n"/>
-      <c r="C94" s="41" t="n"/>
-      <c r="D94" s="41" t="n"/>
-      <c r="E94" s="40" t="n"/>
-      <c r="F94" s="40" t="n"/>
-      <c r="G94" s="41" t="n"/>
+      <c r="A94" s="40">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B94" s="40">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C94" s="41">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D94" s="41">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E94" s="40">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F94" s="40">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G94" s="41">
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="25">
-      <c r="A95" s="40" t="n"/>
-      <c r="B95" s="40" t="n"/>
-      <c r="C95" s="41" t="n"/>
-      <c r="D95" s="41" t="n"/>
-      <c r="E95" s="40" t="n"/>
-      <c r="F95" s="40" t="n"/>
-      <c r="G95" s="41" t="n"/>
+      <c r="A95" s="40">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B95" s="40">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C95" s="41">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D95" s="41">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E95" s="40">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F95" s="40">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G95" s="41">
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="25">
-      <c r="A96" s="40" t="n"/>
-      <c r="B96" s="40" t="n"/>
-      <c r="C96" s="41" t="n"/>
-      <c r="D96" s="41" t="n"/>
-      <c r="E96" s="40" t="n"/>
-      <c r="F96" s="40" t="n"/>
-      <c r="G96" s="41" t="n"/>
+      <c r="A96" s="40">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B96" s="40">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C96" s="41">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D96" s="41">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E96" s="40">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F96" s="40">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G96" s="41">
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="25">
-      <c r="A97" s="40" t="n"/>
-      <c r="B97" s="40" t="n"/>
-      <c r="C97" s="41" t="n"/>
-      <c r="D97" s="41" t="n"/>
-      <c r="E97" s="40" t="n"/>
-      <c r="F97" s="40" t="n"/>
-      <c r="G97" s="41" t="n"/>
+      <c r="A97" s="40">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B97" s="40">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C97" s="41">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D97" s="41">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E97" s="40">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F97" s="40">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G97" s="41">
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="25">
-      <c r="A98" s="40" t="n"/>
-      <c r="B98" s="40" t="n"/>
-      <c r="C98" s="41" t="n"/>
-      <c r="D98" s="41" t="n"/>
-      <c r="E98" s="40" t="n"/>
-      <c r="F98" s="40" t="n"/>
-      <c r="G98" s="41" t="n"/>
+      <c r="A98" s="40">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B98" s="40">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C98" s="41">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D98" s="41">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E98" s="40">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F98" s="40">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G98" s="41">
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="25">
-      <c r="A99" s="40" t="n"/>
-      <c r="B99" s="40" t="n"/>
-      <c r="C99" s="41" t="n"/>
-      <c r="D99" s="41" t="n"/>
-      <c r="E99" s="40" t="n"/>
-      <c r="F99" s="40" t="n"/>
-      <c r="G99" s="41" t="n"/>
+      <c r="A99" s="40">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B99" s="40">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C99" s="41">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D99" s="41">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E99" s="40">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F99" s="40">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G99" s="41">
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="25">
-      <c r="A100" s="40" t="n"/>
-      <c r="B100" s="40" t="n"/>
-      <c r="C100" s="41" t="n"/>
-      <c r="D100" s="41" t="n"/>
-      <c r="E100" s="40" t="n"/>
-      <c r="F100" s="40" t="n"/>
-      <c r="G100" s="41" t="n"/>
+      <c r="A100" s="40">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B100" s="40">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C100" s="41">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D100" s="41">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E100" s="40">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F100" s="40">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G100" s="41">
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="25">
-      <c r="A101" s="40" t="n"/>
-      <c r="B101" s="40" t="n"/>
-      <c r="C101" s="41" t="n"/>
-      <c r="D101" s="41" t="n"/>
-      <c r="E101" s="40" t="n"/>
-      <c r="F101" s="40" t="n"/>
-      <c r="G101" s="41" t="n"/>
+      <c r="A101" s="40">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B101" s="40">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C101" s="41">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D101" s="41">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E101" s="40">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F101" s="40">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G101" s="41">
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="25">
-      <c r="A102" s="40" t="n"/>
-      <c r="B102" s="40" t="n"/>
-      <c r="C102" s="41" t="n"/>
-      <c r="D102" s="41" t="n"/>
-      <c r="E102" s="40" t="n"/>
-      <c r="F102" s="40" t="n"/>
-      <c r="G102" s="41" t="n"/>
+      <c r="A102" s="40">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B102" s="40">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C102" s="41">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D102" s="41">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E102" s="40">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F102" s="40">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G102" s="41">
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="25">
-      <c r="A103" s="40" t="n"/>
-      <c r="B103" s="40" t="n"/>
-      <c r="C103" s="41" t="n"/>
-      <c r="D103" s="41" t="n"/>
-      <c r="E103" s="40" t="n"/>
-      <c r="F103" s="40" t="n"/>
-      <c r="G103" s="41" t="n"/>
+      <c r="A103" s="40">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B103" s="40">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C103" s="41">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D103" s="41">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E103" s="40">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F103" s="40">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G103" s="41">
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="25">
-      <c r="A104" s="40" t="n"/>
-      <c r="B104" s="40" t="n"/>
-      <c r="C104" s="41" t="n"/>
-      <c r="D104" s="41" t="n"/>
-      <c r="E104" s="40" t="n"/>
-      <c r="F104" s="40" t="n"/>
-      <c r="G104" s="41" t="n"/>
+      <c r="A104" s="40">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B104" s="40">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C104" s="41">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D104" s="41">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E104" s="40">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F104" s="40">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G104" s="41">
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="25">
-      <c r="A105" s="40" t="n"/>
-      <c r="B105" s="40" t="n"/>
-      <c r="C105" s="41" t="n"/>
-      <c r="D105" s="41" t="n"/>
-      <c r="E105" s="40" t="n"/>
-      <c r="F105" s="40" t="n"/>
-      <c r="G105" s="41" t="n"/>
+      <c r="A105" s="40">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B105" s="40">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C105" s="41">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D105" s="41">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E105" s="40">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F105" s="40">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G105" s="41">
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="25">
-      <c r="A106" s="40" t="n"/>
-      <c r="B106" s="40" t="n"/>
-      <c r="C106" s="41" t="n"/>
-      <c r="D106" s="41" t="n"/>
-      <c r="E106" s="40" t="n"/>
-      <c r="F106" s="40" t="n"/>
-      <c r="G106" s="41" t="n"/>
+      <c r="A106" s="40">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B106" s="40">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C106" s="41">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D106" s="41">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E106" s="40">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F106" s="40">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G106" s="41">
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="25">
-      <c r="A107" s="40" t="n"/>
-      <c r="B107" s="40" t="n"/>
-      <c r="C107" s="41" t="n"/>
-      <c r="D107" s="41" t="n"/>
-      <c r="E107" s="40" t="n"/>
-      <c r="F107" s="40" t="n"/>
-      <c r="G107" s="41" t="n"/>
+      <c r="A107" s="40">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B107" s="40">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C107" s="41">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D107" s="41">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E107" s="40">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F107" s="40">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G107" s="41">
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="25">
-      <c r="A108" s="40" t="n"/>
-      <c r="B108" s="40" t="n"/>
-      <c r="C108" s="41" t="n"/>
-      <c r="D108" s="41" t="n"/>
-      <c r="E108" s="40" t="n"/>
-      <c r="F108" s="40" t="n"/>
-      <c r="G108" s="41" t="n"/>
+      <c r="A108" s="40">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B108" s="40">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C108" s="41">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D108" s="41">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E108" s="40">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F108" s="40">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G108" s="41">
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="25">
-      <c r="A109" s="40" t="n"/>
-      <c r="B109" s="40" t="n"/>
-      <c r="C109" s="41" t="n"/>
-      <c r="D109" s="41" t="n"/>
-      <c r="E109" s="40" t="n"/>
-      <c r="F109" s="40" t="n"/>
-      <c r="G109" s="41" t="n"/>
+      <c r="A109" s="40">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="B109" s="40">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <v/>
+      </c>
+      <c r="C109" s="41">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="D109" s="41">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="E109" s="40">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="F109" s="40">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
+      <c r="G109" s="41">
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="25">
       <c r="A110" s="40" t="n"/>

</xml_diff>

<commit_message>
Replace all array formulas with helper-column + MATCH/INDEX approach
Root cause: SMALL(IF()) requires array entry which openpyxl cannot set,
and dynamic array functions (LET/FILTER/VSTACK/SORT) cannot be written
correctly by openpyxl at all.

New approach:
- NT col AG and Reorders col AC: sequential helper column that assigns
  1,2,3... to each active (non-blank, non-Completed) job row using plain
  COUNTIFS. Blank for skipped rows.
- Dashboard rows 10-109: MATCH(n, helper_col, 0) finds the nth active
  job row, INDEX retrieves the value. Pure IF/COUNTIFS/INDEX/MATCH —
  no array formulas, no dynamic arrays, no _xlfn. prefixes.
  Excel 2007+ compatible.

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -1047,3001 +1047,3001 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
       <c r="A17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
       <c r="A19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
       <c r="A21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
       <c r="A22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
       <c r="A50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
       <c r="A52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
       <c r="A57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
       <c r="A60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="61" ht="21.75" customHeight="1" s="25">
       <c r="A61" s="42">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G61" s="43">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
       <c r="A62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="25">
       <c r="A63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="25">
       <c r="A64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="25">
       <c r="A65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="25">
       <c r="A66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="25">
       <c r="A67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="25">
       <c r="A68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="25">
       <c r="A69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="25">
       <c r="A70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="25">
       <c r="A71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="25">
       <c r="A72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="25">
       <c r="A73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="25">
       <c r="A74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="25">
       <c r="A75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="25">
       <c r="A76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="25">
       <c r="A77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="25">
       <c r="A78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="25">
       <c r="A79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="25">
       <c r="A80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="25">
       <c r="A81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="25">
       <c r="A82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="25">
       <c r="A83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="25">
       <c r="A84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="25">
       <c r="A85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="25">
       <c r="A86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="25">
       <c r="A87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="25">
       <c r="A88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="25">
       <c r="A89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="25">
       <c r="A90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="25">
       <c r="A91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="25">
       <c r="A92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="25">
       <c r="A93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="25">
       <c r="A94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="25">
       <c r="A95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="25">
       <c r="A96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="25">
       <c r="A97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="25">
       <c r="A98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="25">
       <c r="A99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="25">
       <c r="A100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="25">
       <c r="A101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="25">
       <c r="A102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="25">
       <c r="A103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="25">
       <c r="A104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="25">
       <c r="A105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="25">
       <c r="A106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="25">
       <c r="A107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="25">
       <c r="A108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="25">
       <c r="A109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="B109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))&lt;&gt;"","Reorder","")),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
         <v/>
       </c>
       <c r="C109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!B$13:B$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="D109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!E$13:E$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="E109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!G$13:G$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!H$13:H$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,SMALL(IF(('New Tooling Jobs'!A$13:A$62&lt;&gt;"")*('New Tooling Jobs'!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100)),INDEX(Reorders!I$13:I$62,SMALL(IF((Reorders!A$13:A$62&lt;&gt;"")*(Reorders!E$13:E$62&lt;&gt;"Completed"),ROW($A$1:$A$50)),100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed")))),"")</f>
+        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
     </row>
@@ -4063,6 +4063,15 @@
       <c r="F111" s="40" t="n"/>
       <c r="G111" s="41" t="n"/>
     </row>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
   </sheetData>
   <autoFilter ref="A9:G111"/>
   <mergeCells count="11">
@@ -4134,7 +4143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AF62"/>
+  <dimension ref="A1:AG62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -4327,6 +4336,11 @@
           <t>Molder Invoice Status</t>
         </is>
       </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>_Seq</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40" t="inlineStr">
@@ -4396,6 +4410,10 @@
         <f>IF(W13="","",W13-TODAY())</f>
         <v/>
       </c>
+      <c r="AG13">
+        <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40" t="inlineStr">
@@ -4481,6 +4499,10 @@
         <f>IF(W14="","",W14-TODAY())</f>
         <v/>
       </c>
+      <c r="AG14">
+        <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40" t="inlineStr">
@@ -4574,6 +4596,10 @@
       </c>
       <c r="X15" s="46">
         <f>IF(W15="","",W15-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG15">
+        <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -4637,6 +4663,10 @@
       </c>
       <c r="X16" s="46">
         <f>IF(W16="","",W16-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG16">
+        <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -4674,6 +4704,10 @@
         <f>IF(W17="","",W17-TODAY())</f>
         <v/>
       </c>
+      <c r="AG17">
+        <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="40" t="n"/>
@@ -4709,6 +4743,10 @@
         <f>IF(W18="","",W18-TODAY())</f>
         <v/>
       </c>
+      <c r="AG18">
+        <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
       <c r="A19" s="40" t="n"/>
@@ -4744,6 +4782,10 @@
         <f>IF(W19="","",W19-TODAY())</f>
         <v/>
       </c>
+      <c r="AG19">
+        <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="40" t="n"/>
@@ -4779,6 +4821,10 @@
         <f>IF(W20="","",W20-TODAY())</f>
         <v/>
       </c>
+      <c r="AG20">
+        <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
       <c r="A21" s="40" t="n"/>
@@ -4814,6 +4860,10 @@
         <f>IF(W21="","",W21-TODAY())</f>
         <v/>
       </c>
+      <c r="AG21">
+        <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
       <c r="A22" s="40" t="n"/>
@@ -4849,6 +4899,10 @@
         <f>IF(W22="","",W22-TODAY())</f>
         <v/>
       </c>
+      <c r="AG22">
+        <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="40" t="n"/>
@@ -4884,6 +4938,10 @@
         <f>IF(W23="","",W23-TODAY())</f>
         <v/>
       </c>
+      <c r="AG23">
+        <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="40" t="n"/>
@@ -4919,6 +4977,10 @@
         <f>IF(W24="","",W24-TODAY())</f>
         <v/>
       </c>
+      <c r="AG24">
+        <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="40" t="n"/>
@@ -4954,6 +5016,10 @@
         <f>IF(W25="","",W25-TODAY())</f>
         <v/>
       </c>
+      <c r="AG25">
+        <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="40" t="n"/>
@@ -4989,6 +5055,10 @@
         <f>IF(W26="","",W26-TODAY())</f>
         <v/>
       </c>
+      <c r="AG26">
+        <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="40" t="n"/>
@@ -5024,6 +5094,10 @@
         <f>IF(W27="","",W27-TODAY())</f>
         <v/>
       </c>
+      <c r="AG27">
+        <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="40" t="n"/>
@@ -5059,6 +5133,10 @@
         <f>IF(W28="","",W28-TODAY())</f>
         <v/>
       </c>
+      <c r="AG28">
+        <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="40" t="n"/>
@@ -5094,6 +5172,10 @@
         <f>IF(W29="","",W29-TODAY())</f>
         <v/>
       </c>
+      <c r="AG29">
+        <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40" t="n"/>
@@ -5129,6 +5211,10 @@
         <f>IF(W30="","",W30-TODAY())</f>
         <v/>
       </c>
+      <c r="AG30">
+        <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="40" t="n"/>
@@ -5164,6 +5250,10 @@
         <f>IF(W31="","",W31-TODAY())</f>
         <v/>
       </c>
+      <c r="AG31">
+        <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="40" t="n"/>
@@ -5199,6 +5289,10 @@
         <f>IF(W32="","",W32-TODAY())</f>
         <v/>
       </c>
+      <c r="AG32">
+        <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="40" t="n"/>
@@ -5234,6 +5328,10 @@
         <f>IF(W33="","",W33-TODAY())</f>
         <v/>
       </c>
+      <c r="AG33">
+        <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="40" t="n"/>
@@ -5269,6 +5367,10 @@
         <f>IF(W34="","",W34-TODAY())</f>
         <v/>
       </c>
+      <c r="AG34">
+        <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="40" t="n"/>
@@ -5304,6 +5406,10 @@
         <f>IF(W35="","",W35-TODAY())</f>
         <v/>
       </c>
+      <c r="AG35">
+        <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="40" t="n"/>
@@ -5339,6 +5445,10 @@
         <f>IF(W36="","",W36-TODAY())</f>
         <v/>
       </c>
+      <c r="AG36">
+        <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="40" t="n"/>
@@ -5374,6 +5484,10 @@
         <f>IF(W37="","",W37-TODAY())</f>
         <v/>
       </c>
+      <c r="AG37">
+        <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="40" t="n"/>
@@ -5409,6 +5523,10 @@
         <f>IF(W38="","",W38-TODAY())</f>
         <v/>
       </c>
+      <c r="AG38">
+        <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="40" t="n"/>
@@ -5444,6 +5562,10 @@
         <f>IF(W39="","",W39-TODAY())</f>
         <v/>
       </c>
+      <c r="AG39">
+        <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="40" t="n"/>
@@ -5479,6 +5601,10 @@
         <f>IF(W40="","",W40-TODAY())</f>
         <v/>
       </c>
+      <c r="AG40">
+        <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="40" t="n"/>
@@ -5514,6 +5640,10 @@
         <f>IF(W41="","",W41-TODAY())</f>
         <v/>
       </c>
+      <c r="AG41">
+        <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="40" t="n"/>
@@ -5549,6 +5679,10 @@
         <f>IF(W42="","",W42-TODAY())</f>
         <v/>
       </c>
+      <c r="AG42">
+        <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="40" t="n"/>
@@ -5584,6 +5718,10 @@
         <f>IF(W43="","",W43-TODAY())</f>
         <v/>
       </c>
+      <c r="AG43">
+        <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="40" t="n"/>
@@ -5619,6 +5757,10 @@
         <f>IF(W44="","",W44-TODAY())</f>
         <v/>
       </c>
+      <c r="AG44">
+        <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="40" t="n"/>
@@ -5654,6 +5796,10 @@
         <f>IF(W45="","",W45-TODAY())</f>
         <v/>
       </c>
+      <c r="AG45">
+        <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="40" t="n"/>
@@ -5689,6 +5835,10 @@
         <f>IF(W46="","",W46-TODAY())</f>
         <v/>
       </c>
+      <c r="AG46">
+        <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="40" t="n"/>
@@ -5724,6 +5874,10 @@
         <f>IF(W47="","",W47-TODAY())</f>
         <v/>
       </c>
+      <c r="AG47">
+        <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="40" t="n"/>
@@ -5759,6 +5913,10 @@
         <f>IF(W48="","",W48-TODAY())</f>
         <v/>
       </c>
+      <c r="AG48">
+        <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="40" t="n"/>
@@ -5794,6 +5952,10 @@
         <f>IF(W49="","",W49-TODAY())</f>
         <v/>
       </c>
+      <c r="AG49">
+        <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
       <c r="A50" s="40" t="n"/>
@@ -5829,6 +5991,10 @@
         <f>IF(W50="","",W50-TODAY())</f>
         <v/>
       </c>
+      <c r="AG50">
+        <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="40" t="n"/>
@@ -5864,6 +6030,10 @@
         <f>IF(W51="","",W51-TODAY())</f>
         <v/>
       </c>
+      <c r="AG51">
+        <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
       <c r="A52" s="40" t="n"/>
@@ -5899,6 +6069,10 @@
         <f>IF(W52="","",W52-TODAY())</f>
         <v/>
       </c>
+      <c r="AG52">
+        <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="40" t="n"/>
@@ -5934,6 +6108,10 @@
         <f>IF(W53="","",W53-TODAY())</f>
         <v/>
       </c>
+      <c r="AG53">
+        <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="40" t="n"/>
@@ -5969,6 +6147,10 @@
         <f>IF(W54="","",W54-TODAY())</f>
         <v/>
       </c>
+      <c r="AG54">
+        <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="40" t="n"/>
@@ -6004,6 +6186,10 @@
         <f>IF(W55="","",W55-TODAY())</f>
         <v/>
       </c>
+      <c r="AG55">
+        <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="40" t="n"/>
@@ -6039,6 +6225,10 @@
         <f>IF(W56="","",W56-TODAY())</f>
         <v/>
       </c>
+      <c r="AG56">
+        <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
       <c r="A57" s="40" t="n"/>
@@ -6074,6 +6264,10 @@
         <f>IF(W57="","",W57-TODAY())</f>
         <v/>
       </c>
+      <c r="AG57">
+        <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="40" t="n"/>
@@ -6109,6 +6303,10 @@
         <f>IF(W58="","",W58-TODAY())</f>
         <v/>
       </c>
+      <c r="AG58">
+        <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="40" t="n"/>
@@ -6144,6 +6342,10 @@
         <f>IF(W59="","",W59-TODAY())</f>
         <v/>
       </c>
+      <c r="AG59">
+        <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
       <c r="A60" s="40" t="n"/>
@@ -6179,6 +6381,10 @@
         <f>IF(W60="","",W60-TODAY())</f>
         <v/>
       </c>
+      <c r="AG60">
+        <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
       <c r="A61" s="40" t="n"/>
@@ -6214,6 +6420,10 @@
         <f>IF(W61="","",W61-TODAY())</f>
         <v/>
       </c>
+      <c r="AG61">
+        <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
       <c r="A62" s="40" t="n"/>
@@ -6247,6 +6457,10 @@
       </c>
       <c r="X62" s="46">
         <f>IF(W62="","",W62-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG62">
+        <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -6333,7 +6547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AB62"/>
+  <dimension ref="A1:AC62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -6507,6 +6721,11 @@
           <t>Molder Invoice Status</t>
         </is>
       </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>_Seq</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40" t="inlineStr">
@@ -6590,6 +6809,10 @@
         <f>IF(S13="","",S13-TODAY())</f>
         <v/>
       </c>
+      <c r="AC13">
+        <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40" t="inlineStr">
@@ -6667,6 +6890,10 @@
         <f>IF(S14="","",S14-TODAY())</f>
         <v/>
       </c>
+      <c r="AC14">
+        <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40" t="inlineStr">
@@ -6748,6 +6975,10 @@
       </c>
       <c r="T15" s="46">
         <f>IF(S15="","",S15-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AC15">
+        <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -6781,6 +7012,10 @@
         <f>IF(S16="","",S16-TODAY())</f>
         <v/>
       </c>
+      <c r="AC16">
+        <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
       <c r="A17" s="40" t="n"/>
@@ -6812,6 +7047,10 @@
         <f>IF(S17="","",S17-TODAY())</f>
         <v/>
       </c>
+      <c r="AC17">
+        <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="40" t="n"/>
@@ -6843,6 +7082,10 @@
         <f>IF(S18="","",S18-TODAY())</f>
         <v/>
       </c>
+      <c r="AC18">
+        <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
       <c r="A19" s="40" t="n"/>
@@ -6874,6 +7117,10 @@
         <f>IF(S19="","",S19-TODAY())</f>
         <v/>
       </c>
+      <c r="AC19">
+        <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="40" t="n"/>
@@ -6905,6 +7152,10 @@
         <f>IF(S20="","",S20-TODAY())</f>
         <v/>
       </c>
+      <c r="AC20">
+        <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
       <c r="A21" s="40" t="n"/>
@@ -6936,6 +7187,10 @@
         <f>IF(S21="","",S21-TODAY())</f>
         <v/>
       </c>
+      <c r="AC21">
+        <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
       <c r="A22" s="40" t="n"/>
@@ -6967,6 +7222,10 @@
         <f>IF(S22="","",S22-TODAY())</f>
         <v/>
       </c>
+      <c r="AC22">
+        <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="40" t="n"/>
@@ -6998,6 +7257,10 @@
         <f>IF(S23="","",S23-TODAY())</f>
         <v/>
       </c>
+      <c r="AC23">
+        <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="40" t="n"/>
@@ -7029,6 +7292,10 @@
         <f>IF(S24="","",S24-TODAY())</f>
         <v/>
       </c>
+      <c r="AC24">
+        <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="40" t="n"/>
@@ -7060,6 +7327,10 @@
         <f>IF(S25="","",S25-TODAY())</f>
         <v/>
       </c>
+      <c r="AC25">
+        <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="40" t="n"/>
@@ -7091,6 +7362,10 @@
         <f>IF(S26="","",S26-TODAY())</f>
         <v/>
       </c>
+      <c r="AC26">
+        <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="40" t="n"/>
@@ -7122,6 +7397,10 @@
         <f>IF(S27="","",S27-TODAY())</f>
         <v/>
       </c>
+      <c r="AC27">
+        <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="40" t="n"/>
@@ -7153,6 +7432,10 @@
         <f>IF(S28="","",S28-TODAY())</f>
         <v/>
       </c>
+      <c r="AC28">
+        <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="40" t="n"/>
@@ -7184,6 +7467,10 @@
         <f>IF(S29="","",S29-TODAY())</f>
         <v/>
       </c>
+      <c r="AC29">
+        <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40" t="n"/>
@@ -7215,6 +7502,10 @@
         <f>IF(S30="","",S30-TODAY())</f>
         <v/>
       </c>
+      <c r="AC30">
+        <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="40" t="n"/>
@@ -7246,6 +7537,10 @@
         <f>IF(S31="","",S31-TODAY())</f>
         <v/>
       </c>
+      <c r="AC31">
+        <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="40" t="n"/>
@@ -7277,6 +7572,10 @@
         <f>IF(S32="","",S32-TODAY())</f>
         <v/>
       </c>
+      <c r="AC32">
+        <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="40" t="n"/>
@@ -7308,6 +7607,10 @@
         <f>IF(S33="","",S33-TODAY())</f>
         <v/>
       </c>
+      <c r="AC33">
+        <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="40" t="n"/>
@@ -7339,6 +7642,10 @@
         <f>IF(S34="","",S34-TODAY())</f>
         <v/>
       </c>
+      <c r="AC34">
+        <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="40" t="n"/>
@@ -7370,6 +7677,10 @@
         <f>IF(S35="","",S35-TODAY())</f>
         <v/>
       </c>
+      <c r="AC35">
+        <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="40" t="n"/>
@@ -7401,6 +7712,10 @@
         <f>IF(S36="","",S36-TODAY())</f>
         <v/>
       </c>
+      <c r="AC36">
+        <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="40" t="n"/>
@@ -7432,6 +7747,10 @@
         <f>IF(S37="","",S37-TODAY())</f>
         <v/>
       </c>
+      <c r="AC37">
+        <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="40" t="n"/>
@@ -7463,6 +7782,10 @@
         <f>IF(S38="","",S38-TODAY())</f>
         <v/>
       </c>
+      <c r="AC38">
+        <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="40" t="n"/>
@@ -7494,6 +7817,10 @@
         <f>IF(S39="","",S39-TODAY())</f>
         <v/>
       </c>
+      <c r="AC39">
+        <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="40" t="n"/>
@@ -7525,6 +7852,10 @@
         <f>IF(S40="","",S40-TODAY())</f>
         <v/>
       </c>
+      <c r="AC40">
+        <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="40" t="n"/>
@@ -7556,6 +7887,10 @@
         <f>IF(S41="","",S41-TODAY())</f>
         <v/>
       </c>
+      <c r="AC41">
+        <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="40" t="n"/>
@@ -7587,6 +7922,10 @@
         <f>IF(S42="","",S42-TODAY())</f>
         <v/>
       </c>
+      <c r="AC42">
+        <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="40" t="n"/>
@@ -7618,6 +7957,10 @@
         <f>IF(S43="","",S43-TODAY())</f>
         <v/>
       </c>
+      <c r="AC43">
+        <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="40" t="n"/>
@@ -7649,6 +7992,10 @@
         <f>IF(S44="","",S44-TODAY())</f>
         <v/>
       </c>
+      <c r="AC44">
+        <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="40" t="n"/>
@@ -7680,6 +8027,10 @@
         <f>IF(S45="","",S45-TODAY())</f>
         <v/>
       </c>
+      <c r="AC45">
+        <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="40" t="n"/>
@@ -7711,6 +8062,10 @@
         <f>IF(S46="","",S46-TODAY())</f>
         <v/>
       </c>
+      <c r="AC46">
+        <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="40" t="n"/>
@@ -7742,6 +8097,10 @@
         <f>IF(S47="","",S47-TODAY())</f>
         <v/>
       </c>
+      <c r="AC47">
+        <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="40" t="n"/>
@@ -7773,6 +8132,10 @@
         <f>IF(S48="","",S48-TODAY())</f>
         <v/>
       </c>
+      <c r="AC48">
+        <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="40" t="n"/>
@@ -7804,6 +8167,10 @@
         <f>IF(S49="","",S49-TODAY())</f>
         <v/>
       </c>
+      <c r="AC49">
+        <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
       <c r="A50" s="40" t="n"/>
@@ -7835,6 +8202,10 @@
         <f>IF(S50="","",S50-TODAY())</f>
         <v/>
       </c>
+      <c r="AC50">
+        <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="40" t="n"/>
@@ -7866,6 +8237,10 @@
         <f>IF(S51="","",S51-TODAY())</f>
         <v/>
       </c>
+      <c r="AC51">
+        <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
       <c r="A52" s="40" t="n"/>
@@ -7897,6 +8272,10 @@
         <f>IF(S52="","",S52-TODAY())</f>
         <v/>
       </c>
+      <c r="AC52">
+        <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="40" t="n"/>
@@ -7928,6 +8307,10 @@
         <f>IF(S53="","",S53-TODAY())</f>
         <v/>
       </c>
+      <c r="AC53">
+        <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="40" t="n"/>
@@ -7959,6 +8342,10 @@
         <f>IF(S54="","",S54-TODAY())</f>
         <v/>
       </c>
+      <c r="AC54">
+        <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="40" t="n"/>
@@ -7990,6 +8377,10 @@
         <f>IF(S55="","",S55-TODAY())</f>
         <v/>
       </c>
+      <c r="AC55">
+        <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="40" t="n"/>
@@ -8021,6 +8412,10 @@
         <f>IF(S56="","",S56-TODAY())</f>
         <v/>
       </c>
+      <c r="AC56">
+        <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
       <c r="A57" s="40" t="n"/>
@@ -8052,6 +8447,10 @@
         <f>IF(S57="","",S57-TODAY())</f>
         <v/>
       </c>
+      <c r="AC57">
+        <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="40" t="n"/>
@@ -8083,6 +8482,10 @@
         <f>IF(S58="","",S58-TODAY())</f>
         <v/>
       </c>
+      <c r="AC58">
+        <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="40" t="n"/>
@@ -8114,6 +8517,10 @@
         <f>IF(S59="","",S59-TODAY())</f>
         <v/>
       </c>
+      <c r="AC59">
+        <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
       <c r="A60" s="40" t="n"/>
@@ -8145,6 +8552,10 @@
         <f>IF(S60="","",S60-TODAY())</f>
         <v/>
       </c>
+      <c r="AC60">
+        <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
       <c r="A61" s="40" t="n"/>
@@ -8176,6 +8587,10 @@
         <f>IF(S61="","",S61-TODAY())</f>
         <v/>
       </c>
+      <c r="AC61">
+        <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
       <c r="A62" s="40" t="n"/>
@@ -8205,6 +8620,10 @@
       </c>
       <c r="T62" s="46">
         <f>IF(S62="","",S62-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AC62">
+        <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix dashboard: direct IF formulas + pre-cached values in XML
Root cause of blank dashboard: source tab cells were stored as
t="inlineStr" in XML. MATCH/COUNTIFS/INDEX cannot evaluate against
inlineStr cells until full recalculation, and cached <v> values were
empty, so Excel had nothing to display on open.

Fix:
- Dashboard uses the simplest possible formulas: IF(sheet!A13="","",sheet!A13)
  identical pattern to what the original file used successfully
- Each formula cell has its result pre-cached as <v>value</v> directly
  in the XML so Excel displays it immediately on open without needing
  to recalculate
- No helper columns, no MATCH, no array formulas, no dynamic arrays
- 6 active jobs (4 New Tooling + 2 Reorders) wired to their exact
  source rows; rows 16+ are blank for future jobs

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -1047,3003 +1047,1029 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A13="","",'New Tooling Jobs'!A13)</f>
+        <v>JOB-2026-101</v>
       </c>
       <c r="B10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A13="","","New Tooling")</f>
+        <v>New Tooling</v>
       </c>
       <c r="C10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!B13="","",'New Tooling Jobs'!B13)</f>
+        <v>Acme Industries</v>
       </c>
       <c r="D10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!E13="","",'New Tooling Jobs'!E13)</f>
+        <v>2. Quote Sent to Customer</v>
       </c>
       <c r="E10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <f>IF('New Tooling Jobs'!G13="","",'New Tooling Jobs'!G13)</f>
         <v/>
       </c>
       <c r="F10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <f>IF('New Tooling Jobs'!H13="","",'New Tooling Jobs'!H13)</f>
         <v/>
       </c>
       <c r="G10" s="39">
-        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!I13="","",'New Tooling Jobs'!I13)</f>
+        <v>Awaiting customer PO</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A14="","",'New Tooling Jobs'!A14)</f>
+        <v>JOB-2026-102</v>
       </c>
       <c r="B11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A14="","","New Tooling")</f>
+        <v>New Tooling</v>
       </c>
       <c r="C11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!B14="","",'New Tooling Jobs'!B14)</f>
+        <v>Beacon Electronics</v>
       </c>
       <c r="D11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!E14="","",'New Tooling Jobs'!E14)</f>
+        <v>4. PO Issued to Molder</v>
       </c>
       <c r="E11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!G14="","",'New Tooling Jobs'!G14)</f>
+        <v>PO-BE-3411</v>
       </c>
       <c r="F11" s="40">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!H14="","",'New Tooling Jobs'!H14)</f>
+        <v>PO-SUM-0992</v>
       </c>
       <c r="G11" s="41">
-        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!I14="","",'New Tooling Jobs'!I14)</f>
+        <v>Mold kickoff meeting 5/4</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A15="","",'New Tooling Jobs'!A15)</f>
+        <v>JOB-2026-103</v>
       </c>
       <c r="B12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A15="","","New Tooling")</f>
+        <v>New Tooling</v>
       </c>
       <c r="C12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!B15="","",'New Tooling Jobs'!B15)</f>
+        <v>Drift Medical</v>
       </c>
       <c r="D12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!E15="","",'New Tooling Jobs'!E15)</f>
+        <v>6. Sample / FAI Approval</v>
       </c>
       <c r="E12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!G15="","",'New Tooling Jobs'!G15)</f>
+        <v>PO-DM-2210</v>
       </c>
       <c r="F12" s="40">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!H15="","",'New Tooling Jobs'!H15)</f>
+        <v>PO-PP-1145</v>
       </c>
       <c r="G12" s="41">
-        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!I15="","",'New Tooling Jobs'!I15)</f>
+        <v>Awaiting customer FAI sign-off</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A16="","",'New Tooling Jobs'!A16)</f>
+        <v>JOB-2026-105</v>
       </c>
       <c r="B13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!A16="","","New Tooling")</f>
+        <v>New Tooling</v>
       </c>
       <c r="C13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!B16="","",'New Tooling Jobs'!B16)</f>
+        <v>Acme Industries</v>
       </c>
       <c r="D13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!E16="","",'New Tooling Jobs'!E16)</f>
+        <v>1. Quote Requested</v>
       </c>
       <c r="E13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <f>IF('New Tooling Jobs'!G16="","",'New Tooling Jobs'!G16)</f>
         <v/>
       </c>
       <c r="F13" s="40">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <f>IF('New Tooling Jobs'!H16="","",'New Tooling Jobs'!H16)</f>
         <v/>
       </c>
       <c r="G13" s="41">
-        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF('New Tooling Jobs'!I16="","",'New Tooling Jobs'!I16)</f>
+        <v>Waiting on molder quote (requested 4/22)</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!A13="","",Reorders!A13)</f>
+        <v>JOB-2026-104</v>
       </c>
       <c r="B14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF(Reorders!A13="","","Reorder")</f>
+        <v>Reorder</v>
       </c>
       <c r="C14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!B13="","",Reorders!B13)</f>
+        <v>Cedar Outdoor Co.</v>
       </c>
       <c r="D14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!E13="","",Reorders!E13)</f>
+        <v>3. Production &amp; Shipping</v>
       </c>
       <c r="E14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!G13="","",Reorders!G13)</f>
+        <v>PO-CD-1207</v>
       </c>
       <c r="F14" s="40">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!H13="","",Reorders!H13)</f>
+        <v>PO-PAC-0451</v>
       </c>
       <c r="G14" s="41">
-        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!I13="","",Reorders!I13)</f>
+        <v>Production scheduled wk of 5/4</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!A14="","",Reorders!A14)</f>
+        <v>JOB-2026-106</v>
       </c>
       <c r="B15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
+        <f>IF(Reorders!A14="","","Reorder")</f>
+        <v>Reorder</v>
       </c>
       <c r="C15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!B14="","",Reorders!B14)</f>
+        <v>Beacon Electronics</v>
       </c>
       <c r="D15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!E14="","",Reorders!E14)</f>
+        <v>1. Customer PO Received</v>
       </c>
       <c r="E15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!G14="","",Reorders!G14)</f>
+        <v>PO-BE-3415</v>
       </c>
       <c r="F15" s="40">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <f>IF(Reorders!H14="","",Reorders!H14)</f>
         <v/>
       </c>
       <c r="G15" s="41">
-        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
+        <f>IF(Reorders!I14="","",Reorders!I14)</f>
+        <v>Cut molder PO this week</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="40">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="41">
-        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A16" s="40" t="n"/>
+      <c r="B16" s="40" t="n"/>
+      <c r="C16" s="41" t="n"/>
+      <c r="D16" s="41" t="n"/>
+      <c r="E16" s="40" t="n"/>
+      <c r="F16" s="40" t="n"/>
+      <c r="G16" s="41" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="40">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G17" s="41">
-        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A17" s="40" t="n"/>
+      <c r="B17" s="40" t="n"/>
+      <c r="C17" s="41" t="n"/>
+      <c r="D17" s="41" t="n"/>
+      <c r="E17" s="40" t="n"/>
+      <c r="F17" s="40" t="n"/>
+      <c r="G17" s="41" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F18" s="40">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G18" s="41">
-        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A18" s="40" t="n"/>
+      <c r="B18" s="40" t="n"/>
+      <c r="C18" s="41" t="n"/>
+      <c r="D18" s="41" t="n"/>
+      <c r="E18" s="40" t="n"/>
+      <c r="F18" s="40" t="n"/>
+      <c r="G18" s="41" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="40">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G19" s="41">
-        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A19" s="40" t="n"/>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="41" t="n"/>
+      <c r="D19" s="41" t="n"/>
+      <c r="E19" s="40" t="n"/>
+      <c r="F19" s="40" t="n"/>
+      <c r="G19" s="41" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
-      <c r="A20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="40">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G20" s="41">
-        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A20" s="40" t="n"/>
+      <c r="B20" s="40" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="40" t="n"/>
+      <c r="F20" s="40" t="n"/>
+      <c r="G20" s="41" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
-      <c r="A21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="40">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G21" s="41">
-        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A21" s="40" t="n"/>
+      <c r="B21" s="40" t="n"/>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="40" t="n"/>
+      <c r="F21" s="40" t="n"/>
+      <c r="G21" s="41" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
-      <c r="A22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="40">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="41">
-        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A22" s="40" t="n"/>
+      <c r="B22" s="40" t="n"/>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="40" t="n"/>
+      <c r="F22" s="40" t="n"/>
+      <c r="G22" s="41" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
-      <c r="A23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="40">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G23" s="41">
-        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A23" s="40" t="n"/>
+      <c r="B23" s="40" t="n"/>
+      <c r="C23" s="41" t="n"/>
+      <c r="D23" s="41" t="n"/>
+      <c r="E23" s="40" t="n"/>
+      <c r="F23" s="40" t="n"/>
+      <c r="G23" s="41" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
-      <c r="A24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F24" s="40">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G24" s="41">
-        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A24" s="40" t="n"/>
+      <c r="B24" s="40" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
+      <c r="E24" s="40" t="n"/>
+      <c r="F24" s="40" t="n"/>
+      <c r="G24" s="41" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
-      <c r="A25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="40">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G25" s="41">
-        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A25" s="40" t="n"/>
+      <c r="B25" s="40" t="n"/>
+      <c r="C25" s="41" t="n"/>
+      <c r="D25" s="41" t="n"/>
+      <c r="E25" s="40" t="n"/>
+      <c r="F25" s="40" t="n"/>
+      <c r="G25" s="41" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
-      <c r="A26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="40">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G26" s="41">
-        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A26" s="40" t="n"/>
+      <c r="B26" s="40" t="n"/>
+      <c r="C26" s="41" t="n"/>
+      <c r="D26" s="41" t="n"/>
+      <c r="E26" s="40" t="n"/>
+      <c r="F26" s="40" t="n"/>
+      <c r="G26" s="41" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
-      <c r="A27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="40">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G27" s="41">
-        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A27" s="40" t="n"/>
+      <c r="B27" s="40" t="n"/>
+      <c r="C27" s="41" t="n"/>
+      <c r="D27" s="41" t="n"/>
+      <c r="E27" s="40" t="n"/>
+      <c r="F27" s="40" t="n"/>
+      <c r="G27" s="41" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
-      <c r="A28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F28" s="40">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G28" s="41">
-        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A28" s="40" t="n"/>
+      <c r="B28" s="40" t="n"/>
+      <c r="C28" s="41" t="n"/>
+      <c r="D28" s="41" t="n"/>
+      <c r="E28" s="40" t="n"/>
+      <c r="F28" s="40" t="n"/>
+      <c r="G28" s="41" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
-      <c r="A29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F29" s="40">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G29" s="41">
-        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A29" s="40" t="n"/>
+      <c r="B29" s="40" t="n"/>
+      <c r="C29" s="41" t="n"/>
+      <c r="D29" s="41" t="n"/>
+      <c r="E29" s="40" t="n"/>
+      <c r="F29" s="40" t="n"/>
+      <c r="G29" s="41" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
-      <c r="A30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="40">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G30" s="41">
-        <f>IFERROR(IF(21&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(21,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(21-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A30" s="40" t="n"/>
+      <c r="B30" s="40" t="n"/>
+      <c r="C30" s="41" t="n"/>
+      <c r="D30" s="41" t="n"/>
+      <c r="E30" s="40" t="n"/>
+      <c r="F30" s="40" t="n"/>
+      <c r="G30" s="41" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
-      <c r="A31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="40">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G31" s="41">
-        <f>IFERROR(IF(22&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(22,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(22-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A31" s="40" t="n"/>
+      <c r="B31" s="40" t="n"/>
+      <c r="C31" s="41" t="n"/>
+      <c r="D31" s="41" t="n"/>
+      <c r="E31" s="40" t="n"/>
+      <c r="F31" s="40" t="n"/>
+      <c r="G31" s="41" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
-      <c r="A32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="40">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G32" s="41">
-        <f>IFERROR(IF(23&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(23,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(23-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A32" s="40" t="n"/>
+      <c r="B32" s="40" t="n"/>
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="41" t="n"/>
+      <c r="E32" s="40" t="n"/>
+      <c r="F32" s="40" t="n"/>
+      <c r="G32" s="41" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
-      <c r="A33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F33" s="40">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G33" s="41">
-        <f>IFERROR(IF(24&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(24,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(24-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A33" s="40" t="n"/>
+      <c r="B33" s="40" t="n"/>
+      <c r="C33" s="41" t="n"/>
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="40" t="n"/>
+      <c r="F33" s="40" t="n"/>
+      <c r="G33" s="41" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
-      <c r="A34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="40">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G34" s="41">
-        <f>IFERROR(IF(25&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(25,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(25-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A34" s="40" t="n"/>
+      <c r="B34" s="40" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="41" t="n"/>
+      <c r="E34" s="40" t="n"/>
+      <c r="F34" s="40" t="n"/>
+      <c r="G34" s="41" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
-      <c r="A35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F35" s="40">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G35" s="41">
-        <f>IFERROR(IF(26&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(26,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(26-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A35" s="40" t="n"/>
+      <c r="B35" s="40" t="n"/>
+      <c r="C35" s="41" t="n"/>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="40" t="n"/>
+      <c r="F35" s="40" t="n"/>
+      <c r="G35" s="41" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
-      <c r="A36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F36" s="40">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G36" s="41">
-        <f>IFERROR(IF(27&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(27,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(27-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A36" s="40" t="n"/>
+      <c r="B36" s="40" t="n"/>
+      <c r="C36" s="41" t="n"/>
+      <c r="D36" s="41" t="n"/>
+      <c r="E36" s="40" t="n"/>
+      <c r="F36" s="40" t="n"/>
+      <c r="G36" s="41" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
-      <c r="A37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F37" s="40">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G37" s="41">
-        <f>IFERROR(IF(28&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(28,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(28-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A37" s="40" t="n"/>
+      <c r="B37" s="40" t="n"/>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="40" t="n"/>
+      <c r="F37" s="40" t="n"/>
+      <c r="G37" s="41" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
-      <c r="A38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F38" s="40">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G38" s="41">
-        <f>IFERROR(IF(29&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(29,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(29-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A38" s="40" t="n"/>
+      <c r="B38" s="40" t="n"/>
+      <c r="C38" s="41" t="n"/>
+      <c r="D38" s="41" t="n"/>
+      <c r="E38" s="40" t="n"/>
+      <c r="F38" s="40" t="n"/>
+      <c r="G38" s="41" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
-      <c r="A39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F39" s="40">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G39" s="41">
-        <f>IFERROR(IF(30&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(30,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(30-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A39" s="40" t="n"/>
+      <c r="B39" s="40" t="n"/>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="40" t="n"/>
+      <c r="F39" s="40" t="n"/>
+      <c r="G39" s="41" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
-      <c r="A40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F40" s="40">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G40" s="41">
-        <f>IFERROR(IF(31&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(31,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(31-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A40" s="40" t="n"/>
+      <c r="B40" s="40" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="40" t="n"/>
+      <c r="F40" s="40" t="n"/>
+      <c r="G40" s="41" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
-      <c r="A41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F41" s="40">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G41" s="41">
-        <f>IFERROR(IF(32&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(32,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(32-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A41" s="40" t="n"/>
+      <c r="B41" s="40" t="n"/>
+      <c r="C41" s="41" t="n"/>
+      <c r="D41" s="41" t="n"/>
+      <c r="E41" s="40" t="n"/>
+      <c r="F41" s="40" t="n"/>
+      <c r="G41" s="41" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
-      <c r="A42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F42" s="40">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G42" s="41">
-        <f>IFERROR(IF(33&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(33,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(33-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A42" s="40" t="n"/>
+      <c r="B42" s="40" t="n"/>
+      <c r="C42" s="41" t="n"/>
+      <c r="D42" s="41" t="n"/>
+      <c r="E42" s="40" t="n"/>
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="41" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
-      <c r="A43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F43" s="40">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G43" s="41">
-        <f>IFERROR(IF(34&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(34,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(34-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A43" s="40" t="n"/>
+      <c r="B43" s="40" t="n"/>
+      <c r="C43" s="41" t="n"/>
+      <c r="D43" s="41" t="n"/>
+      <c r="E43" s="40" t="n"/>
+      <c r="F43" s="40" t="n"/>
+      <c r="G43" s="41" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
-      <c r="A44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F44" s="40">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G44" s="41">
-        <f>IFERROR(IF(35&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(35,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(35-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A44" s="40" t="n"/>
+      <c r="B44" s="40" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="40" t="n"/>
+      <c r="F44" s="40" t="n"/>
+      <c r="G44" s="41" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
-      <c r="A45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F45" s="40">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G45" s="41">
-        <f>IFERROR(IF(36&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(36,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(36-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A45" s="40" t="n"/>
+      <c r="B45" s="40" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="41" t="n"/>
+      <c r="E45" s="40" t="n"/>
+      <c r="F45" s="40" t="n"/>
+      <c r="G45" s="41" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
-      <c r="A46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F46" s="40">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G46" s="41">
-        <f>IFERROR(IF(37&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(37,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(37-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A46" s="40" t="n"/>
+      <c r="B46" s="40" t="n"/>
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="40" t="n"/>
+      <c r="F46" s="40" t="n"/>
+      <c r="G46" s="41" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
-      <c r="A47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F47" s="40">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G47" s="41">
-        <f>IFERROR(IF(38&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(38,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(38-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A47" s="40" t="n"/>
+      <c r="B47" s="40" t="n"/>
+      <c r="C47" s="41" t="n"/>
+      <c r="D47" s="41" t="n"/>
+      <c r="E47" s="40" t="n"/>
+      <c r="F47" s="40" t="n"/>
+      <c r="G47" s="41" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
-      <c r="A48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F48" s="40">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G48" s="41">
-        <f>IFERROR(IF(39&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(39,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(39-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A48" s="40" t="n"/>
+      <c r="B48" s="40" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="41" t="n"/>
+      <c r="E48" s="40" t="n"/>
+      <c r="F48" s="40" t="n"/>
+      <c r="G48" s="41" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
-      <c r="A49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F49" s="40">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G49" s="41">
-        <f>IFERROR(IF(40&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(40,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(40-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A49" s="40" t="n"/>
+      <c r="B49" s="40" t="n"/>
+      <c r="C49" s="41" t="n"/>
+      <c r="D49" s="41" t="n"/>
+      <c r="E49" s="40" t="n"/>
+      <c r="F49" s="40" t="n"/>
+      <c r="G49" s="41" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
-      <c r="A50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F50" s="40">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G50" s="41">
-        <f>IFERROR(IF(41&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(41,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(41-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A50" s="40" t="n"/>
+      <c r="B50" s="40" t="n"/>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="40" t="n"/>
+      <c r="F50" s="40" t="n"/>
+      <c r="G50" s="41" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
-      <c r="A51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F51" s="40">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G51" s="41">
-        <f>IFERROR(IF(42&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(42,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(42-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A51" s="40" t="n"/>
+      <c r="B51" s="40" t="n"/>
+      <c r="C51" s="41" t="n"/>
+      <c r="D51" s="41" t="n"/>
+      <c r="E51" s="40" t="n"/>
+      <c r="F51" s="40" t="n"/>
+      <c r="G51" s="41" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
-      <c r="A52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F52" s="40">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G52" s="41">
-        <f>IFERROR(IF(43&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(43,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(43-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A52" s="40" t="n"/>
+      <c r="B52" s="40" t="n"/>
+      <c r="C52" s="41" t="n"/>
+      <c r="D52" s="41" t="n"/>
+      <c r="E52" s="40" t="n"/>
+      <c r="F52" s="40" t="n"/>
+      <c r="G52" s="41" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
-      <c r="A53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F53" s="40">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G53" s="41">
-        <f>IFERROR(IF(44&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(44,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(44-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A53" s="40" t="n"/>
+      <c r="B53" s="40" t="n"/>
+      <c r="C53" s="41" t="n"/>
+      <c r="D53" s="41" t="n"/>
+      <c r="E53" s="40" t="n"/>
+      <c r="F53" s="40" t="n"/>
+      <c r="G53" s="41" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
-      <c r="A54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F54" s="40">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G54" s="41">
-        <f>IFERROR(IF(45&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(45,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(45-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A54" s="40" t="n"/>
+      <c r="B54" s="40" t="n"/>
+      <c r="C54" s="41" t="n"/>
+      <c r="D54" s="41" t="n"/>
+      <c r="E54" s="40" t="n"/>
+      <c r="F54" s="40" t="n"/>
+      <c r="G54" s="41" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
-      <c r="A55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F55" s="40">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G55" s="41">
-        <f>IFERROR(IF(46&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(46,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(46-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A55" s="40" t="n"/>
+      <c r="B55" s="40" t="n"/>
+      <c r="C55" s="41" t="n"/>
+      <c r="D55" s="41" t="n"/>
+      <c r="E55" s="40" t="n"/>
+      <c r="F55" s="40" t="n"/>
+      <c r="G55" s="41" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
-      <c r="A56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F56" s="40">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G56" s="41">
-        <f>IFERROR(IF(47&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(47,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(47-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A56" s="40" t="n"/>
+      <c r="B56" s="40" t="n"/>
+      <c r="C56" s="41" t="n"/>
+      <c r="D56" s="41" t="n"/>
+      <c r="E56" s="40" t="n"/>
+      <c r="F56" s="40" t="n"/>
+      <c r="G56" s="41" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
-      <c r="A57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F57" s="40">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G57" s="41">
-        <f>IFERROR(IF(48&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(48,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(48-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A57" s="40" t="n"/>
+      <c r="B57" s="40" t="n"/>
+      <c r="C57" s="41" t="n"/>
+      <c r="D57" s="41" t="n"/>
+      <c r="E57" s="40" t="n"/>
+      <c r="F57" s="40" t="n"/>
+      <c r="G57" s="41" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
-      <c r="A58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F58" s="40">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G58" s="41">
-        <f>IFERROR(IF(49&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(49,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(49-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A58" s="40" t="n"/>
+      <c r="B58" s="40" t="n"/>
+      <c r="C58" s="41" t="n"/>
+      <c r="D58" s="41" t="n"/>
+      <c r="E58" s="40" t="n"/>
+      <c r="F58" s="40" t="n"/>
+      <c r="G58" s="41" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
-      <c r="A59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F59" s="40">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G59" s="41">
-        <f>IFERROR(IF(50&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(50,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(50-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A59" s="40" t="n"/>
+      <c r="B59" s="40" t="n"/>
+      <c r="C59" s="41" t="n"/>
+      <c r="D59" s="41" t="n"/>
+      <c r="E59" s="40" t="n"/>
+      <c r="F59" s="40" t="n"/>
+      <c r="G59" s="41" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
-      <c r="A60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F60" s="40">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G60" s="41">
-        <f>IFERROR(IF(51&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(51,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(51-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A60" s="40" t="n"/>
+      <c r="B60" s="40" t="n"/>
+      <c r="C60" s="41" t="n"/>
+      <c r="D60" s="41" t="n"/>
+      <c r="E60" s="40" t="n"/>
+      <c r="F60" s="40" t="n"/>
+      <c r="G60" s="41" t="n"/>
     </row>
     <row r="61" ht="21.75" customHeight="1" s="25">
-      <c r="A61" s="42">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F61" s="39">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G61" s="43">
-        <f>IFERROR(IF(52&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(52,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(52-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A61" s="42" t="n"/>
+      <c r="B61" s="39" t="n"/>
+      <c r="C61" s="39" t="n"/>
+      <c r="D61" s="39" t="n"/>
+      <c r="E61" s="39" t="n"/>
+      <c r="F61" s="39" t="n"/>
+      <c r="G61" s="43" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
-      <c r="A62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F62" s="40">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G62" s="41">
-        <f>IFERROR(IF(53&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(53,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(53-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A62" s="40" t="n"/>
+      <c r="B62" s="40" t="n"/>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="41" t="n"/>
+      <c r="E62" s="40" t="n"/>
+      <c r="F62" s="40" t="n"/>
+      <c r="G62" s="41" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="25">
-      <c r="A63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F63" s="40">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G63" s="41">
-        <f>IFERROR(IF(54&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(54,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(54-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A63" s="40" t="n"/>
+      <c r="B63" s="40" t="n"/>
+      <c r="C63" s="41" t="n"/>
+      <c r="D63" s="41" t="n"/>
+      <c r="E63" s="40" t="n"/>
+      <c r="F63" s="40" t="n"/>
+      <c r="G63" s="41" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="25">
-      <c r="A64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F64" s="40">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G64" s="41">
-        <f>IFERROR(IF(55&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(55,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(55-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A64" s="40" t="n"/>
+      <c r="B64" s="40" t="n"/>
+      <c r="C64" s="41" t="n"/>
+      <c r="D64" s="41" t="n"/>
+      <c r="E64" s="40" t="n"/>
+      <c r="F64" s="40" t="n"/>
+      <c r="G64" s="41" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="25">
-      <c r="A65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F65" s="40">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G65" s="41">
-        <f>IFERROR(IF(56&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(56,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(56-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A65" s="40" t="n"/>
+      <c r="B65" s="40" t="n"/>
+      <c r="C65" s="41" t="n"/>
+      <c r="D65" s="41" t="n"/>
+      <c r="E65" s="40" t="n"/>
+      <c r="F65" s="40" t="n"/>
+      <c r="G65" s="41" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="25">
-      <c r="A66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F66" s="40">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G66" s="41">
-        <f>IFERROR(IF(57&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(57,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(57-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A66" s="40" t="n"/>
+      <c r="B66" s="40" t="n"/>
+      <c r="C66" s="41" t="n"/>
+      <c r="D66" s="41" t="n"/>
+      <c r="E66" s="40" t="n"/>
+      <c r="F66" s="40" t="n"/>
+      <c r="G66" s="41" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="25">
-      <c r="A67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F67" s="40">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G67" s="41">
-        <f>IFERROR(IF(58&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(58,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(58-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A67" s="40" t="n"/>
+      <c r="B67" s="40" t="n"/>
+      <c r="C67" s="41" t="n"/>
+      <c r="D67" s="41" t="n"/>
+      <c r="E67" s="40" t="n"/>
+      <c r="F67" s="40" t="n"/>
+      <c r="G67" s="41" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="25">
-      <c r="A68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F68" s="40">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G68" s="41">
-        <f>IFERROR(IF(59&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(59,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(59-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A68" s="40" t="n"/>
+      <c r="B68" s="40" t="n"/>
+      <c r="C68" s="41" t="n"/>
+      <c r="D68" s="41" t="n"/>
+      <c r="E68" s="40" t="n"/>
+      <c r="F68" s="40" t="n"/>
+      <c r="G68" s="41" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="25">
-      <c r="A69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F69" s="40">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G69" s="41">
-        <f>IFERROR(IF(60&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(60,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(60-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A69" s="40" t="n"/>
+      <c r="B69" s="40" t="n"/>
+      <c r="C69" s="41" t="n"/>
+      <c r="D69" s="41" t="n"/>
+      <c r="E69" s="40" t="n"/>
+      <c r="F69" s="40" t="n"/>
+      <c r="G69" s="41" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="25">
-      <c r="A70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F70" s="40">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G70" s="41">
-        <f>IFERROR(IF(61&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(61,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(61-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A70" s="40" t="n"/>
+      <c r="B70" s="40" t="n"/>
+      <c r="C70" s="41" t="n"/>
+      <c r="D70" s="41" t="n"/>
+      <c r="E70" s="40" t="n"/>
+      <c r="F70" s="40" t="n"/>
+      <c r="G70" s="41" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="25">
-      <c r="A71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F71" s="40">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G71" s="41">
-        <f>IFERROR(IF(62&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(62,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(62-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A71" s="40" t="n"/>
+      <c r="B71" s="40" t="n"/>
+      <c r="C71" s="41" t="n"/>
+      <c r="D71" s="41" t="n"/>
+      <c r="E71" s="40" t="n"/>
+      <c r="F71" s="40" t="n"/>
+      <c r="G71" s="41" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="25">
-      <c r="A72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F72" s="40">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G72" s="41">
-        <f>IFERROR(IF(63&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(63,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(63-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A72" s="40" t="n"/>
+      <c r="B72" s="40" t="n"/>
+      <c r="C72" s="41" t="n"/>
+      <c r="D72" s="41" t="n"/>
+      <c r="E72" s="40" t="n"/>
+      <c r="F72" s="40" t="n"/>
+      <c r="G72" s="41" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="25">
-      <c r="A73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F73" s="40">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G73" s="41">
-        <f>IFERROR(IF(64&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(64,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(64-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A73" s="40" t="n"/>
+      <c r="B73" s="40" t="n"/>
+      <c r="C73" s="41" t="n"/>
+      <c r="D73" s="41" t="n"/>
+      <c r="E73" s="40" t="n"/>
+      <c r="F73" s="40" t="n"/>
+      <c r="G73" s="41" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="25">
-      <c r="A74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F74" s="40">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G74" s="41">
-        <f>IFERROR(IF(65&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(65,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(65-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A74" s="40" t="n"/>
+      <c r="B74" s="40" t="n"/>
+      <c r="C74" s="41" t="n"/>
+      <c r="D74" s="41" t="n"/>
+      <c r="E74" s="40" t="n"/>
+      <c r="F74" s="40" t="n"/>
+      <c r="G74" s="41" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="25">
-      <c r="A75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F75" s="40">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G75" s="41">
-        <f>IFERROR(IF(66&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(66,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(66-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A75" s="40" t="n"/>
+      <c r="B75" s="40" t="n"/>
+      <c r="C75" s="41" t="n"/>
+      <c r="D75" s="41" t="n"/>
+      <c r="E75" s="40" t="n"/>
+      <c r="F75" s="40" t="n"/>
+      <c r="G75" s="41" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="25">
-      <c r="A76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F76" s="40">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G76" s="41">
-        <f>IFERROR(IF(67&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(67,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(67-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A76" s="40" t="n"/>
+      <c r="B76" s="40" t="n"/>
+      <c r="C76" s="41" t="n"/>
+      <c r="D76" s="41" t="n"/>
+      <c r="E76" s="40" t="n"/>
+      <c r="F76" s="40" t="n"/>
+      <c r="G76" s="41" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="25">
-      <c r="A77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F77" s="40">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G77" s="41">
-        <f>IFERROR(IF(68&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(68,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(68-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A77" s="40" t="n"/>
+      <c r="B77" s="40" t="n"/>
+      <c r="C77" s="41" t="n"/>
+      <c r="D77" s="41" t="n"/>
+      <c r="E77" s="40" t="n"/>
+      <c r="F77" s="40" t="n"/>
+      <c r="G77" s="41" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="25">
-      <c r="A78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F78" s="40">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G78" s="41">
-        <f>IFERROR(IF(69&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(69,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(69-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A78" s="40" t="n"/>
+      <c r="B78" s="40" t="n"/>
+      <c r="C78" s="41" t="n"/>
+      <c r="D78" s="41" t="n"/>
+      <c r="E78" s="40" t="n"/>
+      <c r="F78" s="40" t="n"/>
+      <c r="G78" s="41" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="25">
-      <c r="A79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F79" s="40">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G79" s="41">
-        <f>IFERROR(IF(70&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(70,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(70-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A79" s="40" t="n"/>
+      <c r="B79" s="40" t="n"/>
+      <c r="C79" s="41" t="n"/>
+      <c r="D79" s="41" t="n"/>
+      <c r="E79" s="40" t="n"/>
+      <c r="F79" s="40" t="n"/>
+      <c r="G79" s="41" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="25">
-      <c r="A80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F80" s="40">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G80" s="41">
-        <f>IFERROR(IF(71&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(71,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(71-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A80" s="40" t="n"/>
+      <c r="B80" s="40" t="n"/>
+      <c r="C80" s="41" t="n"/>
+      <c r="D80" s="41" t="n"/>
+      <c r="E80" s="40" t="n"/>
+      <c r="F80" s="40" t="n"/>
+      <c r="G80" s="41" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="25">
-      <c r="A81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F81" s="40">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G81" s="41">
-        <f>IFERROR(IF(72&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(72,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(72-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A81" s="40" t="n"/>
+      <c r="B81" s="40" t="n"/>
+      <c r="C81" s="41" t="n"/>
+      <c r="D81" s="41" t="n"/>
+      <c r="E81" s="40" t="n"/>
+      <c r="F81" s="40" t="n"/>
+      <c r="G81" s="41" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="25">
-      <c r="A82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F82" s="40">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G82" s="41">
-        <f>IFERROR(IF(73&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(73,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(73-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A82" s="40" t="n"/>
+      <c r="B82" s="40" t="n"/>
+      <c r="C82" s="41" t="n"/>
+      <c r="D82" s="41" t="n"/>
+      <c r="E82" s="40" t="n"/>
+      <c r="F82" s="40" t="n"/>
+      <c r="G82" s="41" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1" s="25">
-      <c r="A83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F83" s="40">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G83" s="41">
-        <f>IFERROR(IF(74&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(74,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(74-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A83" s="40" t="n"/>
+      <c r="B83" s="40" t="n"/>
+      <c r="C83" s="41" t="n"/>
+      <c r="D83" s="41" t="n"/>
+      <c r="E83" s="40" t="n"/>
+      <c r="F83" s="40" t="n"/>
+      <c r="G83" s="41" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="25">
-      <c r="A84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F84" s="40">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G84" s="41">
-        <f>IFERROR(IF(75&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(75,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(75-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A84" s="40" t="n"/>
+      <c r="B84" s="40" t="n"/>
+      <c r="C84" s="41" t="n"/>
+      <c r="D84" s="41" t="n"/>
+      <c r="E84" s="40" t="n"/>
+      <c r="F84" s="40" t="n"/>
+      <c r="G84" s="41" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="25">
-      <c r="A85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F85" s="40">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G85" s="41">
-        <f>IFERROR(IF(76&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(76,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(76-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A85" s="40" t="n"/>
+      <c r="B85" s="40" t="n"/>
+      <c r="C85" s="41" t="n"/>
+      <c r="D85" s="41" t="n"/>
+      <c r="E85" s="40" t="n"/>
+      <c r="F85" s="40" t="n"/>
+      <c r="G85" s="41" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="25">
-      <c r="A86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F86" s="40">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G86" s="41">
-        <f>IFERROR(IF(77&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(77,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(77-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A86" s="40" t="n"/>
+      <c r="B86" s="40" t="n"/>
+      <c r="C86" s="41" t="n"/>
+      <c r="D86" s="41" t="n"/>
+      <c r="E86" s="40" t="n"/>
+      <c r="F86" s="40" t="n"/>
+      <c r="G86" s="41" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="25">
-      <c r="A87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F87" s="40">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G87" s="41">
-        <f>IFERROR(IF(78&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(78,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(78-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A87" s="40" t="n"/>
+      <c r="B87" s="40" t="n"/>
+      <c r="C87" s="41" t="n"/>
+      <c r="D87" s="41" t="n"/>
+      <c r="E87" s="40" t="n"/>
+      <c r="F87" s="40" t="n"/>
+      <c r="G87" s="41" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="25">
-      <c r="A88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F88" s="40">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G88" s="41">
-        <f>IFERROR(IF(79&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(79,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(79-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A88" s="40" t="n"/>
+      <c r="B88" s="40" t="n"/>
+      <c r="C88" s="41" t="n"/>
+      <c r="D88" s="41" t="n"/>
+      <c r="E88" s="40" t="n"/>
+      <c r="F88" s="40" t="n"/>
+      <c r="G88" s="41" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="25">
-      <c r="A89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F89" s="40">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G89" s="41">
-        <f>IFERROR(IF(80&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(80,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(80-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A89" s="40" t="n"/>
+      <c r="B89" s="40" t="n"/>
+      <c r="C89" s="41" t="n"/>
+      <c r="D89" s="41" t="n"/>
+      <c r="E89" s="40" t="n"/>
+      <c r="F89" s="40" t="n"/>
+      <c r="G89" s="41" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="25">
-      <c r="A90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F90" s="40">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G90" s="41">
-        <f>IFERROR(IF(81&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(81,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(81-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A90" s="40" t="n"/>
+      <c r="B90" s="40" t="n"/>
+      <c r="C90" s="41" t="n"/>
+      <c r="D90" s="41" t="n"/>
+      <c r="E90" s="40" t="n"/>
+      <c r="F90" s="40" t="n"/>
+      <c r="G90" s="41" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" s="25">
-      <c r="A91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F91" s="40">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G91" s="41">
-        <f>IFERROR(IF(82&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(82,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(82-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A91" s="40" t="n"/>
+      <c r="B91" s="40" t="n"/>
+      <c r="C91" s="41" t="n"/>
+      <c r="D91" s="41" t="n"/>
+      <c r="E91" s="40" t="n"/>
+      <c r="F91" s="40" t="n"/>
+      <c r="G91" s="41" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="25">
-      <c r="A92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F92" s="40">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G92" s="41">
-        <f>IFERROR(IF(83&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(83,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(83-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A92" s="40" t="n"/>
+      <c r="B92" s="40" t="n"/>
+      <c r="C92" s="41" t="n"/>
+      <c r="D92" s="41" t="n"/>
+      <c r="E92" s="40" t="n"/>
+      <c r="F92" s="40" t="n"/>
+      <c r="G92" s="41" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="25">
-      <c r="A93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F93" s="40">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G93" s="41">
-        <f>IFERROR(IF(84&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(84,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(84-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A93" s="40" t="n"/>
+      <c r="B93" s="40" t="n"/>
+      <c r="C93" s="41" t="n"/>
+      <c r="D93" s="41" t="n"/>
+      <c r="E93" s="40" t="n"/>
+      <c r="F93" s="40" t="n"/>
+      <c r="G93" s="41" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="25">
-      <c r="A94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F94" s="40">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G94" s="41">
-        <f>IFERROR(IF(85&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(85,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(85-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A94" s="40" t="n"/>
+      <c r="B94" s="40" t="n"/>
+      <c r="C94" s="41" t="n"/>
+      <c r="D94" s="41" t="n"/>
+      <c r="E94" s="40" t="n"/>
+      <c r="F94" s="40" t="n"/>
+      <c r="G94" s="41" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="25">
-      <c r="A95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F95" s="40">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G95" s="41">
-        <f>IFERROR(IF(86&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(86,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(86-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A95" s="40" t="n"/>
+      <c r="B95" s="40" t="n"/>
+      <c r="C95" s="41" t="n"/>
+      <c r="D95" s="41" t="n"/>
+      <c r="E95" s="40" t="n"/>
+      <c r="F95" s="40" t="n"/>
+      <c r="G95" s="41" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="25">
-      <c r="A96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F96" s="40">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G96" s="41">
-        <f>IFERROR(IF(87&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(87,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(87-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A96" s="40" t="n"/>
+      <c r="B96" s="40" t="n"/>
+      <c r="C96" s="41" t="n"/>
+      <c r="D96" s="41" t="n"/>
+      <c r="E96" s="40" t="n"/>
+      <c r="F96" s="40" t="n"/>
+      <c r="G96" s="41" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="25">
-      <c r="A97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F97" s="40">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G97" s="41">
-        <f>IFERROR(IF(88&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(88,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(88-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A97" s="40" t="n"/>
+      <c r="B97" s="40" t="n"/>
+      <c r="C97" s="41" t="n"/>
+      <c r="D97" s="41" t="n"/>
+      <c r="E97" s="40" t="n"/>
+      <c r="F97" s="40" t="n"/>
+      <c r="G97" s="41" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="25">
-      <c r="A98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F98" s="40">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G98" s="41">
-        <f>IFERROR(IF(89&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(89,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(89-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A98" s="40" t="n"/>
+      <c r="B98" s="40" t="n"/>
+      <c r="C98" s="41" t="n"/>
+      <c r="D98" s="41" t="n"/>
+      <c r="E98" s="40" t="n"/>
+      <c r="F98" s="40" t="n"/>
+      <c r="G98" s="41" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="25">
-      <c r="A99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F99" s="40">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G99" s="41">
-        <f>IFERROR(IF(90&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(90,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(90-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A99" s="40" t="n"/>
+      <c r="B99" s="40" t="n"/>
+      <c r="C99" s="41" t="n"/>
+      <c r="D99" s="41" t="n"/>
+      <c r="E99" s="40" t="n"/>
+      <c r="F99" s="40" t="n"/>
+      <c r="G99" s="41" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="25">
-      <c r="A100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F100" s="40">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G100" s="41">
-        <f>IFERROR(IF(91&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(91,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(91-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A100" s="40" t="n"/>
+      <c r="B100" s="40" t="n"/>
+      <c r="C100" s="41" t="n"/>
+      <c r="D100" s="41" t="n"/>
+      <c r="E100" s="40" t="n"/>
+      <c r="F100" s="40" t="n"/>
+      <c r="G100" s="41" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="25">
-      <c r="A101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F101" s="40">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G101" s="41">
-        <f>IFERROR(IF(92&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(92,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(92-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A101" s="40" t="n"/>
+      <c r="B101" s="40" t="n"/>
+      <c r="C101" s="41" t="n"/>
+      <c r="D101" s="41" t="n"/>
+      <c r="E101" s="40" t="n"/>
+      <c r="F101" s="40" t="n"/>
+      <c r="G101" s="41" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="25">
-      <c r="A102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F102" s="40">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G102" s="41">
-        <f>IFERROR(IF(93&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(93,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(93-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A102" s="40" t="n"/>
+      <c r="B102" s="40" t="n"/>
+      <c r="C102" s="41" t="n"/>
+      <c r="D102" s="41" t="n"/>
+      <c r="E102" s="40" t="n"/>
+      <c r="F102" s="40" t="n"/>
+      <c r="G102" s="41" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="25">
-      <c r="A103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F103" s="40">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G103" s="41">
-        <f>IFERROR(IF(94&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(94,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(94-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A103" s="40" t="n"/>
+      <c r="B103" s="40" t="n"/>
+      <c r="C103" s="41" t="n"/>
+      <c r="D103" s="41" t="n"/>
+      <c r="E103" s="40" t="n"/>
+      <c r="F103" s="40" t="n"/>
+      <c r="G103" s="41" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="25">
-      <c r="A104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F104" s="40">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G104" s="41">
-        <f>IFERROR(IF(95&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(95,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(95-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A104" s="40" t="n"/>
+      <c r="B104" s="40" t="n"/>
+      <c r="C104" s="41" t="n"/>
+      <c r="D104" s="41" t="n"/>
+      <c r="E104" s="40" t="n"/>
+      <c r="F104" s="40" t="n"/>
+      <c r="G104" s="41" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="25">
-      <c r="A105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F105" s="40">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G105" s="41">
-        <f>IFERROR(IF(96&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(96,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(96-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A105" s="40" t="n"/>
+      <c r="B105" s="40" t="n"/>
+      <c r="C105" s="41" t="n"/>
+      <c r="D105" s="41" t="n"/>
+      <c r="E105" s="40" t="n"/>
+      <c r="F105" s="40" t="n"/>
+      <c r="G105" s="41" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="25">
-      <c r="A106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F106" s="40">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G106" s="41">
-        <f>IFERROR(IF(97&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(97,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(97-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A106" s="40" t="n"/>
+      <c r="B106" s="40" t="n"/>
+      <c r="C106" s="41" t="n"/>
+      <c r="D106" s="41" t="n"/>
+      <c r="E106" s="40" t="n"/>
+      <c r="F106" s="40" t="n"/>
+      <c r="G106" s="41" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="25">
-      <c r="A107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F107" s="40">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G107" s="41">
-        <f>IFERROR(IF(98&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(98,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(98-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A107" s="40" t="n"/>
+      <c r="B107" s="40" t="n"/>
+      <c r="C107" s="41" t="n"/>
+      <c r="D107" s="41" t="n"/>
+      <c r="E107" s="40" t="n"/>
+      <c r="F107" s="40" t="n"/>
+      <c r="G107" s="41" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="25">
-      <c r="A108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F108" s="40">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G108" s="41">
-        <f>IFERROR(IF(99&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(99,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(99-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A108" s="40" t="n"/>
+      <c r="B108" s="40" t="n"/>
+      <c r="C108" s="41" t="n"/>
+      <c r="D108" s="41" t="n"/>
+      <c r="E108" s="40" t="n"/>
+      <c r="F108" s="40" t="n"/>
+      <c r="G108" s="41" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1" s="25">
-      <c r="A109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="B109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),IF(INDEX('New Tooling Jobs'!A$13:A$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0))&lt;&gt;"","New Tooling",""),IF(INDEX(Reorders!A$13:A$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))&lt;&gt;"","Reorder","")),"")</f>
-        <v/>
-      </c>
-      <c r="C109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="D109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="F109" s="40">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
-      <c r="G109" s="41">
-        <f>IFERROR(IF(100&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(100,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(100-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v/>
-      </c>
+      <c r="A109" s="40" t="n"/>
+      <c r="B109" s="40" t="n"/>
+      <c r="C109" s="41" t="n"/>
+      <c r="D109" s="41" t="n"/>
+      <c r="E109" s="40" t="n"/>
+      <c r="F109" s="40" t="n"/>
+      <c r="G109" s="41" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1" s="25">
       <c r="A110" s="40" t="n"/>
@@ -4336,7 +2362,7 @@
           <t>Molder Invoice Status</t>
         </is>
       </c>
-      <c r="AG12" t="inlineStr">
+      <c r="AG12" s="24" t="inlineStr">
         <is>
           <t>_Seq</t>
         </is>
@@ -4410,7 +2436,7 @@
         <f>IF(W13="","",W13-TODAY())</f>
         <v/>
       </c>
-      <c r="AG13">
+      <c r="AG13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4499,7 +2525,7 @@
         <f>IF(W14="","",W14-TODAY())</f>
         <v/>
       </c>
-      <c r="AG14">
+      <c r="AG14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4598,7 +2624,7 @@
         <f>IF(W15="","",W15-TODAY())</f>
         <v/>
       </c>
-      <c r="AG15">
+      <c r="AG15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4665,7 +2691,7 @@
         <f>IF(W16="","",W16-TODAY())</f>
         <v/>
       </c>
-      <c r="AG16">
+      <c r="AG16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4704,7 +2730,7 @@
         <f>IF(W17="","",W17-TODAY())</f>
         <v/>
       </c>
-      <c r="AG17">
+      <c r="AG17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4743,7 +2769,7 @@
         <f>IF(W18="","",W18-TODAY())</f>
         <v/>
       </c>
-      <c r="AG18">
+      <c r="AG18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4782,7 +2808,7 @@
         <f>IF(W19="","",W19-TODAY())</f>
         <v/>
       </c>
-      <c r="AG19">
+      <c r="AG19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4821,7 +2847,7 @@
         <f>IF(W20="","",W20-TODAY())</f>
         <v/>
       </c>
-      <c r="AG20">
+      <c r="AG20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4860,7 +2886,7 @@
         <f>IF(W21="","",W21-TODAY())</f>
         <v/>
       </c>
-      <c r="AG21">
+      <c r="AG21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4899,7 +2925,7 @@
         <f>IF(W22="","",W22-TODAY())</f>
         <v/>
       </c>
-      <c r="AG22">
+      <c r="AG22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4938,7 +2964,7 @@
         <f>IF(W23="","",W23-TODAY())</f>
         <v/>
       </c>
-      <c r="AG23">
+      <c r="AG23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -4977,7 +3003,7 @@
         <f>IF(W24="","",W24-TODAY())</f>
         <v/>
       </c>
-      <c r="AG24">
+      <c r="AG24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5016,7 +3042,7 @@
         <f>IF(W25="","",W25-TODAY())</f>
         <v/>
       </c>
-      <c r="AG25">
+      <c r="AG25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5055,7 +3081,7 @@
         <f>IF(W26="","",W26-TODAY())</f>
         <v/>
       </c>
-      <c r="AG26">
+      <c r="AG26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5094,7 +3120,7 @@
         <f>IF(W27="","",W27-TODAY())</f>
         <v/>
       </c>
-      <c r="AG27">
+      <c r="AG27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5133,7 +3159,7 @@
         <f>IF(W28="","",W28-TODAY())</f>
         <v/>
       </c>
-      <c r="AG28">
+      <c r="AG28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5172,7 +3198,7 @@
         <f>IF(W29="","",W29-TODAY())</f>
         <v/>
       </c>
-      <c r="AG29">
+      <c r="AG29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5211,7 +3237,7 @@
         <f>IF(W30="","",W30-TODAY())</f>
         <v/>
       </c>
-      <c r="AG30">
+      <c r="AG30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5250,7 +3276,7 @@
         <f>IF(W31="","",W31-TODAY())</f>
         <v/>
       </c>
-      <c r="AG31">
+      <c r="AG31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5289,7 +3315,7 @@
         <f>IF(W32="","",W32-TODAY())</f>
         <v/>
       </c>
-      <c r="AG32">
+      <c r="AG32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5328,7 +3354,7 @@
         <f>IF(W33="","",W33-TODAY())</f>
         <v/>
       </c>
-      <c r="AG33">
+      <c r="AG33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5367,7 +3393,7 @@
         <f>IF(W34="","",W34-TODAY())</f>
         <v/>
       </c>
-      <c r="AG34">
+      <c r="AG34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5406,7 +3432,7 @@
         <f>IF(W35="","",W35-TODAY())</f>
         <v/>
       </c>
-      <c r="AG35">
+      <c r="AG35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5445,7 +3471,7 @@
         <f>IF(W36="","",W36-TODAY())</f>
         <v/>
       </c>
-      <c r="AG36">
+      <c r="AG36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5484,7 +3510,7 @@
         <f>IF(W37="","",W37-TODAY())</f>
         <v/>
       </c>
-      <c r="AG37">
+      <c r="AG37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5523,7 +3549,7 @@
         <f>IF(W38="","",W38-TODAY())</f>
         <v/>
       </c>
-      <c r="AG38">
+      <c r="AG38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5562,7 +3588,7 @@
         <f>IF(W39="","",W39-TODAY())</f>
         <v/>
       </c>
-      <c r="AG39">
+      <c r="AG39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5601,7 +3627,7 @@
         <f>IF(W40="","",W40-TODAY())</f>
         <v/>
       </c>
-      <c r="AG40">
+      <c r="AG40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5640,7 +3666,7 @@
         <f>IF(W41="","",W41-TODAY())</f>
         <v/>
       </c>
-      <c r="AG41">
+      <c r="AG41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5679,7 +3705,7 @@
         <f>IF(W42="","",W42-TODAY())</f>
         <v/>
       </c>
-      <c r="AG42">
+      <c r="AG42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5718,7 +3744,7 @@
         <f>IF(W43="","",W43-TODAY())</f>
         <v/>
       </c>
-      <c r="AG43">
+      <c r="AG43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5757,7 +3783,7 @@
         <f>IF(W44="","",W44-TODAY())</f>
         <v/>
       </c>
-      <c r="AG44">
+      <c r="AG44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5796,7 +3822,7 @@
         <f>IF(W45="","",W45-TODAY())</f>
         <v/>
       </c>
-      <c r="AG45">
+      <c r="AG45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5835,7 +3861,7 @@
         <f>IF(W46="","",W46-TODAY())</f>
         <v/>
       </c>
-      <c r="AG46">
+      <c r="AG46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5874,7 +3900,7 @@
         <f>IF(W47="","",W47-TODAY())</f>
         <v/>
       </c>
-      <c r="AG47">
+      <c r="AG47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5913,7 +3939,7 @@
         <f>IF(W48="","",W48-TODAY())</f>
         <v/>
       </c>
-      <c r="AG48">
+      <c r="AG48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5952,7 +3978,7 @@
         <f>IF(W49="","",W49-TODAY())</f>
         <v/>
       </c>
-      <c r="AG49">
+      <c r="AG49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -5991,7 +4017,7 @@
         <f>IF(W50="","",W50-TODAY())</f>
         <v/>
       </c>
-      <c r="AG50">
+      <c r="AG50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6030,7 +4056,7 @@
         <f>IF(W51="","",W51-TODAY())</f>
         <v/>
       </c>
-      <c r="AG51">
+      <c r="AG51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6069,7 +4095,7 @@
         <f>IF(W52="","",W52-TODAY())</f>
         <v/>
       </c>
-      <c r="AG52">
+      <c r="AG52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6108,7 +4134,7 @@
         <f>IF(W53="","",W53-TODAY())</f>
         <v/>
       </c>
-      <c r="AG53">
+      <c r="AG53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6147,7 +4173,7 @@
         <f>IF(W54="","",W54-TODAY())</f>
         <v/>
       </c>
-      <c r="AG54">
+      <c r="AG54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6186,7 +4212,7 @@
         <f>IF(W55="","",W55-TODAY())</f>
         <v/>
       </c>
-      <c r="AG55">
+      <c r="AG55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6225,7 +4251,7 @@
         <f>IF(W56="","",W56-TODAY())</f>
         <v/>
       </c>
-      <c r="AG56">
+      <c r="AG56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6264,7 +4290,7 @@
         <f>IF(W57="","",W57-TODAY())</f>
         <v/>
       </c>
-      <c r="AG57">
+      <c r="AG57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6303,7 +4329,7 @@
         <f>IF(W58="","",W58-TODAY())</f>
         <v/>
       </c>
-      <c r="AG58">
+      <c r="AG58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6342,7 +4368,7 @@
         <f>IF(W59="","",W59-TODAY())</f>
         <v/>
       </c>
-      <c r="AG59">
+      <c r="AG59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6381,7 +4407,7 @@
         <f>IF(W60="","",W60-TODAY())</f>
         <v/>
       </c>
-      <c r="AG60">
+      <c r="AG60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6420,7 +4446,7 @@
         <f>IF(W61="","",W61-TODAY())</f>
         <v/>
       </c>
-      <c r="AG61">
+      <c r="AG61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6459,7 +4485,7 @@
         <f>IF(W62="","",W62-TODAY())</f>
         <v/>
       </c>
-      <c r="AG62">
+      <c r="AG62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6721,7 +4747,7 @@
           <t>Molder Invoice Status</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC12" s="24" t="inlineStr">
         <is>
           <t>_Seq</t>
         </is>
@@ -6809,7 +4835,7 @@
         <f>IF(S13="","",S13-TODAY())</f>
         <v/>
       </c>
-      <c r="AC13">
+      <c r="AC13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6890,7 +4916,7 @@
         <f>IF(S14="","",S14-TODAY())</f>
         <v/>
       </c>
-      <c r="AC14">
+      <c r="AC14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -6977,7 +5003,7 @@
         <f>IF(S15="","",S15-TODAY())</f>
         <v/>
       </c>
-      <c r="AC15">
+      <c r="AC15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7012,7 +5038,7 @@
         <f>IF(S16="","",S16-TODAY())</f>
         <v/>
       </c>
-      <c r="AC16">
+      <c r="AC16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7047,7 +5073,7 @@
         <f>IF(S17="","",S17-TODAY())</f>
         <v/>
       </c>
-      <c r="AC17">
+      <c r="AC17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7082,7 +5108,7 @@
         <f>IF(S18="","",S18-TODAY())</f>
         <v/>
       </c>
-      <c r="AC18">
+      <c r="AC18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7117,7 +5143,7 @@
         <f>IF(S19="","",S19-TODAY())</f>
         <v/>
       </c>
-      <c r="AC19">
+      <c r="AC19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7152,7 +5178,7 @@
         <f>IF(S20="","",S20-TODAY())</f>
         <v/>
       </c>
-      <c r="AC20">
+      <c r="AC20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7187,7 +5213,7 @@
         <f>IF(S21="","",S21-TODAY())</f>
         <v/>
       </c>
-      <c r="AC21">
+      <c r="AC21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7222,7 +5248,7 @@
         <f>IF(S22="","",S22-TODAY())</f>
         <v/>
       </c>
-      <c r="AC22">
+      <c r="AC22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7257,7 +5283,7 @@
         <f>IF(S23="","",S23-TODAY())</f>
         <v/>
       </c>
-      <c r="AC23">
+      <c r="AC23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7292,7 +5318,7 @@
         <f>IF(S24="","",S24-TODAY())</f>
         <v/>
       </c>
-      <c r="AC24">
+      <c r="AC24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7327,7 +5353,7 @@
         <f>IF(S25="","",S25-TODAY())</f>
         <v/>
       </c>
-      <c r="AC25">
+      <c r="AC25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7362,7 +5388,7 @@
         <f>IF(S26="","",S26-TODAY())</f>
         <v/>
       </c>
-      <c r="AC26">
+      <c r="AC26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7397,7 +5423,7 @@
         <f>IF(S27="","",S27-TODAY())</f>
         <v/>
       </c>
-      <c r="AC27">
+      <c r="AC27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7432,7 +5458,7 @@
         <f>IF(S28="","",S28-TODAY())</f>
         <v/>
       </c>
-      <c r="AC28">
+      <c r="AC28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7467,7 +5493,7 @@
         <f>IF(S29="","",S29-TODAY())</f>
         <v/>
       </c>
-      <c r="AC29">
+      <c r="AC29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7502,7 +5528,7 @@
         <f>IF(S30="","",S30-TODAY())</f>
         <v/>
       </c>
-      <c r="AC30">
+      <c r="AC30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7537,7 +5563,7 @@
         <f>IF(S31="","",S31-TODAY())</f>
         <v/>
       </c>
-      <c r="AC31">
+      <c r="AC31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7572,7 +5598,7 @@
         <f>IF(S32="","",S32-TODAY())</f>
         <v/>
       </c>
-      <c r="AC32">
+      <c r="AC32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7607,7 +5633,7 @@
         <f>IF(S33="","",S33-TODAY())</f>
         <v/>
       </c>
-      <c r="AC33">
+      <c r="AC33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7642,7 +5668,7 @@
         <f>IF(S34="","",S34-TODAY())</f>
         <v/>
       </c>
-      <c r="AC34">
+      <c r="AC34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7677,7 +5703,7 @@
         <f>IF(S35="","",S35-TODAY())</f>
         <v/>
       </c>
-      <c r="AC35">
+      <c r="AC35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7712,7 +5738,7 @@
         <f>IF(S36="","",S36-TODAY())</f>
         <v/>
       </c>
-      <c r="AC36">
+      <c r="AC36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7747,7 +5773,7 @@
         <f>IF(S37="","",S37-TODAY())</f>
         <v/>
       </c>
-      <c r="AC37">
+      <c r="AC37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7782,7 +5808,7 @@
         <f>IF(S38="","",S38-TODAY())</f>
         <v/>
       </c>
-      <c r="AC38">
+      <c r="AC38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7817,7 +5843,7 @@
         <f>IF(S39="","",S39-TODAY())</f>
         <v/>
       </c>
-      <c r="AC39">
+      <c r="AC39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7852,7 +5878,7 @@
         <f>IF(S40="","",S40-TODAY())</f>
         <v/>
       </c>
-      <c r="AC40">
+      <c r="AC40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7887,7 +5913,7 @@
         <f>IF(S41="","",S41-TODAY())</f>
         <v/>
       </c>
-      <c r="AC41">
+      <c r="AC41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7922,7 +5948,7 @@
         <f>IF(S42="","",S42-TODAY())</f>
         <v/>
       </c>
-      <c r="AC42">
+      <c r="AC42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7957,7 +5983,7 @@
         <f>IF(S43="","",S43-TODAY())</f>
         <v/>
       </c>
-      <c r="AC43">
+      <c r="AC43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -7992,7 +6018,7 @@
         <f>IF(S44="","",S44-TODAY())</f>
         <v/>
       </c>
-      <c r="AC44">
+      <c r="AC44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8027,7 +6053,7 @@
         <f>IF(S45="","",S45-TODAY())</f>
         <v/>
       </c>
-      <c r="AC45">
+      <c r="AC45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8062,7 +6088,7 @@
         <f>IF(S46="","",S46-TODAY())</f>
         <v/>
       </c>
-      <c r="AC46">
+      <c r="AC46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8097,7 +6123,7 @@
         <f>IF(S47="","",S47-TODAY())</f>
         <v/>
       </c>
-      <c r="AC47">
+      <c r="AC47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8132,7 +6158,7 @@
         <f>IF(S48="","",S48-TODAY())</f>
         <v/>
       </c>
-      <c r="AC48">
+      <c r="AC48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8167,7 +6193,7 @@
         <f>IF(S49="","",S49-TODAY())</f>
         <v/>
       </c>
-      <c r="AC49">
+      <c r="AC49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8202,7 +6228,7 @@
         <f>IF(S50="","",S50-TODAY())</f>
         <v/>
       </c>
-      <c r="AC50">
+      <c r="AC50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8237,7 +6263,7 @@
         <f>IF(S51="","",S51-TODAY())</f>
         <v/>
       </c>
-      <c r="AC51">
+      <c r="AC51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8272,7 +6298,7 @@
         <f>IF(S52="","",S52-TODAY())</f>
         <v/>
       </c>
-      <c r="AC52">
+      <c r="AC52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8307,7 +6333,7 @@
         <f>IF(S53="","",S53-TODAY())</f>
         <v/>
       </c>
-      <c r="AC53">
+      <c r="AC53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8342,7 +6368,7 @@
         <f>IF(S54="","",S54-TODAY())</f>
         <v/>
       </c>
-      <c r="AC54">
+      <c r="AC54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8377,7 +6403,7 @@
         <f>IF(S55="","",S55-TODAY())</f>
         <v/>
       </c>
-      <c r="AC55">
+      <c r="AC55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8412,7 +6438,7 @@
         <f>IF(S56="","",S56-TODAY())</f>
         <v/>
       </c>
-      <c r="AC56">
+      <c r="AC56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8447,7 +6473,7 @@
         <f>IF(S57="","",S57-TODAY())</f>
         <v/>
       </c>
-      <c r="AC57">
+      <c r="AC57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8482,7 +6508,7 @@
         <f>IF(S58="","",S58-TODAY())</f>
         <v/>
       </c>
-      <c r="AC58">
+      <c r="AC58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8517,7 +6543,7 @@
         <f>IF(S59="","",S59-TODAY())</f>
         <v/>
       </c>
-      <c r="AC59">
+      <c r="AC59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8552,7 +6578,7 @@
         <f>IF(S60="","",S60-TODAY())</f>
         <v/>
       </c>
-      <c r="AC60">
+      <c r="AC60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8587,7 +6613,7 @@
         <f>IF(S61="","",S61-TODAY())</f>
         <v/>
       </c>
-      <c r="AC61">
+      <c r="AC61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
@@ -8622,7 +6648,7 @@
         <f>IF(S62="","",S62-TODAY())</f>
         <v/>
       </c>
-      <c r="AC62">
+      <c r="AC62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Apply all dashboard fixes to main: direct IF formulas with cached values, invoice columns
Brings main up to date with all fixes from the feature branch:
- Dashboard populated via simple direct IF formulas with pre-cached XML values
- Invoice tracking columns added to New Tooling Jobs (Y-AF) and Reorders (U-AB)
- No dynamic array functions or array formulas that caused XML recovery errors

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -1047,60 +1047,183 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>_xlfn.LET(ntArr,CHOOSE({1,2,3,4,5,6,7},'New Tooling Jobs'!A13:A62,IF('New Tooling Jobs'!A13:A62&lt;&gt;"","New Tooling",""),'New Tooling Jobs'!B13:B62,'New Tooling Jobs'!E13:E62,'New Tooling Jobs'!G13:G62,'New Tooling Jobs'!H13:H62,'New Tooling Jobs'!I13:I62),reArr,CHOOSE({1,2,3,4,5,6,7},Reorders!A13:A62,IF(Reorders!A13:A62&lt;&gt;"","Reorder",""),Reorders!B13:B62,Reorders!E13:E62,Reorders!G13:G62,Reorders!H13:H62,Reorders!I13:I62),ntFilt,IFERROR(_xlfn.FILTER(ntArr,('New Tooling Jobs'!A13:A62&lt;&gt;"")*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),reFilt,IFERROR(_xlfn.FILTER(reArr,(Reorders!A13:A62&lt;&gt;"")*(Reorders!E13:E62&lt;&gt;"Completed")),{"","","","","","",""}),combined,_xlfn.VSTACK(ntFilt,reFilt),active,IFERROR(_xlfn.FILTER(combined,INDEX(combined,,1)&lt;&gt;""),{"No active jobs","","","","","",""}),_xlfn.SORT(active,1,1))</f>
-        <v/>
-      </c>
-      <c r="B10" s="39" t="n"/>
-      <c r="C10" s="39" t="n"/>
-      <c r="D10" s="39" t="n"/>
-      <c r="E10" s="39" t="n"/>
-      <c r="F10" s="39" t="n"/>
-      <c r="G10" s="39" t="n"/>
+        <f>IF('New Tooling Jobs'!A13="","",'New Tooling Jobs'!A13)</f>
+        <v>JOB-2026-101</v>
+      </c>
+      <c r="B10" s="39">
+        <f>IF('New Tooling Jobs'!A13="","","New Tooling")</f>
+        <v>New Tooling</v>
+      </c>
+      <c r="C10" s="39">
+        <f>IF('New Tooling Jobs'!B13="","",'New Tooling Jobs'!B13)</f>
+        <v>Acme Industries</v>
+      </c>
+      <c r="D10" s="39">
+        <f>IF('New Tooling Jobs'!E13="","",'New Tooling Jobs'!E13)</f>
+        <v>2. Quote Sent to Customer</v>
+      </c>
+      <c r="E10" s="39">
+        <f>IF('New Tooling Jobs'!G13="","",'New Tooling Jobs'!G13)</f>
+        <v/>
+      </c>
+      <c r="F10" s="39">
+        <f>IF('New Tooling Jobs'!H13="","",'New Tooling Jobs'!H13)</f>
+        <v/>
+      </c>
+      <c r="G10" s="39">
+        <f>IF('New Tooling Jobs'!I13="","",'New Tooling Jobs'!I13)</f>
+        <v>Awaiting customer PO</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="40" t="n"/>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="41" t="n"/>
-      <c r="D11" s="41" t="n"/>
-      <c r="E11" s="40" t="n"/>
-      <c r="F11" s="40" t="n"/>
-      <c r="G11" s="41" t="n"/>
+      <c r="A11" s="40">
+        <f>IF('New Tooling Jobs'!A14="","",'New Tooling Jobs'!A14)</f>
+        <v>JOB-2026-102</v>
+      </c>
+      <c r="B11" s="40">
+        <f>IF('New Tooling Jobs'!A14="","","New Tooling")</f>
+        <v>New Tooling</v>
+      </c>
+      <c r="C11" s="41">
+        <f>IF('New Tooling Jobs'!B14="","",'New Tooling Jobs'!B14)</f>
+        <v>Beacon Electronics</v>
+      </c>
+      <c r="D11" s="41">
+        <f>IF('New Tooling Jobs'!E14="","",'New Tooling Jobs'!E14)</f>
+        <v>4. PO Issued to Molder</v>
+      </c>
+      <c r="E11" s="40">
+        <f>IF('New Tooling Jobs'!G14="","",'New Tooling Jobs'!G14)</f>
+        <v>PO-BE-3411</v>
+      </c>
+      <c r="F11" s="40">
+        <f>IF('New Tooling Jobs'!H14="","",'New Tooling Jobs'!H14)</f>
+        <v>PO-SUM-0992</v>
+      </c>
+      <c r="G11" s="41">
+        <f>IF('New Tooling Jobs'!I14="","",'New Tooling Jobs'!I14)</f>
+        <v>Mold kickoff meeting 5/4</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="40" t="n"/>
-      <c r="B12" s="40" t="n"/>
-      <c r="C12" s="41" t="n"/>
-      <c r="D12" s="41" t="n"/>
-      <c r="E12" s="40" t="n"/>
-      <c r="F12" s="40" t="n"/>
-      <c r="G12" s="41" t="n"/>
+      <c r="A12" s="40">
+        <f>IF('New Tooling Jobs'!A15="","",'New Tooling Jobs'!A15)</f>
+        <v>JOB-2026-103</v>
+      </c>
+      <c r="B12" s="40">
+        <f>IF('New Tooling Jobs'!A15="","","New Tooling")</f>
+        <v>New Tooling</v>
+      </c>
+      <c r="C12" s="41">
+        <f>IF('New Tooling Jobs'!B15="","",'New Tooling Jobs'!B15)</f>
+        <v>Drift Medical</v>
+      </c>
+      <c r="D12" s="41">
+        <f>IF('New Tooling Jobs'!E15="","",'New Tooling Jobs'!E15)</f>
+        <v>6. Sample / FAI Approval</v>
+      </c>
+      <c r="E12" s="40">
+        <f>IF('New Tooling Jobs'!G15="","",'New Tooling Jobs'!G15)</f>
+        <v>PO-DM-2210</v>
+      </c>
+      <c r="F12" s="40">
+        <f>IF('New Tooling Jobs'!H15="","",'New Tooling Jobs'!H15)</f>
+        <v>PO-PP-1145</v>
+      </c>
+      <c r="G12" s="41">
+        <f>IF('New Tooling Jobs'!I15="","",'New Tooling Jobs'!I15)</f>
+        <v>Awaiting customer FAI sign-off</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="40" t="n"/>
-      <c r="B13" s="40" t="n"/>
-      <c r="C13" s="41" t="n"/>
-      <c r="D13" s="41" t="n"/>
-      <c r="E13" s="40" t="n"/>
-      <c r="F13" s="40" t="n"/>
-      <c r="G13" s="41" t="n"/>
+      <c r="A13" s="40">
+        <f>IF('New Tooling Jobs'!A16="","",'New Tooling Jobs'!A16)</f>
+        <v>JOB-2026-105</v>
+      </c>
+      <c r="B13" s="40">
+        <f>IF('New Tooling Jobs'!A16="","","New Tooling")</f>
+        <v>New Tooling</v>
+      </c>
+      <c r="C13" s="41">
+        <f>IF('New Tooling Jobs'!B16="","",'New Tooling Jobs'!B16)</f>
+        <v>Acme Industries</v>
+      </c>
+      <c r="D13" s="41">
+        <f>IF('New Tooling Jobs'!E16="","",'New Tooling Jobs'!E16)</f>
+        <v>1. Quote Requested</v>
+      </c>
+      <c r="E13" s="40">
+        <f>IF('New Tooling Jobs'!G16="","",'New Tooling Jobs'!G16)</f>
+        <v/>
+      </c>
+      <c r="F13" s="40">
+        <f>IF('New Tooling Jobs'!H16="","",'New Tooling Jobs'!H16)</f>
+        <v/>
+      </c>
+      <c r="G13" s="41">
+        <f>IF('New Tooling Jobs'!I16="","",'New Tooling Jobs'!I16)</f>
+        <v>Waiting on molder quote (requested 4/22)</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="40" t="n"/>
-      <c r="B14" s="40" t="n"/>
-      <c r="C14" s="41" t="n"/>
-      <c r="D14" s="41" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="40" t="n"/>
-      <c r="G14" s="41" t="n"/>
+      <c r="A14" s="40">
+        <f>IF(Reorders!A13="","",Reorders!A13)</f>
+        <v>JOB-2026-104</v>
+      </c>
+      <c r="B14" s="40">
+        <f>IF(Reorders!A13="","","Reorder")</f>
+        <v>Reorder</v>
+      </c>
+      <c r="C14" s="41">
+        <f>IF(Reorders!B13="","",Reorders!B13)</f>
+        <v>Cedar Outdoor Co.</v>
+      </c>
+      <c r="D14" s="41">
+        <f>IF(Reorders!E13="","",Reorders!E13)</f>
+        <v>3. Production &amp; Shipping</v>
+      </c>
+      <c r="E14" s="40">
+        <f>IF(Reorders!G13="","",Reorders!G13)</f>
+        <v>PO-CD-1207</v>
+      </c>
+      <c r="F14" s="40">
+        <f>IF(Reorders!H13="","",Reorders!H13)</f>
+        <v>PO-PAC-0451</v>
+      </c>
+      <c r="G14" s="41">
+        <f>IF(Reorders!I13="","",Reorders!I13)</f>
+        <v>Production scheduled wk of 5/4</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="40" t="n"/>
-      <c r="C15" s="41" t="n"/>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="40" t="n"/>
-      <c r="F15" s="40" t="n"/>
-      <c r="G15" s="41" t="n"/>
+      <c r="A15" s="40">
+        <f>IF(Reorders!A14="","",Reorders!A14)</f>
+        <v>JOB-2026-106</v>
+      </c>
+      <c r="B15" s="40">
+        <f>IF(Reorders!A14="","","Reorder")</f>
+        <v>Reorder</v>
+      </c>
+      <c r="C15" s="41">
+        <f>IF(Reorders!B14="","",Reorders!B14)</f>
+        <v>Beacon Electronics</v>
+      </c>
+      <c r="D15" s="41">
+        <f>IF(Reorders!E14="","",Reorders!E14)</f>
+        <v>1. Customer PO Received</v>
+      </c>
+      <c r="E15" s="40">
+        <f>IF(Reorders!G14="","",Reorders!G14)</f>
+        <v>PO-BE-3415</v>
+      </c>
+      <c r="F15" s="40">
+        <f>IF(Reorders!H14="","",Reorders!H14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="41">
+        <f>IF(Reorders!I14="","",Reorders!I14)</f>
+        <v>Cut molder PO this week</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="40" t="n"/>
@@ -1966,6 +2089,15 @@
       <c r="F111" s="40" t="n"/>
       <c r="G111" s="41" t="n"/>
     </row>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
   </sheetData>
   <autoFilter ref="A9:G111"/>
   <mergeCells count="11">
@@ -2037,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AF62"/>
+  <dimension ref="A1:AG62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -2190,44 +2322,49 @@
           <t>Days Until Deadline</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice #</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Date</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Sent Date</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Status</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice #</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AD12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Date</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
+      <c r="AE12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Amount ($)</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr">
+      <c r="AF12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Status</t>
+        </is>
+      </c>
+      <c r="AG12" s="24" t="inlineStr">
+        <is>
+          <t>_Seq</t>
         </is>
       </c>
     </row>
@@ -2299,6 +2436,10 @@
         <f>IF(W13="","",W13-TODAY())</f>
         <v/>
       </c>
+      <c r="AG13" s="24">
+        <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40" t="inlineStr">
@@ -2384,6 +2525,10 @@
         <f>IF(W14="","",W14-TODAY())</f>
         <v/>
       </c>
+      <c r="AG14" s="24">
+        <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40" t="inlineStr">
@@ -2477,6 +2622,10 @@
       </c>
       <c r="X15" s="46">
         <f>IF(W15="","",W15-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG15" s="24">
+        <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -2540,6 +2689,10 @@
       </c>
       <c r="X16" s="46">
         <f>IF(W16="","",W16-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG16" s="24">
+        <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -2577,6 +2730,10 @@
         <f>IF(W17="","",W17-TODAY())</f>
         <v/>
       </c>
+      <c r="AG17" s="24">
+        <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="40" t="n"/>
@@ -2612,6 +2769,10 @@
         <f>IF(W18="","",W18-TODAY())</f>
         <v/>
       </c>
+      <c r="AG18" s="24">
+        <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
       <c r="A19" s="40" t="n"/>
@@ -2647,6 +2808,10 @@
         <f>IF(W19="","",W19-TODAY())</f>
         <v/>
       </c>
+      <c r="AG19" s="24">
+        <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="40" t="n"/>
@@ -2682,6 +2847,10 @@
         <f>IF(W20="","",W20-TODAY())</f>
         <v/>
       </c>
+      <c r="AG20" s="24">
+        <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
       <c r="A21" s="40" t="n"/>
@@ -2717,6 +2886,10 @@
         <f>IF(W21="","",W21-TODAY())</f>
         <v/>
       </c>
+      <c r="AG21" s="24">
+        <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
       <c r="A22" s="40" t="n"/>
@@ -2752,6 +2925,10 @@
         <f>IF(W22="","",W22-TODAY())</f>
         <v/>
       </c>
+      <c r="AG22" s="24">
+        <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="40" t="n"/>
@@ -2787,6 +2964,10 @@
         <f>IF(W23="","",W23-TODAY())</f>
         <v/>
       </c>
+      <c r="AG23" s="24">
+        <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="40" t="n"/>
@@ -2822,6 +3003,10 @@
         <f>IF(W24="","",W24-TODAY())</f>
         <v/>
       </c>
+      <c r="AG24" s="24">
+        <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="40" t="n"/>
@@ -2857,6 +3042,10 @@
         <f>IF(W25="","",W25-TODAY())</f>
         <v/>
       </c>
+      <c r="AG25" s="24">
+        <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="40" t="n"/>
@@ -2892,6 +3081,10 @@
         <f>IF(W26="","",W26-TODAY())</f>
         <v/>
       </c>
+      <c r="AG26" s="24">
+        <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="40" t="n"/>
@@ -2927,6 +3120,10 @@
         <f>IF(W27="","",W27-TODAY())</f>
         <v/>
       </c>
+      <c r="AG27" s="24">
+        <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="40" t="n"/>
@@ -2962,6 +3159,10 @@
         <f>IF(W28="","",W28-TODAY())</f>
         <v/>
       </c>
+      <c r="AG28" s="24">
+        <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="40" t="n"/>
@@ -2997,6 +3198,10 @@
         <f>IF(W29="","",W29-TODAY())</f>
         <v/>
       </c>
+      <c r="AG29" s="24">
+        <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40" t="n"/>
@@ -3032,6 +3237,10 @@
         <f>IF(W30="","",W30-TODAY())</f>
         <v/>
       </c>
+      <c r="AG30" s="24">
+        <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="40" t="n"/>
@@ -3067,6 +3276,10 @@
         <f>IF(W31="","",W31-TODAY())</f>
         <v/>
       </c>
+      <c r="AG31" s="24">
+        <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="40" t="n"/>
@@ -3102,6 +3315,10 @@
         <f>IF(W32="","",W32-TODAY())</f>
         <v/>
       </c>
+      <c r="AG32" s="24">
+        <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="40" t="n"/>
@@ -3137,6 +3354,10 @@
         <f>IF(W33="","",W33-TODAY())</f>
         <v/>
       </c>
+      <c r="AG33" s="24">
+        <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="40" t="n"/>
@@ -3172,6 +3393,10 @@
         <f>IF(W34="","",W34-TODAY())</f>
         <v/>
       </c>
+      <c r="AG34" s="24">
+        <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="40" t="n"/>
@@ -3207,6 +3432,10 @@
         <f>IF(W35="","",W35-TODAY())</f>
         <v/>
       </c>
+      <c r="AG35" s="24">
+        <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="40" t="n"/>
@@ -3242,6 +3471,10 @@
         <f>IF(W36="","",W36-TODAY())</f>
         <v/>
       </c>
+      <c r="AG36" s="24">
+        <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="40" t="n"/>
@@ -3277,6 +3510,10 @@
         <f>IF(W37="","",W37-TODAY())</f>
         <v/>
       </c>
+      <c r="AG37" s="24">
+        <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="40" t="n"/>
@@ -3312,6 +3549,10 @@
         <f>IF(W38="","",W38-TODAY())</f>
         <v/>
       </c>
+      <c r="AG38" s="24">
+        <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="40" t="n"/>
@@ -3347,6 +3588,10 @@
         <f>IF(W39="","",W39-TODAY())</f>
         <v/>
       </c>
+      <c r="AG39" s="24">
+        <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="40" t="n"/>
@@ -3382,6 +3627,10 @@
         <f>IF(W40="","",W40-TODAY())</f>
         <v/>
       </c>
+      <c r="AG40" s="24">
+        <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="40" t="n"/>
@@ -3417,6 +3666,10 @@
         <f>IF(W41="","",W41-TODAY())</f>
         <v/>
       </c>
+      <c r="AG41" s="24">
+        <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="40" t="n"/>
@@ -3452,6 +3705,10 @@
         <f>IF(W42="","",W42-TODAY())</f>
         <v/>
       </c>
+      <c r="AG42" s="24">
+        <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="40" t="n"/>
@@ -3487,6 +3744,10 @@
         <f>IF(W43="","",W43-TODAY())</f>
         <v/>
       </c>
+      <c r="AG43" s="24">
+        <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="40" t="n"/>
@@ -3522,6 +3783,10 @@
         <f>IF(W44="","",W44-TODAY())</f>
         <v/>
       </c>
+      <c r="AG44" s="24">
+        <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="40" t="n"/>
@@ -3557,6 +3822,10 @@
         <f>IF(W45="","",W45-TODAY())</f>
         <v/>
       </c>
+      <c r="AG45" s="24">
+        <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="40" t="n"/>
@@ -3592,6 +3861,10 @@
         <f>IF(W46="","",W46-TODAY())</f>
         <v/>
       </c>
+      <c r="AG46" s="24">
+        <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="40" t="n"/>
@@ -3627,6 +3900,10 @@
         <f>IF(W47="","",W47-TODAY())</f>
         <v/>
       </c>
+      <c r="AG47" s="24">
+        <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="40" t="n"/>
@@ -3662,6 +3939,10 @@
         <f>IF(W48="","",W48-TODAY())</f>
         <v/>
       </c>
+      <c r="AG48" s="24">
+        <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="40" t="n"/>
@@ -3697,6 +3978,10 @@
         <f>IF(W49="","",W49-TODAY())</f>
         <v/>
       </c>
+      <c r="AG49" s="24">
+        <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
       <c r="A50" s="40" t="n"/>
@@ -3732,6 +4017,10 @@
         <f>IF(W50="","",W50-TODAY())</f>
         <v/>
       </c>
+      <c r="AG50" s="24">
+        <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="40" t="n"/>
@@ -3767,6 +4056,10 @@
         <f>IF(W51="","",W51-TODAY())</f>
         <v/>
       </c>
+      <c r="AG51" s="24">
+        <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
       <c r="A52" s="40" t="n"/>
@@ -3802,6 +4095,10 @@
         <f>IF(W52="","",W52-TODAY())</f>
         <v/>
       </c>
+      <c r="AG52" s="24">
+        <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="40" t="n"/>
@@ -3837,6 +4134,10 @@
         <f>IF(W53="","",W53-TODAY())</f>
         <v/>
       </c>
+      <c r="AG53" s="24">
+        <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="40" t="n"/>
@@ -3872,6 +4173,10 @@
         <f>IF(W54="","",W54-TODAY())</f>
         <v/>
       </c>
+      <c r="AG54" s="24">
+        <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="40" t="n"/>
@@ -3907,6 +4212,10 @@
         <f>IF(W55="","",W55-TODAY())</f>
         <v/>
       </c>
+      <c r="AG55" s="24">
+        <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="40" t="n"/>
@@ -3942,6 +4251,10 @@
         <f>IF(W56="","",W56-TODAY())</f>
         <v/>
       </c>
+      <c r="AG56" s="24">
+        <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
       <c r="A57" s="40" t="n"/>
@@ -3977,6 +4290,10 @@
         <f>IF(W57="","",W57-TODAY())</f>
         <v/>
       </c>
+      <c r="AG57" s="24">
+        <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="40" t="n"/>
@@ -4012,6 +4329,10 @@
         <f>IF(W58="","",W58-TODAY())</f>
         <v/>
       </c>
+      <c r="AG58" s="24">
+        <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="40" t="n"/>
@@ -4047,6 +4368,10 @@
         <f>IF(W59="","",W59-TODAY())</f>
         <v/>
       </c>
+      <c r="AG59" s="24">
+        <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
       <c r="A60" s="40" t="n"/>
@@ -4082,6 +4407,10 @@
         <f>IF(W60="","",W60-TODAY())</f>
         <v/>
       </c>
+      <c r="AG60" s="24">
+        <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
       <c r="A61" s="40" t="n"/>
@@ -4117,6 +4446,10 @@
         <f>IF(W61="","",W61-TODAY())</f>
         <v/>
       </c>
+      <c r="AG61" s="24">
+        <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
       <c r="A62" s="40" t="n"/>
@@ -4150,6 +4483,10 @@
       </c>
       <c r="X62" s="46">
         <f>IF(W62="","",W62-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AG62" s="24">
+        <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -4236,7 +4573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AB62"/>
+  <dimension ref="A1:AC62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -4370,44 +4707,49 @@
           <t>Days Until Deadline</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice #</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Date</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Sent Date</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X12" s="24" t="inlineStr">
         <is>
           <t>Cust Invoice Status</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice #</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Date</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Amount ($)</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB12" s="24" t="inlineStr">
         <is>
           <t>Molder Invoice Status</t>
+        </is>
+      </c>
+      <c r="AC12" s="24" t="inlineStr">
+        <is>
+          <t>_Seq</t>
         </is>
       </c>
     </row>
@@ -4493,6 +4835,10 @@
         <f>IF(S13="","",S13-TODAY())</f>
         <v/>
       </c>
+      <c r="AC13" s="24">
+        <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40" t="inlineStr">
@@ -4570,6 +4916,10 @@
         <f>IF(S14="","",S14-TODAY())</f>
         <v/>
       </c>
+      <c r="AC14" s="24">
+        <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40" t="inlineStr">
@@ -4651,6 +5001,10 @@
       </c>
       <c r="T15" s="46">
         <f>IF(S15="","",S15-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AC15" s="24">
+        <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>
@@ -4684,6 +5038,10 @@
         <f>IF(S16="","",S16-TODAY())</f>
         <v/>
       </c>
+      <c r="AC16" s="24">
+        <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
       <c r="A17" s="40" t="n"/>
@@ -4715,6 +5073,10 @@
         <f>IF(S17="","",S17-TODAY())</f>
         <v/>
       </c>
+      <c r="AC17" s="24">
+        <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="40" t="n"/>
@@ -4746,6 +5108,10 @@
         <f>IF(S18="","",S18-TODAY())</f>
         <v/>
       </c>
+      <c r="AC18" s="24">
+        <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
       <c r="A19" s="40" t="n"/>
@@ -4777,6 +5143,10 @@
         <f>IF(S19="","",S19-TODAY())</f>
         <v/>
       </c>
+      <c r="AC19" s="24">
+        <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="40" t="n"/>
@@ -4808,6 +5178,10 @@
         <f>IF(S20="","",S20-TODAY())</f>
         <v/>
       </c>
+      <c r="AC20" s="24">
+        <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
       <c r="A21" s="40" t="n"/>
@@ -4839,6 +5213,10 @@
         <f>IF(S21="","",S21-TODAY())</f>
         <v/>
       </c>
+      <c r="AC21" s="24">
+        <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
       <c r="A22" s="40" t="n"/>
@@ -4870,6 +5248,10 @@
         <f>IF(S22="","",S22-TODAY())</f>
         <v/>
       </c>
+      <c r="AC22" s="24">
+        <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="40" t="n"/>
@@ -4901,6 +5283,10 @@
         <f>IF(S23="","",S23-TODAY())</f>
         <v/>
       </c>
+      <c r="AC23" s="24">
+        <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="40" t="n"/>
@@ -4932,6 +5318,10 @@
         <f>IF(S24="","",S24-TODAY())</f>
         <v/>
       </c>
+      <c r="AC24" s="24">
+        <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="40" t="n"/>
@@ -4963,6 +5353,10 @@
         <f>IF(S25="","",S25-TODAY())</f>
         <v/>
       </c>
+      <c r="AC25" s="24">
+        <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="40" t="n"/>
@@ -4994,6 +5388,10 @@
         <f>IF(S26="","",S26-TODAY())</f>
         <v/>
       </c>
+      <c r="AC26" s="24">
+        <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="40" t="n"/>
@@ -5025,6 +5423,10 @@
         <f>IF(S27="","",S27-TODAY())</f>
         <v/>
       </c>
+      <c r="AC27" s="24">
+        <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="40" t="n"/>
@@ -5056,6 +5458,10 @@
         <f>IF(S28="","",S28-TODAY())</f>
         <v/>
       </c>
+      <c r="AC28" s="24">
+        <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="40" t="n"/>
@@ -5087,6 +5493,10 @@
         <f>IF(S29="","",S29-TODAY())</f>
         <v/>
       </c>
+      <c r="AC29" s="24">
+        <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40" t="n"/>
@@ -5118,6 +5528,10 @@
         <f>IF(S30="","",S30-TODAY())</f>
         <v/>
       </c>
+      <c r="AC30" s="24">
+        <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="40" t="n"/>
@@ -5149,6 +5563,10 @@
         <f>IF(S31="","",S31-TODAY())</f>
         <v/>
       </c>
+      <c r="AC31" s="24">
+        <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="40" t="n"/>
@@ -5180,6 +5598,10 @@
         <f>IF(S32="","",S32-TODAY())</f>
         <v/>
       </c>
+      <c r="AC32" s="24">
+        <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="40" t="n"/>
@@ -5211,6 +5633,10 @@
         <f>IF(S33="","",S33-TODAY())</f>
         <v/>
       </c>
+      <c r="AC33" s="24">
+        <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="40" t="n"/>
@@ -5242,6 +5668,10 @@
         <f>IF(S34="","",S34-TODAY())</f>
         <v/>
       </c>
+      <c r="AC34" s="24">
+        <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="40" t="n"/>
@@ -5273,6 +5703,10 @@
         <f>IF(S35="","",S35-TODAY())</f>
         <v/>
       </c>
+      <c r="AC35" s="24">
+        <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="40" t="n"/>
@@ -5304,6 +5738,10 @@
         <f>IF(S36="","",S36-TODAY())</f>
         <v/>
       </c>
+      <c r="AC36" s="24">
+        <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="40" t="n"/>
@@ -5335,6 +5773,10 @@
         <f>IF(S37="","",S37-TODAY())</f>
         <v/>
       </c>
+      <c r="AC37" s="24">
+        <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="40" t="n"/>
@@ -5366,6 +5808,10 @@
         <f>IF(S38="","",S38-TODAY())</f>
         <v/>
       </c>
+      <c r="AC38" s="24">
+        <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="40" t="n"/>
@@ -5397,6 +5843,10 @@
         <f>IF(S39="","",S39-TODAY())</f>
         <v/>
       </c>
+      <c r="AC39" s="24">
+        <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="40" t="n"/>
@@ -5428,6 +5878,10 @@
         <f>IF(S40="","",S40-TODAY())</f>
         <v/>
       </c>
+      <c r="AC40" s="24">
+        <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="40" t="n"/>
@@ -5459,6 +5913,10 @@
         <f>IF(S41="","",S41-TODAY())</f>
         <v/>
       </c>
+      <c r="AC41" s="24">
+        <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="40" t="n"/>
@@ -5490,6 +5948,10 @@
         <f>IF(S42="","",S42-TODAY())</f>
         <v/>
       </c>
+      <c r="AC42" s="24">
+        <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="40" t="n"/>
@@ -5521,6 +5983,10 @@
         <f>IF(S43="","",S43-TODAY())</f>
         <v/>
       </c>
+      <c r="AC43" s="24">
+        <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="40" t="n"/>
@@ -5552,6 +6018,10 @@
         <f>IF(S44="","",S44-TODAY())</f>
         <v/>
       </c>
+      <c r="AC44" s="24">
+        <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="40" t="n"/>
@@ -5583,6 +6053,10 @@
         <f>IF(S45="","",S45-TODAY())</f>
         <v/>
       </c>
+      <c r="AC45" s="24">
+        <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="40" t="n"/>
@@ -5614,6 +6088,10 @@
         <f>IF(S46="","",S46-TODAY())</f>
         <v/>
       </c>
+      <c r="AC46" s="24">
+        <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="40" t="n"/>
@@ -5645,6 +6123,10 @@
         <f>IF(S47="","",S47-TODAY())</f>
         <v/>
       </c>
+      <c r="AC47" s="24">
+        <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="40" t="n"/>
@@ -5676,6 +6158,10 @@
         <f>IF(S48="","",S48-TODAY())</f>
         <v/>
       </c>
+      <c r="AC48" s="24">
+        <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
       <c r="A49" s="40" t="n"/>
@@ -5707,6 +6193,10 @@
         <f>IF(S49="","",S49-TODAY())</f>
         <v/>
       </c>
+      <c r="AC49" s="24">
+        <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
       <c r="A50" s="40" t="n"/>
@@ -5738,6 +6228,10 @@
         <f>IF(S50="","",S50-TODAY())</f>
         <v/>
       </c>
+      <c r="AC50" s="24">
+        <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="40" t="n"/>
@@ -5769,6 +6263,10 @@
         <f>IF(S51="","",S51-TODAY())</f>
         <v/>
       </c>
+      <c r="AC51" s="24">
+        <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
       <c r="A52" s="40" t="n"/>
@@ -5800,6 +6298,10 @@
         <f>IF(S52="","",S52-TODAY())</f>
         <v/>
       </c>
+      <c r="AC52" s="24">
+        <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="40" t="n"/>
@@ -5831,6 +6333,10 @@
         <f>IF(S53="","",S53-TODAY())</f>
         <v/>
       </c>
+      <c r="AC53" s="24">
+        <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
       <c r="A54" s="40" t="n"/>
@@ -5862,6 +6368,10 @@
         <f>IF(S54="","",S54-TODAY())</f>
         <v/>
       </c>
+      <c r="AC54" s="24">
+        <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
       <c r="A55" s="40" t="n"/>
@@ -5893,6 +6403,10 @@
         <f>IF(S55="","",S55-TODAY())</f>
         <v/>
       </c>
+      <c r="AC55" s="24">
+        <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="40" t="n"/>
@@ -5924,6 +6438,10 @@
         <f>IF(S56="","",S56-TODAY())</f>
         <v/>
       </c>
+      <c r="AC56" s="24">
+        <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
       <c r="A57" s="40" t="n"/>
@@ -5955,6 +6473,10 @@
         <f>IF(S57="","",S57-TODAY())</f>
         <v/>
       </c>
+      <c r="AC57" s="24">
+        <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="40" t="n"/>
@@ -5986,6 +6508,10 @@
         <f>IF(S58="","",S58-TODAY())</f>
         <v/>
       </c>
+      <c r="AC58" s="24">
+        <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="40" t="n"/>
@@ -6017,6 +6543,10 @@
         <f>IF(S59="","",S59-TODAY())</f>
         <v/>
       </c>
+      <c r="AC59" s="24">
+        <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
       <c r="A60" s="40" t="n"/>
@@ -6048,6 +6578,10 @@
         <f>IF(S60="","",S60-TODAY())</f>
         <v/>
       </c>
+      <c r="AC60" s="24">
+        <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
       <c r="A61" s="40" t="n"/>
@@ -6079,6 +6613,10 @@
         <f>IF(S61="","",S61-TODAY())</f>
         <v/>
       </c>
+      <c r="AC61" s="24">
+        <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
       <c r="A62" s="40" t="n"/>
@@ -6108,6 +6646,10 @@
       </c>
       <c r="T62" s="46">
         <f>IF(S62="","",S62-TODAY())</f>
+        <v/>
+      </c>
+      <c r="AC62" s="24">
+        <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: hide Completed jobs using helper column + MATCH with cached values
- New Tooling Jobs col AG and Reorders col AC: sequential rank formula
  assigns 1,2,3... only to active (non-blank, non-Completed) rows
  using COUNTIFS. Blank for completed or empty rows.
- Dashboard MATCH(n, helper_col, 0) finds the nth active job dynamically:
  when a job is marked Completed its helper cell goes blank, it drops
  out of the sequence, and the dashboard row goes blank automatically.
- All helper col and dashboard cells pre-cached in XML so file displays
  correctly on open without needing a recalculation.

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -1047,309 +1047,603 @@
     </row>
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
-        <f>IF('New Tooling Jobs'!A13="","",'New Tooling Jobs'!A13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-101</v>
       </c>
       <c r="B10" s="39">
-        <f>IF('New Tooling Jobs'!A13="","","New Tooling")</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>New Tooling</v>
       </c>
       <c r="C10" s="39">
-        <f>IF('New Tooling Jobs'!B13="","",'New Tooling Jobs'!B13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Acme Industries</v>
       </c>
       <c r="D10" s="39">
-        <f>IF('New Tooling Jobs'!E13="","",'New Tooling Jobs'!E13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>2. Quote Sent to Customer</v>
       </c>
       <c r="E10" s="39">
-        <f>IF('New Tooling Jobs'!G13="","",'New Tooling Jobs'!G13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F10" s="39">
-        <f>IF('New Tooling Jobs'!H13="","",'New Tooling Jobs'!H13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G10" s="39">
-        <f>IF('New Tooling Jobs'!I13="","",'New Tooling Jobs'!I13)</f>
+        <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Awaiting customer PO</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="40">
-        <f>IF('New Tooling Jobs'!A14="","",'New Tooling Jobs'!A14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-102</v>
       </c>
       <c r="B11" s="40">
-        <f>IF('New Tooling Jobs'!A14="","","New Tooling")</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>New Tooling</v>
       </c>
       <c r="C11" s="41">
-        <f>IF('New Tooling Jobs'!B14="","",'New Tooling Jobs'!B14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Beacon Electronics</v>
       </c>
       <c r="D11" s="41">
-        <f>IF('New Tooling Jobs'!E14="","",'New Tooling Jobs'!E14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>4. PO Issued to Molder</v>
       </c>
       <c r="E11" s="40">
-        <f>IF('New Tooling Jobs'!G14="","",'New Tooling Jobs'!G14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-BE-3411</v>
       </c>
       <c r="F11" s="40">
-        <f>IF('New Tooling Jobs'!H14="","",'New Tooling Jobs'!H14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-SUM-0992</v>
       </c>
       <c r="G11" s="41">
-        <f>IF('New Tooling Jobs'!I14="","",'New Tooling Jobs'!I14)</f>
+        <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Mold kickoff meeting 5/4</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="40">
-        <f>IF('New Tooling Jobs'!A15="","",'New Tooling Jobs'!A15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-103</v>
       </c>
       <c r="B12" s="40">
-        <f>IF('New Tooling Jobs'!A15="","","New Tooling")</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>New Tooling</v>
       </c>
       <c r="C12" s="41">
-        <f>IF('New Tooling Jobs'!B15="","",'New Tooling Jobs'!B15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Drift Medical</v>
       </c>
       <c r="D12" s="41">
-        <f>IF('New Tooling Jobs'!E15="","",'New Tooling Jobs'!E15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>6. Sample / FAI Approval</v>
       </c>
       <c r="E12" s="40">
-        <f>IF('New Tooling Jobs'!G15="","",'New Tooling Jobs'!G15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-DM-2210</v>
       </c>
       <c r="F12" s="40">
-        <f>IF('New Tooling Jobs'!H15="","",'New Tooling Jobs'!H15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-PP-1145</v>
       </c>
       <c r="G12" s="41">
-        <f>IF('New Tooling Jobs'!I15="","",'New Tooling Jobs'!I15)</f>
+        <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Awaiting customer FAI sign-off</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40">
-        <f>IF('New Tooling Jobs'!A16="","",'New Tooling Jobs'!A16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-105</v>
       </c>
       <c r="B13" s="40">
-        <f>IF('New Tooling Jobs'!A16="","","New Tooling")</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>New Tooling</v>
       </c>
       <c r="C13" s="41">
-        <f>IF('New Tooling Jobs'!B16="","",'New Tooling Jobs'!B16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Acme Industries</v>
       </c>
       <c r="D13" s="41">
-        <f>IF('New Tooling Jobs'!E16="","",'New Tooling Jobs'!E16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>1. Quote Requested</v>
       </c>
       <c r="E13" s="40">
-        <f>IF('New Tooling Jobs'!G16="","",'New Tooling Jobs'!G16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="F13" s="40">
-        <f>IF('New Tooling Jobs'!H16="","",'New Tooling Jobs'!H16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G13" s="41">
-        <f>IF('New Tooling Jobs'!I16="","",'New Tooling Jobs'!I16)</f>
+        <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Waiting on molder quote (requested 4/22)</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40">
-        <f>IF(Reorders!A13="","",Reorders!A13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-104</v>
       </c>
       <c r="B14" s="40">
-        <f>IF(Reorders!A13="","","Reorder")</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>Reorder</v>
       </c>
       <c r="C14" s="41">
-        <f>IF(Reorders!B13="","",Reorders!B13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Cedar Outdoor Co.</v>
       </c>
       <c r="D14" s="41">
-        <f>IF(Reorders!E13="","",Reorders!E13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>3. Production &amp; Shipping</v>
       </c>
       <c r="E14" s="40">
-        <f>IF(Reorders!G13="","",Reorders!G13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-CD-1207</v>
       </c>
       <c r="F14" s="40">
-        <f>IF(Reorders!H13="","",Reorders!H13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-PAC-0451</v>
       </c>
       <c r="G14" s="41">
-        <f>IF(Reorders!I13="","",Reorders!I13)</f>
+        <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Production scheduled wk of 5/4</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40">
-        <f>IF(Reorders!A14="","",Reorders!A14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>JOB-2026-106</v>
       </c>
       <c r="B15" s="40">
-        <f>IF(Reorders!A14="","","Reorder")</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
         <v>Reorder</v>
       </c>
       <c r="C15" s="41">
-        <f>IF(Reorders!B14="","",Reorders!B14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Beacon Electronics</v>
       </c>
       <c r="D15" s="41">
-        <f>IF(Reorders!E14="","",Reorders!E14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>1. Customer PO Received</v>
       </c>
       <c r="E15" s="40">
-        <f>IF(Reorders!G14="","",Reorders!G14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>PO-BE-3415</v>
       </c>
       <c r="F15" s="40">
-        <f>IF(Reorders!H14="","",Reorders!H14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v/>
       </c>
       <c r="G15" s="41">
-        <f>IF(Reorders!I14="","",Reorders!I14)</f>
+        <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
         <v>Cut molder PO this week</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="40" t="n"/>
-      <c r="B16" s="40" t="n"/>
-      <c r="C16" s="41" t="n"/>
-      <c r="D16" s="41" t="n"/>
-      <c r="E16" s="40" t="n"/>
-      <c r="F16" s="40" t="n"/>
-      <c r="G16" s="41" t="n"/>
+      <c r="A16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="40">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="41">
+        <f>IFERROR(IF(7&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(7,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(7-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="40" t="n"/>
-      <c r="B17" s="40" t="n"/>
-      <c r="C17" s="41" t="n"/>
-      <c r="D17" s="41" t="n"/>
-      <c r="E17" s="40" t="n"/>
-      <c r="F17" s="40" t="n"/>
-      <c r="G17" s="41" t="n"/>
+      <c r="A17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="40">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="41">
+        <f>IFERROR(IF(8&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(8,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(8-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="40" t="n"/>
-      <c r="B18" s="40" t="n"/>
-      <c r="C18" s="41" t="n"/>
-      <c r="D18" s="41" t="n"/>
-      <c r="E18" s="40" t="n"/>
-      <c r="F18" s="40" t="n"/>
-      <c r="G18" s="41" t="n"/>
+      <c r="A18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="40">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="41">
+        <f>IFERROR(IF(9&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(9,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(9-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="40" t="n"/>
-      <c r="B19" s="40" t="n"/>
-      <c r="C19" s="41" t="n"/>
-      <c r="D19" s="41" t="n"/>
-      <c r="E19" s="40" t="n"/>
-      <c r="F19" s="40" t="n"/>
-      <c r="G19" s="41" t="n"/>
+      <c r="A19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="40">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="41">
+        <f>IFERROR(IF(10&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(10,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(10-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
-      <c r="A20" s="40" t="n"/>
-      <c r="B20" s="40" t="n"/>
-      <c r="C20" s="41" t="n"/>
-      <c r="D20" s="41" t="n"/>
-      <c r="E20" s="40" t="n"/>
-      <c r="F20" s="40" t="n"/>
-      <c r="G20" s="41" t="n"/>
+      <c r="A20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="40">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="41">
+        <f>IFERROR(IF(11&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(11,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(11-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="40" t="n"/>
-      <c r="C21" s="41" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="40" t="n"/>
-      <c r="F21" s="40" t="n"/>
-      <c r="G21" s="41" t="n"/>
+      <c r="A21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="40">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="41">
+        <f>IFERROR(IF(12&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(12,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(12-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
-      <c r="A22" s="40" t="n"/>
-      <c r="B22" s="40" t="n"/>
-      <c r="C22" s="41" t="n"/>
-      <c r="D22" s="41" t="n"/>
-      <c r="E22" s="40" t="n"/>
-      <c r="F22" s="40" t="n"/>
-      <c r="G22" s="41" t="n"/>
+      <c r="A22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="40">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="41">
+        <f>IFERROR(IF(13&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(13,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(13-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
-      <c r="A23" s="40" t="n"/>
-      <c r="B23" s="40" t="n"/>
-      <c r="C23" s="41" t="n"/>
-      <c r="D23" s="41" t="n"/>
-      <c r="E23" s="40" t="n"/>
-      <c r="F23" s="40" t="n"/>
-      <c r="G23" s="41" t="n"/>
+      <c r="A23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="40">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>IFERROR(IF(14&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(14,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(14-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
-      <c r="A24" s="40" t="n"/>
-      <c r="B24" s="40" t="n"/>
-      <c r="C24" s="41" t="n"/>
-      <c r="D24" s="41" t="n"/>
-      <c r="E24" s="40" t="n"/>
-      <c r="F24" s="40" t="n"/>
-      <c r="G24" s="41" t="n"/>
+      <c r="A24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="41">
+        <f>IFERROR(IF(15&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(15,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(15-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
-      <c r="A25" s="40" t="n"/>
-      <c r="B25" s="40" t="n"/>
-      <c r="C25" s="41" t="n"/>
-      <c r="D25" s="41" t="n"/>
-      <c r="E25" s="40" t="n"/>
-      <c r="F25" s="40" t="n"/>
-      <c r="G25" s="41" t="n"/>
+      <c r="A25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>IFERROR(IF(16&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(16,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(16-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
-      <c r="A26" s="40" t="n"/>
-      <c r="B26" s="40" t="n"/>
-      <c r="C26" s="41" t="n"/>
-      <c r="D26" s="41" t="n"/>
-      <c r="E26" s="40" t="n"/>
-      <c r="F26" s="40" t="n"/>
-      <c r="G26" s="41" t="n"/>
+      <c r="A26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="40">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="41">
+        <f>IFERROR(IF(17&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(17,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(17-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
-      <c r="A27" s="40" t="n"/>
-      <c r="B27" s="40" t="n"/>
-      <c r="C27" s="41" t="n"/>
-      <c r="D27" s="41" t="n"/>
-      <c r="E27" s="40" t="n"/>
-      <c r="F27" s="40" t="n"/>
-      <c r="G27" s="41" t="n"/>
+      <c r="A27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="40">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="41">
+        <f>IFERROR(IF(18&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(18,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(18-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
-      <c r="A28" s="40" t="n"/>
-      <c r="B28" s="40" t="n"/>
-      <c r="C28" s="41" t="n"/>
-      <c r="D28" s="41" t="n"/>
-      <c r="E28" s="40" t="n"/>
-      <c r="F28" s="40" t="n"/>
-      <c r="G28" s="41" t="n"/>
+      <c r="A28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="40">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="41">
+        <f>IFERROR(IF(19&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(19,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(19-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
-      <c r="A29" s="40" t="n"/>
-      <c r="B29" s="40" t="n"/>
-      <c r="C29" s="41" t="n"/>
-      <c r="D29" s="41" t="n"/>
-      <c r="E29" s="40" t="n"/>
-      <c r="F29" s="40" t="n"/>
-      <c r="G29" s="41" t="n"/>
+      <c r="A29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="B29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="D29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="40">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="41">
+        <f>IFERROR(IF(20&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(20,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(20-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="40" t="n"/>
@@ -2089,15 +2383,6 @@
       <c r="F111" s="40" t="n"/>
       <c r="G111" s="41" t="n"/>
     </row>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
   </sheetData>
   <autoFilter ref="A9:G111"/>
   <mergeCells count="11">
@@ -2438,7 +2723,7 @@
       </c>
       <c r="AG13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
@@ -2527,7 +2812,7 @@
       </c>
       <c r="AG14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
@@ -2626,7 +2911,7 @@
       </c>
       <c r="AG15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="16" ht="23.85" customHeight="1" s="25">
@@ -2693,7 +2978,7 @@
       </c>
       <c r="AG16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
@@ -2732,7 +3017,6 @@
       </c>
       <c r="AG17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
@@ -2771,7 +3055,6 @@
       </c>
       <c r="AG18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
@@ -2810,7 +3093,6 @@
       </c>
       <c r="AG19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
@@ -2849,7 +3131,6 @@
       </c>
       <c r="AG20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
@@ -2888,7 +3169,6 @@
       </c>
       <c r="AG21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
@@ -2927,7 +3207,6 @@
       </c>
       <c r="AG22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
@@ -2966,7 +3245,6 @@
       </c>
       <c r="AG23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
@@ -3005,7 +3283,6 @@
       </c>
       <c r="AG24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
@@ -3044,7 +3321,6 @@
       </c>
       <c r="AG25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
@@ -3083,7 +3359,6 @@
       </c>
       <c r="AG26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
@@ -3122,7 +3397,6 @@
       </c>
       <c r="AG27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
@@ -3161,7 +3435,6 @@
       </c>
       <c r="AG28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
@@ -3200,7 +3473,6 @@
       </c>
       <c r="AG29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
@@ -3239,7 +3511,6 @@
       </c>
       <c r="AG30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
@@ -3278,7 +3549,6 @@
       </c>
       <c r="AG31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
@@ -3317,7 +3587,6 @@
       </c>
       <c r="AG32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
@@ -3356,7 +3625,6 @@
       </c>
       <c r="AG33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
@@ -3395,7 +3663,6 @@
       </c>
       <c r="AG34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
@@ -3434,7 +3701,6 @@
       </c>
       <c r="AG35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
@@ -3473,7 +3739,6 @@
       </c>
       <c r="AG36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
@@ -3512,7 +3777,6 @@
       </c>
       <c r="AG37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
@@ -3551,7 +3815,6 @@
       </c>
       <c r="AG38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
@@ -3590,7 +3853,6 @@
       </c>
       <c r="AG39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
@@ -3629,7 +3891,6 @@
       </c>
       <c r="AG40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
@@ -3668,7 +3929,6 @@
       </c>
       <c r="AG41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
@@ -3707,7 +3967,6 @@
       </c>
       <c r="AG42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
@@ -3746,7 +4005,6 @@
       </c>
       <c r="AG43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
@@ -3785,7 +4043,6 @@
       </c>
       <c r="AG44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
@@ -3824,7 +4081,6 @@
       </c>
       <c r="AG45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
@@ -3863,7 +4119,6 @@
       </c>
       <c r="AG46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
@@ -3902,7 +4157,6 @@
       </c>
       <c r="AG47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
@@ -3941,7 +4195,6 @@
       </c>
       <c r="AG48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
@@ -3980,7 +4233,6 @@
       </c>
       <c r="AG49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
@@ -4019,7 +4271,6 @@
       </c>
       <c r="AG50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
@@ -4058,7 +4309,6 @@
       </c>
       <c r="AG51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
@@ -4097,7 +4347,6 @@
       </c>
       <c r="AG52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
@@ -4136,7 +4385,6 @@
       </c>
       <c r="AG53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
@@ -4175,7 +4423,6 @@
       </c>
       <c r="AG54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
@@ -4214,7 +4461,6 @@
       </c>
       <c r="AG55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
@@ -4253,7 +4499,6 @@
       </c>
       <c r="AG56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
@@ -4292,7 +4537,6 @@
       </c>
       <c r="AG57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
@@ -4331,7 +4575,6 @@
       </c>
       <c r="AG58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
@@ -4370,7 +4613,6 @@
       </c>
       <c r="AG59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
@@ -4409,7 +4651,6 @@
       </c>
       <c r="AG60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
@@ -4448,7 +4689,6 @@
       </c>
       <c r="AG61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
@@ -4487,7 +4727,6 @@
       </c>
       <c r="AG62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
   </sheetData>
@@ -4837,7 +5076,7 @@
       </c>
       <c r="AC13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
@@ -4918,7 +5157,7 @@
       </c>
       <c r="AC14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
@@ -5005,7 +5244,6 @@
       </c>
       <c r="AC15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
@@ -5040,7 +5278,6 @@
       </c>
       <c r="AC16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
@@ -5075,7 +5312,6 @@
       </c>
       <c r="AC17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
@@ -5110,7 +5346,6 @@
       </c>
       <c r="AC18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
@@ -5145,7 +5380,6 @@
       </c>
       <c r="AC19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
@@ -5180,7 +5414,6 @@
       </c>
       <c r="AC20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
@@ -5215,7 +5448,6 @@
       </c>
       <c r="AC21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
@@ -5250,7 +5482,6 @@
       </c>
       <c r="AC22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
@@ -5285,7 +5516,6 @@
       </c>
       <c r="AC23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
@@ -5320,7 +5550,6 @@
       </c>
       <c r="AC24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
@@ -5355,7 +5584,6 @@
       </c>
       <c r="AC25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
@@ -5390,7 +5618,6 @@
       </c>
       <c r="AC26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
@@ -5425,7 +5652,6 @@
       </c>
       <c r="AC27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
@@ -5460,7 +5686,6 @@
       </c>
       <c r="AC28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
@@ -5495,7 +5720,6 @@
       </c>
       <c r="AC29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
@@ -5530,7 +5754,6 @@
       </c>
       <c r="AC30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
@@ -5565,7 +5788,6 @@
       </c>
       <c r="AC31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
@@ -5600,7 +5822,6 @@
       </c>
       <c r="AC32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
@@ -5635,7 +5856,6 @@
       </c>
       <c r="AC33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
@@ -5670,7 +5890,6 @@
       </c>
       <c r="AC34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
@@ -5705,7 +5924,6 @@
       </c>
       <c r="AC35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
@@ -5740,7 +5958,6 @@
       </c>
       <c r="AC36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
@@ -5775,7 +5992,6 @@
       </c>
       <c r="AC37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
@@ -5810,7 +6026,6 @@
       </c>
       <c r="AC38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
@@ -5845,7 +6060,6 @@
       </c>
       <c r="AC39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
@@ -5880,7 +6094,6 @@
       </c>
       <c r="AC40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
@@ -5915,7 +6128,6 @@
       </c>
       <c r="AC41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
@@ -5950,7 +6162,6 @@
       </c>
       <c r="AC42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
@@ -5985,7 +6196,6 @@
       </c>
       <c r="AC43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
@@ -6020,7 +6230,6 @@
       </c>
       <c r="AC44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
@@ -6055,7 +6264,6 @@
       </c>
       <c r="AC45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
@@ -6090,7 +6298,6 @@
       </c>
       <c r="AC46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
@@ -6125,7 +6332,6 @@
       </c>
       <c r="AC47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
@@ -6160,7 +6366,6 @@
       </c>
       <c r="AC48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
@@ -6195,7 +6400,6 @@
       </c>
       <c r="AC49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
@@ -6230,7 +6434,6 @@
       </c>
       <c r="AC50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
@@ -6265,7 +6468,6 @@
       </c>
       <c r="AC51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
@@ -6300,7 +6502,6 @@
       </c>
       <c r="AC52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
@@ -6335,7 +6536,6 @@
       </c>
       <c r="AC53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
@@ -6370,7 +6570,6 @@
       </c>
       <c r="AC54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
@@ -6405,7 +6604,6 @@
       </c>
       <c r="AC55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
@@ -6440,7 +6638,6 @@
       </c>
       <c r="AC56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
@@ -6475,7 +6672,6 @@
       </c>
       <c r="AC57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
@@ -6510,7 +6706,6 @@
       </c>
       <c r="AC58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
@@ -6545,7 +6740,6 @@
       </c>
       <c r="AC59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
@@ -6580,7 +6774,6 @@
       </c>
       <c r="AC60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
@@ -6615,7 +6808,6 @@
       </c>
       <c r="AC61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
@@ -6650,7 +6842,6 @@
       </c>
       <c r="AC62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Overdue counter: replace SUMPRODUCT with COUNTIFS
SUMPRODUCT with cross-sheet formula cell references was not evaluating
correctly in this file. Replaced with COUNTIFS which is consistent with
how Active Jobs / New Tooling / Reorders counts already work:
- Counts rows where Days Until Deadline < 0 (past due)
- AND Stage is not Completed
- AND Job # is not blank

Co-authored-by: Brudius <Brudius@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Injection_Mold_Job_Dashboard.xlsx
+++ b/Injection_Mold_Job_Dashboard.xlsx
@@ -1004,7 +1004,7 @@
         <v/>
       </c>
       <c r="G6" s="36">
-        <f>SUMPRODUCT(('New Tooling Jobs'!X13:X62&lt;&gt;"")*(IFERROR('New Tooling Jobs'!X13:X62+0,99999)&lt;0)*('New Tooling Jobs'!E13:E62&lt;&gt;"Completed"))+SUMPRODUCT((Reorders!T13:T62&lt;&gt;"")*(IFERROR(Reorders!T13:T62+0,99999)&lt;0)*(Reorders!E13:E62&lt;&gt;"Completed"))</f>
+        <f>COUNTIFS('New Tooling Jobs'!X13:X62,"&lt;0",'New Tooling Jobs'!E13:E62,"&lt;&gt;Completed",'New Tooling Jobs'!A13:A62,"&lt;&gt;")+COUNTIFS(Reorders!T13:T62,"&lt;0",Reorders!E13:E62,"&lt;&gt;Completed",Reorders!A13:A62,"&lt;&gt;")</f>
         <v/>
       </c>
     </row>
@@ -1048,19 +1048,19 @@
     <row r="10" ht="21.75" customHeight="1" s="25">
       <c r="A10" s="38">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-101</v>
+        <v/>
       </c>
       <c r="B10" s="39">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>New Tooling</v>
+        <v/>
       </c>
       <c r="C10" s="39">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Acme Industries</v>
+        <v/>
       </c>
       <c r="D10" s="39">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>2. Quote Sent to Customer</v>
+        <v/>
       </c>
       <c r="E10" s="39">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
@@ -1072,85 +1072,85 @@
       </c>
       <c r="G10" s="39">
         <f>IFERROR(IF(1&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(1,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(1-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Awaiting customer PO</v>
+        <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="40">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-102</v>
+        <v/>
       </c>
       <c r="B11" s="40">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>New Tooling</v>
+        <v/>
       </c>
       <c r="C11" s="41">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Beacon Electronics</v>
+        <v/>
       </c>
       <c r="D11" s="41">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>4. PO Issued to Molder</v>
+        <v/>
       </c>
       <c r="E11" s="40">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-BE-3411</v>
+        <v/>
       </c>
       <c r="F11" s="40">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-SUM-0992</v>
+        <v/>
       </c>
       <c r="G11" s="41">
         <f>IFERROR(IF(2&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(2,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(2-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Mold kickoff meeting 5/4</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="40">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-103</v>
+        <v/>
       </c>
       <c r="B12" s="40">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>New Tooling</v>
+        <v/>
       </c>
       <c r="C12" s="41">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Drift Medical</v>
+        <v/>
       </c>
       <c r="D12" s="41">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>6. Sample / FAI Approval</v>
+        <v/>
       </c>
       <c r="E12" s="40">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-DM-2210</v>
+        <v/>
       </c>
       <c r="F12" s="40">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-PP-1145</v>
+        <v/>
       </c>
       <c r="G12" s="41">
         <f>IFERROR(IF(3&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(3,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(3-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Awaiting customer FAI sign-off</v>
+        <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="40">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-105</v>
+        <v/>
       </c>
       <c r="B13" s="40">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>New Tooling</v>
+        <v/>
       </c>
       <c r="C13" s="41">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Acme Industries</v>
+        <v/>
       </c>
       <c r="D13" s="41">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>1. Quote Requested</v>
+        <v/>
       </c>
       <c r="E13" s="40">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
@@ -1162,59 +1162,59 @@
       </c>
       <c r="G13" s="41">
         <f>IFERROR(IF(4&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(4,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(4-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Waiting on molder quote (requested 4/22)</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="40">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-104</v>
+        <v/>
       </c>
       <c r="B14" s="40">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>Reorder</v>
+        <v/>
       </c>
       <c r="C14" s="41">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Cedar Outdoor Co.</v>
+        <v/>
       </c>
       <c r="D14" s="41">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>3. Production &amp; Shipping</v>
+        <v/>
       </c>
       <c r="E14" s="40">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-CD-1207</v>
+        <v/>
       </c>
       <c r="F14" s="40">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-PAC-0451</v>
+        <v/>
       </c>
       <c r="G14" s="41">
         <f>IFERROR(IF(5&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(5,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(5-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Production scheduled wk of 5/4</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="40">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!A$13:A$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!A$13:A$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>JOB-2026-106</v>
+        <v/>
       </c>
       <c r="B15" s="40">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),"New Tooling","Reorder"),"")</f>
-        <v>Reorder</v>
+        <v/>
       </c>
       <c r="C15" s="41">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!B$13:B$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!B$13:B$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Beacon Electronics</v>
+        <v/>
       </c>
       <c r="D15" s="41">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!E$13:E$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!E$13:E$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>1. Customer PO Received</v>
+        <v/>
       </c>
       <c r="E15" s="40">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!G$13:G$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!G$13:G$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>PO-BE-3415</v>
+        <v/>
       </c>
       <c r="F15" s="40">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!H$13:H$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!H$13:H$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="G15" s="41">
         <f>IFERROR(IF(6&lt;=COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),INDEX('New Tooling Jobs'!I$13:I$62,MATCH(6,'New Tooling Jobs'!AG$13:AG$62,0)),INDEX(Reorders!I$13:I$62,MATCH(6-COUNTIFS('New Tooling Jobs'!A$13:A$62,"&lt;&gt;",'New Tooling Jobs'!E$13:E$62,"&lt;&gt;Completed"),Reorders!AC$13:AC$62,0))),"")</f>
-        <v>Cut molder PO this week</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="AG13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="AG14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
-        <v>2</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="AG15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
-        <v>3</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="23.85" customHeight="1" s="25">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="AG16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
-        <v>4</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
@@ -3017,6 +3017,7 @@
       </c>
       <c r="AG17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
@@ -3055,6 +3056,7 @@
       </c>
       <c r="AG18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
@@ -3093,6 +3095,7 @@
       </c>
       <c r="AG19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
@@ -3131,6 +3134,7 @@
       </c>
       <c r="AG20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
@@ -3169,6 +3173,7 @@
       </c>
       <c r="AG21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
@@ -3207,6 +3212,7 @@
       </c>
       <c r="AG22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
@@ -3245,6 +3251,7 @@
       </c>
       <c r="AG23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
@@ -3283,6 +3290,7 @@
       </c>
       <c r="AG24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
@@ -3321,6 +3329,7 @@
       </c>
       <c r="AG25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
@@ -3359,6 +3368,7 @@
       </c>
       <c r="AG26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
@@ -3397,6 +3407,7 @@
       </c>
       <c r="AG27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
@@ -3435,6 +3446,7 @@
       </c>
       <c r="AG28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
@@ -3473,6 +3485,7 @@
       </c>
       <c r="AG29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
@@ -3511,6 +3524,7 @@
       </c>
       <c r="AG30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
@@ -3549,6 +3563,7 @@
       </c>
       <c r="AG31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
@@ -3587,6 +3602,7 @@
       </c>
       <c r="AG32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
@@ -3625,6 +3641,7 @@
       </c>
       <c r="AG33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
@@ -3663,6 +3680,7 @@
       </c>
       <c r="AG34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
@@ -3701,6 +3719,7 @@
       </c>
       <c r="AG35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
@@ -3739,6 +3758,7 @@
       </c>
       <c r="AG36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
@@ -3777,6 +3797,7 @@
       </c>
       <c r="AG37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
@@ -3815,6 +3836,7 @@
       </c>
       <c r="AG38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
@@ -3853,6 +3875,7 @@
       </c>
       <c r="AG39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
@@ -3891,6 +3914,7 @@
       </c>
       <c r="AG40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
@@ -3929,6 +3953,7 @@
       </c>
       <c r="AG41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
@@ -3967,6 +3992,7 @@
       </c>
       <c r="AG42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
@@ -4005,6 +4031,7 @@
       </c>
       <c r="AG43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
@@ -4043,6 +4070,7 @@
       </c>
       <c r="AG44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
@@ -4081,6 +4109,7 @@
       </c>
       <c r="AG45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
@@ -4119,6 +4148,7 @@
       </c>
       <c r="AG46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
@@ -4157,6 +4187,7 @@
       </c>
       <c r="AG47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
@@ -4195,6 +4226,7 @@
       </c>
       <c r="AG48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
@@ -4233,6 +4265,7 @@
       </c>
       <c r="AG49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
@@ -4271,6 +4304,7 @@
       </c>
       <c r="AG50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
@@ -4309,6 +4343,7 @@
       </c>
       <c r="AG51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
@@ -4347,6 +4382,7 @@
       </c>
       <c r="AG52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
@@ -4385,6 +4421,7 @@
       </c>
       <c r="AG53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
@@ -4423,6 +4460,7 @@
       </c>
       <c r="AG54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
@@ -4461,6 +4499,7 @@
       </c>
       <c r="AG55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
@@ -4499,6 +4538,7 @@
       </c>
       <c r="AG56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
@@ -4537,6 +4577,7 @@
       </c>
       <c r="AG57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
@@ -4575,6 +4616,7 @@
       </c>
       <c r="AG58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
@@ -4613,6 +4655,7 @@
       </c>
       <c r="AG59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
@@ -4651,6 +4694,7 @@
       </c>
       <c r="AG60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
@@ -4689,6 +4733,7 @@
       </c>
       <c r="AG61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
@@ -4727,6 +4772,7 @@
       </c>
       <c r="AG62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -5076,7 +5122,7 @@
       </c>
       <c r="AC13" s="24">
         <f>IF(AND(A13&lt;&gt;"",E13&lt;&gt;"Completed"),COUNTIFS(A$13:A13,"&lt;&gt;",E$13:E13,"&lt;&gt;Completed"),"")</f>
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
@@ -5157,7 +5203,7 @@
       </c>
       <c r="AC14" s="24">
         <f>IF(AND(A14&lt;&gt;"",E14&lt;&gt;"Completed"),COUNTIFS(A$13:A14,"&lt;&gt;",E$13:E14,"&lt;&gt;Completed"),"")</f>
-        <v>2</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
@@ -5244,6 +5290,7 @@
       </c>
       <c r="AC15" s="24">
         <f>IF(AND(A15&lt;&gt;"",E15&lt;&gt;"Completed"),COUNTIFS(A$13:A15,"&lt;&gt;",E$13:E15,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
@@ -5278,6 +5325,7 @@
       </c>
       <c r="AC16" s="24">
         <f>IF(AND(A16&lt;&gt;"",E16&lt;&gt;"Completed"),COUNTIFS(A$13:A16,"&lt;&gt;",E$13:E16,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
@@ -5312,6 +5360,7 @@
       </c>
       <c r="AC17" s="24">
         <f>IF(AND(A17&lt;&gt;"",E17&lt;&gt;"Completed"),COUNTIFS(A$13:A17,"&lt;&gt;",E$13:E17,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
@@ -5346,6 +5395,7 @@
       </c>
       <c r="AC18" s="24">
         <f>IF(AND(A18&lt;&gt;"",E18&lt;&gt;"Completed"),COUNTIFS(A$13:A18,"&lt;&gt;",E$13:E18,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
@@ -5380,6 +5430,7 @@
       </c>
       <c r="AC19" s="24">
         <f>IF(AND(A19&lt;&gt;"",E19&lt;&gt;"Completed"),COUNTIFS(A$13:A19,"&lt;&gt;",E$13:E19,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="25">
@@ -5414,6 +5465,7 @@
       </c>
       <c r="AC20" s="24">
         <f>IF(AND(A20&lt;&gt;"",E20&lt;&gt;"Completed"),COUNTIFS(A$13:A20,"&lt;&gt;",E$13:E20,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="25">
@@ -5448,6 +5500,7 @@
       </c>
       <c r="AC21" s="24">
         <f>IF(AND(A21&lt;&gt;"",E21&lt;&gt;"Completed"),COUNTIFS(A$13:A21,"&lt;&gt;",E$13:E21,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="25">
@@ -5482,6 +5535,7 @@
       </c>
       <c r="AC22" s="24">
         <f>IF(AND(A22&lt;&gt;"",E22&lt;&gt;"Completed"),COUNTIFS(A$13:A22,"&lt;&gt;",E$13:E22,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="25">
@@ -5516,6 +5570,7 @@
       </c>
       <c r="AC23" s="24">
         <f>IF(AND(A23&lt;&gt;"",E23&lt;&gt;"Completed"),COUNTIFS(A$13:A23,"&lt;&gt;",E$13:E23,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
@@ -5550,6 +5605,7 @@
       </c>
       <c r="AC24" s="24">
         <f>IF(AND(A24&lt;&gt;"",E24&lt;&gt;"Completed"),COUNTIFS(A$13:A24,"&lt;&gt;",E$13:E24,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
@@ -5584,6 +5640,7 @@
       </c>
       <c r="AC25" s="24">
         <f>IF(AND(A25&lt;&gt;"",E25&lt;&gt;"Completed"),COUNTIFS(A$13:A25,"&lt;&gt;",E$13:E25,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
@@ -5618,6 +5675,7 @@
       </c>
       <c r="AC26" s="24">
         <f>IF(AND(A26&lt;&gt;"",E26&lt;&gt;"Completed"),COUNTIFS(A$13:A26,"&lt;&gt;",E$13:E26,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
@@ -5652,6 +5710,7 @@
       </c>
       <c r="AC27" s="24">
         <f>IF(AND(A27&lt;&gt;"",E27&lt;&gt;"Completed"),COUNTIFS(A$13:A27,"&lt;&gt;",E$13:E27,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
@@ -5686,6 +5745,7 @@
       </c>
       <c r="AC28" s="24">
         <f>IF(AND(A28&lt;&gt;"",E28&lt;&gt;"Completed"),COUNTIFS(A$13:A28,"&lt;&gt;",E$13:E28,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="25">
@@ -5720,6 +5780,7 @@
       </c>
       <c r="AC29" s="24">
         <f>IF(AND(A29&lt;&gt;"",E29&lt;&gt;"Completed"),COUNTIFS(A$13:A29,"&lt;&gt;",E$13:E29,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
@@ -5754,6 +5815,7 @@
       </c>
       <c r="AC30" s="24">
         <f>IF(AND(A30&lt;&gt;"",E30&lt;&gt;"Completed"),COUNTIFS(A$13:A30,"&lt;&gt;",E$13:E30,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
@@ -5788,6 +5850,7 @@
       </c>
       <c r="AC31" s="24">
         <f>IF(AND(A31&lt;&gt;"",E31&lt;&gt;"Completed"),COUNTIFS(A$13:A31,"&lt;&gt;",E$13:E31,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="25">
@@ -5822,6 +5885,7 @@
       </c>
       <c r="AC32" s="24">
         <f>IF(AND(A32&lt;&gt;"",E32&lt;&gt;"Completed"),COUNTIFS(A$13:A32,"&lt;&gt;",E$13:E32,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
@@ -5856,6 +5920,7 @@
       </c>
       <c r="AC33" s="24">
         <f>IF(AND(A33&lt;&gt;"",E33&lt;&gt;"Completed"),COUNTIFS(A$13:A33,"&lt;&gt;",E$13:E33,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
@@ -5890,6 +5955,7 @@
       </c>
       <c r="AC34" s="24">
         <f>IF(AND(A34&lt;&gt;"",E34&lt;&gt;"Completed"),COUNTIFS(A$13:A34,"&lt;&gt;",E$13:E34,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
@@ -5924,6 +5990,7 @@
       </c>
       <c r="AC35" s="24">
         <f>IF(AND(A35&lt;&gt;"",E35&lt;&gt;"Completed"),COUNTIFS(A$13:A35,"&lt;&gt;",E$13:E35,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
@@ -5958,6 +6025,7 @@
       </c>
       <c r="AC36" s="24">
         <f>IF(AND(A36&lt;&gt;"",E36&lt;&gt;"Completed"),COUNTIFS(A$13:A36,"&lt;&gt;",E$13:E36,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="25">
@@ -5992,6 +6060,7 @@
       </c>
       <c r="AC37" s="24">
         <f>IF(AND(A37&lt;&gt;"",E37&lt;&gt;"Completed"),COUNTIFS(A$13:A37,"&lt;&gt;",E$13:E37,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
@@ -6026,6 +6095,7 @@
       </c>
       <c r="AC38" s="24">
         <f>IF(AND(A38&lt;&gt;"",E38&lt;&gt;"Completed"),COUNTIFS(A$13:A38,"&lt;&gt;",E$13:E38,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="25">
@@ -6060,6 +6130,7 @@
       </c>
       <c r="AC39" s="24">
         <f>IF(AND(A39&lt;&gt;"",E39&lt;&gt;"Completed"),COUNTIFS(A$13:A39,"&lt;&gt;",E$13:E39,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
@@ -6094,6 +6165,7 @@
       </c>
       <c r="AC40" s="24">
         <f>IF(AND(A40&lt;&gt;"",E40&lt;&gt;"Completed"),COUNTIFS(A$13:A40,"&lt;&gt;",E$13:E40,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
@@ -6128,6 +6200,7 @@
       </c>
       <c r="AC41" s="24">
         <f>IF(AND(A41&lt;&gt;"",E41&lt;&gt;"Completed"),COUNTIFS(A$13:A41,"&lt;&gt;",E$13:E41,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="25">
@@ -6162,6 +6235,7 @@
       </c>
       <c r="AC42" s="24">
         <f>IF(AND(A42&lt;&gt;"",E42&lt;&gt;"Completed"),COUNTIFS(A$13:A42,"&lt;&gt;",E$13:E42,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="25">
@@ -6196,6 +6270,7 @@
       </c>
       <c r="AC43" s="24">
         <f>IF(AND(A43&lt;&gt;"",E43&lt;&gt;"Completed"),COUNTIFS(A$13:A43,"&lt;&gt;",E$13:E43,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
@@ -6230,6 +6305,7 @@
       </c>
       <c r="AC44" s="24">
         <f>IF(AND(A44&lt;&gt;"",E44&lt;&gt;"Completed"),COUNTIFS(A$13:A44,"&lt;&gt;",E$13:E44,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
@@ -6264,6 +6340,7 @@
       </c>
       <c r="AC45" s="24">
         <f>IF(AND(A45&lt;&gt;"",E45&lt;&gt;"Completed"),COUNTIFS(A$13:A45,"&lt;&gt;",E$13:E45,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
@@ -6298,6 +6375,7 @@
       </c>
       <c r="AC46" s="24">
         <f>IF(AND(A46&lt;&gt;"",E46&lt;&gt;"Completed"),COUNTIFS(A$13:A46,"&lt;&gt;",E$13:E46,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
@@ -6332,6 +6410,7 @@
       </c>
       <c r="AC47" s="24">
         <f>IF(AND(A47&lt;&gt;"",E47&lt;&gt;"Completed"),COUNTIFS(A$13:A47,"&lt;&gt;",E$13:E47,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="25">
@@ -6366,6 +6445,7 @@
       </c>
       <c r="AC48" s="24">
         <f>IF(AND(A48&lt;&gt;"",E48&lt;&gt;"Completed"),COUNTIFS(A$13:A48,"&lt;&gt;",E$13:E48,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="25">
@@ -6400,6 +6480,7 @@
       </c>
       <c r="AC49" s="24">
         <f>IF(AND(A49&lt;&gt;"",E49&lt;&gt;"Completed"),COUNTIFS(A$13:A49,"&lt;&gt;",E$13:E49,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="25">
@@ -6434,6 +6515,7 @@
       </c>
       <c r="AC50" s="24">
         <f>IF(AND(A50&lt;&gt;"",E50&lt;&gt;"Completed"),COUNTIFS(A$13:A50,"&lt;&gt;",E$13:E50,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
@@ -6468,6 +6550,7 @@
       </c>
       <c r="AC51" s="24">
         <f>IF(AND(A51&lt;&gt;"",E51&lt;&gt;"Completed"),COUNTIFS(A$13:A51,"&lt;&gt;",E$13:E51,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="25">
@@ -6502,6 +6585,7 @@
       </c>
       <c r="AC52" s="24">
         <f>IF(AND(A52&lt;&gt;"",E52&lt;&gt;"Completed"),COUNTIFS(A$13:A52,"&lt;&gt;",E$13:E52,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
@@ -6536,6 +6620,7 @@
       </c>
       <c r="AC53" s="24">
         <f>IF(AND(A53&lt;&gt;"",E53&lt;&gt;"Completed"),COUNTIFS(A$13:A53,"&lt;&gt;",E$13:E53,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="25">
@@ -6570,6 +6655,7 @@
       </c>
       <c r="AC54" s="24">
         <f>IF(AND(A54&lt;&gt;"",E54&lt;&gt;"Completed"),COUNTIFS(A$13:A54,"&lt;&gt;",E$13:E54,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="25">
@@ -6604,6 +6690,7 @@
       </c>
       <c r="AC55" s="24">
         <f>IF(AND(A55&lt;&gt;"",E55&lt;&gt;"Completed"),COUNTIFS(A$13:A55,"&lt;&gt;",E$13:E55,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
@@ -6638,6 +6725,7 @@
       </c>
       <c r="AC56" s="24">
         <f>IF(AND(A56&lt;&gt;"",E56&lt;&gt;"Completed"),COUNTIFS(A$13:A56,"&lt;&gt;",E$13:E56,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="25">
@@ -6672,6 +6760,7 @@
       </c>
       <c r="AC57" s="24">
         <f>IF(AND(A57&lt;&gt;"",E57&lt;&gt;"Completed"),COUNTIFS(A$13:A57,"&lt;&gt;",E$13:E57,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
@@ -6706,6 +6795,7 @@
       </c>
       <c r="AC58" s="24">
         <f>IF(AND(A58&lt;&gt;"",E58&lt;&gt;"Completed"),COUNTIFS(A$13:A58,"&lt;&gt;",E$13:E58,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
@@ -6740,6 +6830,7 @@
       </c>
       <c r="AC59" s="24">
         <f>IF(AND(A59&lt;&gt;"",E59&lt;&gt;"Completed"),COUNTIFS(A$13:A59,"&lt;&gt;",E$13:E59,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="25">
@@ -6774,6 +6865,7 @@
       </c>
       <c r="AC60" s="24">
         <f>IF(AND(A60&lt;&gt;"",E60&lt;&gt;"Completed"),COUNTIFS(A$13:A60,"&lt;&gt;",E$13:E60,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="25">
@@ -6808,6 +6900,7 @@
       </c>
       <c r="AC61" s="24">
         <f>IF(AND(A61&lt;&gt;"",E61&lt;&gt;"Completed"),COUNTIFS(A$13:A61,"&lt;&gt;",E$13:E61,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="25">
@@ -6842,6 +6935,7 @@
       </c>
       <c r="AC62" s="24">
         <f>IF(AND(A62&lt;&gt;"",E62&lt;&gt;"Completed"),COUNTIFS(A$13:A62,"&lt;&gt;",E$13:E62,"&lt;&gt;Completed"),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>